<commit_message>
removed graphs from git
</commit_message>
<xml_diff>
--- a/results/graphs/benchmark_results.xlsx
+++ b/results/graphs/benchmark_results.xlsx
@@ -496,7 +496,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E2" t="n">
-        <v>0.207128643989563</v>
+        <v>0.2548599243164062</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -538,7 +538,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2037955522537231</v>
+        <v>0.2560474872589111</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -580,7 +580,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1550735235214233</v>
+        <v>0.2323299646377563</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -622,7 +622,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1605579853057861</v>
+        <v>0.209613561630249</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -664,7 +664,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1451530456542969</v>
+        <v>0.2195870876312256</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -706,7 +706,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1230236291885376</v>
+        <v>0.1800320148468018</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -748,28 +748,28 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E8" t="n">
-        <v>1.443973541259766</v>
+        <v>2.208785533905029</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>14.85380497008206</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="H8" t="n">
-        <v>16.97265533633956</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="I8" t="n">
-        <v>14.85380497008206</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="J8" t="n">
-        <v>16.97265533633956</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="K8" t="n">
-        <v>2.996506924600562</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>40.8812863223495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -790,7 +790,7 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E9" t="n">
-        <v>1.384750962257385</v>
+        <v>1.87408185005188</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -799,19 +799,19 @@
         <v>53.31120138136255</v>
       </c>
       <c r="H9" t="n">
-        <v>61.93413105711938</v>
+        <v>71.54312232662042</v>
       </c>
       <c r="I9" t="n">
         <v>53.31120138136255</v>
       </c>
       <c r="J9" t="n">
-        <v>61.93413105711938</v>
+        <v>71.54312232662042</v>
       </c>
       <c r="K9" t="n">
-        <v>12.19466409484474</v>
+        <v>25.78382986889779</v>
       </c>
       <c r="L9" t="n">
-        <v>16.17470522577903</v>
+        <v>34.19904348963274</v>
       </c>
     </row>
     <row r="10">
@@ -832,28 +832,28 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E10" t="n">
-        <v>1.29051148891449</v>
+        <v>2.076209902763367</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>15.8005198685139</v>
+        <v>14.30549412930885</v>
       </c>
       <c r="H10" t="n">
-        <v>30.2245905953487</v>
+        <v>15.70865287257833</v>
       </c>
       <c r="I10" t="n">
-        <v>15.8005198685139</v>
+        <v>14.30549412930885</v>
       </c>
       <c r="J10" t="n">
-        <v>30.2245905953487</v>
+        <v>15.70865287257833</v>
       </c>
       <c r="K10" t="n">
-        <v>20.39871644651851</v>
+        <v>1.984366124894086</v>
       </c>
       <c r="L10" t="n">
-        <v>150.8787881011339</v>
+        <v>30.38945169303061</v>
       </c>
     </row>
     <row r="11">
@@ -874,28 +874,28 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E11" t="n">
-        <v>1.1657555103302</v>
+        <v>2.172906517982483</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>72.52918392036464</v>
+        <v>92.26506707964212</v>
       </c>
       <c r="H11" t="n">
-        <v>83.1256302365048</v>
+        <v>96.48899236834549</v>
       </c>
       <c r="I11" t="n">
-        <v>72.52918392036464</v>
+        <v>92.26506707964212</v>
       </c>
       <c r="J11" t="n">
-        <v>83.1256302365048</v>
+        <v>96.48899236834549</v>
       </c>
       <c r="K11" t="n">
-        <v>14.98563809324384</v>
+        <v>5.973532429735007</v>
       </c>
       <c r="L11" t="n">
-        <v>55.92526163847678</v>
+        <v>80.9919676694395</v>
       </c>
     </row>
     <row r="12">
@@ -916,28 +916,28 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5183384418487549</v>
+        <v>1.024685978889465</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>12.65112876324897</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="H12" t="n">
-        <v>13.47831144627891</v>
+        <v>12.79500035314562</v>
       </c>
       <c r="I12" t="n">
-        <v>12.65112876324897</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="J12" t="n">
-        <v>13.47831144627891</v>
+        <v>12.79500035314562</v>
       </c>
       <c r="K12" t="n">
-        <v>1.169812968901101</v>
+        <v>1.057142838240327</v>
       </c>
       <c r="L12" t="n">
-        <v>11.87653412954634</v>
+        <v>6.204720034975211</v>
       </c>
     </row>
     <row r="13">
@@ -958,7 +958,7 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E13" t="n">
-        <v>0.7316831350326538</v>
+        <v>0.9763690233230591</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -966,10 +966,10 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>51.88359465737358</v>
+        <v>68.92877929865904</v>
       </c>
       <c r="J13" t="n">
-        <v>82.06383020095066</v>
+        <v>69.17090219324498</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -992,7 +992,7 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E14" t="n">
-        <v>1.582887530326843</v>
+        <v>2.249275088310242</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1001,19 +1001,19 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="H14" t="n">
-        <v>-11.80593354076133</v>
+        <v>-8.711459618087822</v>
       </c>
       <c r="I14" t="n">
         <v>-11.80593354076133</v>
       </c>
       <c r="J14" t="n">
-        <v>-11.80593354076133</v>
+        <v>-8.711459618087822</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>4.376246989854746</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>26.21117518567663</v>
       </c>
     </row>
     <row r="15">
@@ -1034,7 +1034,7 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E15" t="n">
-        <v>1.621106863021851</v>
+        <v>2.926261067390442</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1043,19 +1043,19 @@
         <v>13.7263575295875</v>
       </c>
       <c r="H15" t="n">
-        <v>31.61766331366255</v>
+        <v>31.77703718137579</v>
       </c>
       <c r="I15" t="n">
         <v>13.7263575295875</v>
       </c>
       <c r="J15" t="n">
-        <v>31.61766331366255</v>
+        <v>31.77703718137579</v>
       </c>
       <c r="K15" t="n">
-        <v>25.30212728840313</v>
+        <v>25.52751597361105</v>
       </c>
       <c r="L15" t="n">
-        <v>130.3427055976787</v>
+        <v>131.5037846921851</v>
       </c>
     </row>
     <row r="16">
@@ -1076,28 +1076,28 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E16" t="n">
-        <v>1.309327960014343</v>
+        <v>2.407869577407837</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>39.72488517994941</v>
+        <v>0.5026689075177071</v>
       </c>
       <c r="H16" t="n">
-        <v>40.98727807210688</v>
+        <v>19.20625020654619</v>
       </c>
       <c r="I16" t="n">
-        <v>39.72488517994941</v>
+        <v>0.5026689075177071</v>
       </c>
       <c r="J16" t="n">
-        <v>40.98727807210688</v>
+        <v>19.20625020654619</v>
       </c>
       <c r="K16" t="n">
-        <v>1.785293149132492</v>
+        <v>26.45085833803386</v>
       </c>
       <c r="L16" t="n">
-        <v>447.175239726648</v>
+        <v>262.6830283283776</v>
       </c>
     </row>
     <row r="17">
@@ -1118,28 +1118,28 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E17" t="n">
-        <v>1.405153036117554</v>
+        <v>2.028071999549866</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>13.7263575295875</v>
+        <v>25.88816206668601</v>
       </c>
       <c r="H17" t="n">
-        <v>36.66666803133866</v>
+        <v>34.7539309139832</v>
       </c>
       <c r="I17" t="n">
-        <v>13.7263575295875</v>
+        <v>25.88816206668601</v>
       </c>
       <c r="J17" t="n">
-        <v>36.66666803133866</v>
+        <v>34.7539309139832</v>
       </c>
       <c r="K17" t="n">
-        <v>32.44249823662643</v>
+        <v>12.53809054471256</v>
       </c>
       <c r="L17" t="n">
-        <v>167.1259870093195</v>
+        <v>153.1912114271411</v>
       </c>
     </row>
     <row r="18">
@@ -1160,28 +1160,28 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E18" t="n">
-        <v>0.4789414405822754</v>
+        <v>0.698172926902771</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>-11.80593354076133</v>
+        <v>-8.169823059957809</v>
       </c>
       <c r="H18" t="n">
-        <v>-11.72964416890517</v>
+        <v>-7.102065796069484</v>
       </c>
       <c r="I18" t="n">
-        <v>-11.80593354076133</v>
+        <v>-8.169823059957809</v>
       </c>
       <c r="J18" t="n">
-        <v>-11.72964416890517</v>
+        <v>-7.102065796069484</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1078894643439047</v>
+        <v>1.510036803913257</v>
       </c>
       <c r="L18" t="n">
-        <v>0.6461951661235557</v>
+        <v>39.84325109447048</v>
       </c>
     </row>
     <row r="19">
@@ -1202,28 +1202,28 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E19" t="n">
-        <v>0.4869565963745117</v>
+        <v>0.6382509469985962</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>45.30650006659124</v>
+        <v>62.4553615479396</v>
       </c>
       <c r="H19" t="n">
-        <v>67.02436933573958</v>
+        <v>71.34469295659733</v>
       </c>
       <c r="I19" t="n">
-        <v>45.30650006659124</v>
+        <v>62.4553615479396</v>
       </c>
       <c r="J19" t="n">
-        <v>67.02436933573958</v>
+        <v>71.34469295659733</v>
       </c>
       <c r="K19" t="n">
-        <v>30.71370526627544</v>
+        <v>12.5714130385529</v>
       </c>
       <c r="L19" t="n">
-        <v>388.2895494399508</v>
+        <v>419.7642040345523</v>
       </c>
     </row>
     <row r="20">
@@ -1244,7 +1244,7 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E20" t="n">
-        <v>1.84122896194458</v>
+        <v>3.315737009048462</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
@@ -1253,19 +1253,19 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="H20" t="n">
-        <v>-3.525999573404519</v>
+        <v>-6.610943701841151</v>
       </c>
       <c r="I20" t="n">
         <v>-9.463170998014522</v>
       </c>
       <c r="J20" t="n">
-        <v>-3.525999573404519</v>
+        <v>-6.610943701841151</v>
       </c>
       <c r="K20" t="n">
-        <v>8.396428350817457</v>
+        <v>4.033658525219125</v>
       </c>
       <c r="L20" t="n">
-        <v>62.73976689056646</v>
+        <v>30.14029120652897</v>
       </c>
     </row>
     <row r="21">
@@ -1286,28 +1286,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E21" t="n">
-        <v>1.776646018028259</v>
+        <v>2.555391430854797</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>24.95684465099749</v>
+        <v>18.7915703518064</v>
       </c>
       <c r="H21" t="n">
-        <v>38.69295841698259</v>
+        <v>21.87420750140194</v>
       </c>
       <c r="I21" t="n">
-        <v>24.95684465099749</v>
+        <v>18.7915703518064</v>
       </c>
       <c r="J21" t="n">
-        <v>38.69295841698259</v>
+        <v>21.87420750140194</v>
       </c>
       <c r="K21" t="n">
-        <v>19.4257983821559</v>
+        <v>4.359507264833161</v>
       </c>
       <c r="L21" t="n">
-        <v>156.7638052472738</v>
+        <v>45.15573335853543</v>
       </c>
     </row>
     <row r="22">
@@ -1328,28 +1328,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E22" t="n">
-        <v>1.591809511184692</v>
+        <v>3.023475885391235</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>10.33393430533935</v>
+        <v>62.63282583590009</v>
       </c>
       <c r="H22" t="n">
-        <v>25.73572911723092</v>
+        <v>62.79666229882476</v>
       </c>
       <c r="I22" t="n">
-        <v>10.33393430533935</v>
+        <v>62.63282583590009</v>
       </c>
       <c r="J22" t="n">
-        <v>25.73572911723092</v>
+        <v>62.79666229882476</v>
       </c>
       <c r="K22" t="n">
-        <v>21.78142710786463</v>
+        <v>0.2316997478793013</v>
       </c>
       <c r="L22" t="n">
-        <v>371.9567164392419</v>
+        <v>763.5900620627079</v>
       </c>
     </row>
     <row r="23">
@@ -1370,28 +1370,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E23" t="n">
-        <v>1.499621033668518</v>
+        <v>2.651947498321533</v>
       </c>
       <c r="F23" t="n">
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>46.29537378316995</v>
+        <v>32.96849945095311</v>
       </c>
       <c r="H23" t="n">
-        <v>48.37569742446321</v>
+        <v>52.19100454732985</v>
       </c>
       <c r="I23" t="n">
-        <v>46.29537378316995</v>
+        <v>32.96849945095311</v>
       </c>
       <c r="J23" t="n">
-        <v>48.37569742446321</v>
+        <v>52.19100454732985</v>
       </c>
       <c r="K23" t="n">
-        <v>2.942021907642308</v>
+        <v>27.18472741008192</v>
       </c>
       <c r="L23" t="n">
-        <v>221.0177939442388</v>
+        <v>246.3359090518265</v>
       </c>
     </row>
     <row r="24">
@@ -1412,7 +1412,7 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E24" t="n">
-        <v>0.5403419733047485</v>
+        <v>0.8672384023666382</v>
       </c>
       <c r="F24" t="n">
         <v>100</v>
@@ -1454,28 +1454,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E25" t="n">
-        <v>0.5433415174484253</v>
+        <v>0.8521039485931396</v>
       </c>
       <c r="F25" t="n">
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>18.7915703518064</v>
+        <v>16.24913000637435</v>
       </c>
       <c r="H25" t="n">
-        <v>29.99509282652012</v>
+        <v>33.10464389075921</v>
       </c>
       <c r="I25" t="n">
-        <v>18.7915703518064</v>
+        <v>16.24913000637435</v>
       </c>
       <c r="J25" t="n">
-        <v>29.99509282652012</v>
+        <v>33.10464389075921</v>
       </c>
       <c r="K25" t="n">
-        <v>15.84417343009194</v>
+        <v>23.83729633606507</v>
       </c>
       <c r="L25" t="n">
-        <v>99.04536866589675</v>
+        <v>119.6801352107652</v>
       </c>
     </row>
     <row r="26">
@@ -1496,28 +1496,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E26" t="n">
-        <v>1.924139976501465</v>
+        <v>2.750033020973206</v>
       </c>
       <c r="F26" t="n">
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>-2.607775564475329</v>
+        <v>-21.96317396534843</v>
       </c>
       <c r="H26" t="n">
-        <v>-1.457238682166235</v>
+        <v>-15.27342337758164</v>
       </c>
       <c r="I26" t="n">
-        <v>-2.607775564475329</v>
+        <v>-21.96317396534843</v>
       </c>
       <c r="J26" t="n">
-        <v>-1.457238682166235</v>
+        <v>-15.27342337758164</v>
       </c>
       <c r="K26" t="n">
-        <v>1.627104862971978</v>
+        <v>9.460736010113177</v>
       </c>
       <c r="L26" t="n">
-        <v>93.36508154756986</v>
+        <v>30.45894276629275</v>
       </c>
     </row>
     <row r="27">
@@ -1538,28 +1538,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E27" t="n">
-        <v>1.895413517951965</v>
+        <v>2.646108508110046</v>
       </c>
       <c r="F27" t="n">
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>65.15238928403269</v>
+        <v>41.59734965676242</v>
       </c>
       <c r="H27" t="n">
-        <v>68.85094121238041</v>
+        <v>41.59734965676242</v>
       </c>
       <c r="I27" t="n">
-        <v>65.15238928403269</v>
+        <v>41.59734965676242</v>
       </c>
       <c r="J27" t="n">
-        <v>68.85094121238041</v>
+        <v>41.59734965676242</v>
       </c>
       <c r="K27" t="n">
-        <v>5.230542298210488</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>201.3898058879608</v>
+        <v>82.08926294606582</v>
       </c>
     </row>
     <row r="28">
@@ -1580,28 +1580,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E28" t="n">
-        <v>1.604251384735107</v>
+        <v>2.440184473991394</v>
       </c>
       <c r="F28" t="n">
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>8.365720359311478</v>
+        <v>0.2335566311363841</v>
       </c>
       <c r="H28" t="n">
-        <v>24.65419204330385</v>
+        <v>1.151394825260116</v>
       </c>
       <c r="I28" t="n">
-        <v>8.365720359311478</v>
+        <v>0.2335566311363841</v>
       </c>
       <c r="J28" t="n">
-        <v>24.65419204330385</v>
+        <v>1.151394825260116</v>
       </c>
       <c r="K28" t="n">
-        <v>23.03537756583214</v>
+        <v>1.298019222193811</v>
       </c>
       <c r="L28" t="n">
-        <v>212.2524097937806</v>
+        <v>105.2423881315</v>
       </c>
     </row>
     <row r="29">
@@ -1622,28 +1622,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E29" t="n">
-        <v>1.534374475479126</v>
+        <v>2.216222524642944</v>
       </c>
       <c r="F29" t="n">
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>47.33674845291898</v>
+        <v>61.15072389658807</v>
       </c>
       <c r="H29" t="n">
-        <v>57.43106372002855</v>
+        <v>66.85010851865809</v>
       </c>
       <c r="I29" t="n">
-        <v>47.33674845291898</v>
+        <v>61.15072389658807</v>
       </c>
       <c r="J29" t="n">
-        <v>57.43106372002855</v>
+        <v>66.85010851865809</v>
       </c>
       <c r="K29" t="n">
-        <v>14.27551755361615</v>
+        <v>8.060147029712075</v>
       </c>
       <c r="L29" t="n">
-        <v>151.4001528770107</v>
+        <v>192.6313115731899</v>
       </c>
     </row>
     <row r="30">
@@ -1664,28 +1664,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E30" t="n">
-        <v>0.6272546052932739</v>
+        <v>0.8654625415802002</v>
       </c>
       <c r="F30" t="n">
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>-15.98727674000891</v>
+        <v>-13.14594454439719</v>
       </c>
       <c r="H30" t="n">
-        <v>-15.54734572373263</v>
+        <v>-9.392834872245661</v>
       </c>
       <c r="I30" t="n">
-        <v>-15.98727674000891</v>
+        <v>-13.14594454439719</v>
       </c>
       <c r="J30" t="n">
-        <v>-15.54734572373263</v>
+        <v>-9.392834872245661</v>
       </c>
       <c r="K30" t="n">
-        <v>0.6221564097264832</v>
+        <v>5.307698599430339</v>
       </c>
       <c r="L30" t="n">
-        <v>29.21175350947968</v>
+        <v>57.23370908473952</v>
       </c>
     </row>
     <row r="31">
@@ -1706,7 +1706,7 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E31" t="n">
-        <v>0.8941030502319336</v>
+        <v>1.278178930282593</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1714,10 +1714,10 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>16.43121162157897</v>
+        <v>46.6984995090151</v>
       </c>
       <c r="J31" t="n">
-        <v>39.06670239999863</v>
+        <v>95.85394678574264</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -1740,7 +1740,7 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E32" t="n">
-        <v>2.170654058456421</v>
+        <v>465.5156199932098</v>
       </c>
       <c r="F32" t="n">
         <v>100</v>
@@ -1782,28 +1782,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E33" t="n">
-        <v>2.151087045669556</v>
+        <v>3.683505535125732</v>
       </c>
       <c r="F33" t="n">
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9171894075994231</v>
+        <v>8.879139472792978</v>
       </c>
       <c r="H33" t="n">
-        <v>1.135611476462101</v>
+        <v>38.75393089650036</v>
       </c>
       <c r="I33" t="n">
-        <v>0.9171894075994231</v>
+        <v>8.879139472792978</v>
       </c>
       <c r="J33" t="n">
-        <v>1.135611476462101</v>
+        <v>38.75393089650036</v>
       </c>
       <c r="K33" t="n">
-        <v>0.3088954521071889</v>
+        <v>42.24933520447441</v>
       </c>
       <c r="L33" t="n">
-        <v>208.080991424326</v>
+        <v>3788.377019517875</v>
       </c>
     </row>
     <row r="34">
@@ -1824,28 +1824,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E34" t="n">
-        <v>1.96436595916748</v>
+        <v>3.425153017044067</v>
       </c>
       <c r="F34" t="n">
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>36.68505247955579</v>
+        <v>28.85855892124502</v>
       </c>
       <c r="H34" t="n">
-        <v>46.15967760528618</v>
+        <v>48.26793310539241</v>
       </c>
       <c r="I34" t="n">
-        <v>36.68505247955579</v>
+        <v>28.85855892124502</v>
       </c>
       <c r="J34" t="n">
-        <v>46.15967760528618</v>
+        <v>48.26793310539241</v>
       </c>
       <c r="K34" t="n">
-        <v>13.3991433512088</v>
+        <v>27.44900020839546</v>
       </c>
       <c r="L34" t="n">
-        <v>622.0921072558835</v>
+        <v>645.937671475297</v>
       </c>
     </row>
     <row r="35">
@@ -1866,28 +1866,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E35" t="n">
-        <v>2.056630492210388</v>
+        <v>3.061335921287537</v>
       </c>
       <c r="F35" t="n">
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>97.402649913666</v>
+        <v>36.30781961336751</v>
       </c>
       <c r="H35" t="n">
-        <v>134.2291270962957</v>
+        <v>71.40702222719864</v>
       </c>
       <c r="I35" t="n">
-        <v>97.402649913666</v>
+        <v>36.30781961336751</v>
       </c>
       <c r="J35" t="n">
-        <v>134.2291270962957</v>
+        <v>71.40702222719864</v>
       </c>
       <c r="K35" t="n">
-        <v>52.08050348609818</v>
+        <v>49.63776836496116</v>
       </c>
       <c r="L35" t="n">
-        <v>12875.15896527104</v>
+        <v>6896.111096920636</v>
       </c>
     </row>
     <row r="36">
@@ -1908,28 +1908,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E36" t="n">
-        <v>0.6229759454727173</v>
+        <v>0.9803160429000854</v>
       </c>
       <c r="F36" t="n">
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>-7.721703651991684</v>
+        <v>-7.873400703841429</v>
       </c>
       <c r="H36" t="n">
-        <v>-6.737756866620251</v>
+        <v>-5.339245001016813</v>
       </c>
       <c r="I36" t="n">
-        <v>-7.721703651991684</v>
+        <v>-7.873400703841429</v>
       </c>
       <c r="J36" t="n">
-        <v>-6.737756866620251</v>
+        <v>-5.339245001016813</v>
       </c>
       <c r="K36" t="n">
-        <v>1.39151088852569</v>
+        <v>3.583837364099694</v>
       </c>
       <c r="L36" t="n">
-        <v>23.79215230331856</v>
+        <v>39.61011388396095</v>
       </c>
     </row>
     <row r="37">
@@ -1950,28 +1950,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E37" t="n">
-        <v>0.6217255592346191</v>
+        <v>1.021799564361572</v>
       </c>
       <c r="F37" t="n">
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>30.74712463818992</v>
+        <v>36.88818255616685</v>
       </c>
       <c r="H37" t="n">
-        <v>42.39067593702021</v>
+        <v>41.60736433343054</v>
       </c>
       <c r="I37" t="n">
-        <v>30.74712463818992</v>
+        <v>36.88818255616685</v>
       </c>
       <c r="J37" t="n">
-        <v>42.39067593702021</v>
+        <v>41.60736433343054</v>
       </c>
       <c r="K37" t="n">
-        <v>16.46646816099266</v>
+        <v>6.673930872710275</v>
       </c>
       <c r="L37" t="n">
-        <v>4134.50156799588</v>
+        <v>4059.950459218867</v>
       </c>
     </row>
     <row r="38">
@@ -1992,28 +1992,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E38" t="n">
-        <v>2.21416449546814</v>
+        <v>3.443254470825195</v>
       </c>
       <c r="F38" t="n">
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>9.383712874145662</v>
+        <v>22.59132042530658</v>
       </c>
       <c r="H38" t="n">
-        <v>19.5772252172476</v>
+        <v>22.59132042530658</v>
       </c>
       <c r="I38" t="n">
-        <v>9.383712874145662</v>
+        <v>22.59132042530658</v>
       </c>
       <c r="J38" t="n">
-        <v>19.5772252172476</v>
+        <v>22.59132042530658</v>
       </c>
       <c r="K38" t="n">
-        <v>14.4158034038323</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>108.6298406592071</v>
+        <v>140.7503376147729</v>
       </c>
     </row>
     <row r="39">
@@ -2034,28 +2034,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E39" t="n">
-        <v>2.120435953140259</v>
+        <v>3.465409636497498</v>
       </c>
       <c r="F39" t="n">
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>28.76144092819549</v>
+        <v>47.11403373166605</v>
       </c>
       <c r="H39" t="n">
-        <v>43.71740847522364</v>
+        <v>51.25518788027289</v>
       </c>
       <c r="I39" t="n">
-        <v>28.76144092819549</v>
+        <v>47.11403373166605</v>
       </c>
       <c r="J39" t="n">
-        <v>43.71740847522364</v>
+        <v>51.25518788027289</v>
       </c>
       <c r="K39" t="n">
-        <v>21.15093214341908</v>
+        <v>5.856476360837397</v>
       </c>
       <c r="L39" t="n">
-        <v>66.75728120358741</v>
+        <v>95.50966254867075</v>
       </c>
     </row>
     <row r="40">
@@ -2076,28 +2076,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E40" t="n">
-        <v>1.899668455123901</v>
+        <v>465.5606260299683</v>
       </c>
       <c r="F40" t="n">
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>57.64306213640211</v>
+        <v>24.33836247401486</v>
       </c>
       <c r="H40" t="n">
-        <v>64.3881658379531</v>
+        <v>46.14170880979383</v>
       </c>
       <c r="I40" t="n">
-        <v>57.64306213640211</v>
+        <v>24.33836247401486</v>
       </c>
       <c r="J40" t="n">
-        <v>64.3881658379531</v>
+        <v>46.14170880979383</v>
       </c>
       <c r="K40" t="n">
-        <v>9.539017134346382</v>
+        <v>30.83458809317634</v>
       </c>
       <c r="L40" t="n">
-        <v>586.1693947963568</v>
+        <v>391.7212347462709</v>
       </c>
     </row>
     <row r="41">
@@ -2118,28 +2118,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E41" t="n">
-        <v>1.86066460609436</v>
+        <v>2.627735137939453</v>
       </c>
       <c r="F41" t="n">
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>45.21469087899347</v>
+        <v>64.85251503761866</v>
       </c>
       <c r="H41" t="n">
-        <v>54.16162450635362</v>
+        <v>68.43066255375317</v>
       </c>
       <c r="I41" t="n">
-        <v>45.21469087899347</v>
+        <v>64.85251503761866</v>
       </c>
       <c r="J41" t="n">
-        <v>54.16162450635362</v>
+        <v>68.43066255375317</v>
       </c>
       <c r="K41" t="n">
-        <v>12.65287487746464</v>
+        <v>5.060264745489033</v>
       </c>
       <c r="L41" t="n">
-        <v>106.5960806749975</v>
+        <v>161.0244210813926</v>
       </c>
     </row>
     <row r="42">
@@ -2160,28 +2160,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E42" t="n">
-        <v>0.6116855144500732</v>
+        <v>1.117673993110657</v>
       </c>
       <c r="F42" t="n">
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>17.26945599762524</v>
+        <v>12.27487551745429</v>
       </c>
       <c r="H42" t="n">
-        <v>20.90655424000018</v>
+        <v>15.81821726544116</v>
       </c>
       <c r="I42" t="n">
-        <v>17.26945599762524</v>
+        <v>12.27487551745429</v>
       </c>
       <c r="J42" t="n">
-        <v>20.90655424000018</v>
+        <v>15.81821726544116</v>
       </c>
       <c r="K42" t="n">
-        <v>5.143633662049984</v>
+        <v>5.011041956125819</v>
       </c>
       <c r="L42" t="n">
-        <v>122.7961844144087</v>
+        <v>68.57098546806635</v>
       </c>
     </row>
     <row r="43">
@@ -2202,28 +2202,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E43" t="n">
-        <v>0.6274008750915527</v>
+        <v>1.000574111938477</v>
       </c>
       <c r="F43" t="n">
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>51.11787422330842</v>
+        <v>37.30839655754299</v>
       </c>
       <c r="H43" t="n">
-        <v>58.65245821165009</v>
+        <v>45.05696213871855</v>
       </c>
       <c r="I43" t="n">
-        <v>51.11787422330842</v>
+        <v>37.30839655754299</v>
       </c>
       <c r="J43" t="n">
-        <v>58.65245821165009</v>
+        <v>45.05696213871855</v>
       </c>
       <c r="K43" t="n">
-        <v>10.65551086315196</v>
+        <v>10.95812653383584</v>
       </c>
       <c r="L43" t="n">
-        <v>123.7260809461044</v>
+        <v>71.8669236719262</v>
       </c>
     </row>
     <row r="44">
@@ -2244,7 +2244,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E44" t="n">
-        <v>0.389163613319397</v>
+        <v>0.6547136306762695</v>
       </c>
       <c r="F44" t="n">
         <v>100</v>
@@ -2286,7 +2286,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E45" t="n">
-        <v>0.4014264345169067</v>
+        <v>0.6624289751052856</v>
       </c>
       <c r="F45" t="n">
         <v>100</v>
@@ -2328,7 +2328,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3391854763031006</v>
+        <v>0.5523040294647217</v>
       </c>
       <c r="F46" t="n">
         <v>100</v>
@@ -2370,7 +2370,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3458728790283203</v>
+        <v>0.6156669855117798</v>
       </c>
       <c r="F47" t="n">
         <v>100</v>
@@ -2412,7 +2412,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E48" t="n">
-        <v>0.2402980327606201</v>
+        <v>0.411470890045166</v>
       </c>
       <c r="F48" t="n">
         <v>100</v>
@@ -2454,7 +2454,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E49" t="n">
-        <v>0.2479870319366455</v>
+        <v>0.4161912202835083</v>
       </c>
       <c r="F49" t="n">
         <v>100</v>
@@ -2496,28 +2496,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E50" t="n">
-        <v>3.59077000617981</v>
+        <v>5.851077079772949</v>
       </c>
       <c r="F50" t="n">
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>18.1160688409129</v>
+        <v>23.33980807164679</v>
       </c>
       <c r="H50" t="n">
-        <v>29.08139214152294</v>
+        <v>30.5050819500722</v>
       </c>
       <c r="I50" t="n">
-        <v>18.1160688409129</v>
+        <v>23.33980807164679</v>
       </c>
       <c r="J50" t="n">
-        <v>29.08139214152294</v>
+        <v>30.5050819500722</v>
       </c>
       <c r="K50" t="n">
-        <v>15.50730892752843</v>
+        <v>10.13322749698689</v>
       </c>
       <c r="L50" t="n">
-        <v>123.2819507959453</v>
+        <v>134.2127974429772</v>
       </c>
     </row>
     <row r="51">
@@ -2538,28 +2538,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E51" t="n">
-        <v>3.48322606086731</v>
+        <v>5.607861042022705</v>
       </c>
       <c r="F51" t="n">
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>50.42459305219376</v>
+        <v>37.60618409062889</v>
       </c>
       <c r="H51" t="n">
-        <v>60.86071461069994</v>
+        <v>62.58086547125905</v>
       </c>
       <c r="I51" t="n">
-        <v>50.42459305219376</v>
+        <v>37.60618409062889</v>
       </c>
       <c r="J51" t="n">
-        <v>60.86071461069994</v>
+        <v>62.58086547125905</v>
       </c>
       <c r="K51" t="n">
-        <v>14.75890464661369</v>
+        <v>35.31953312443398</v>
       </c>
       <c r="L51" t="n">
-        <v>160.7602664672986</v>
+        <v>168.1303244699447</v>
       </c>
     </row>
     <row r="52">
@@ -2580,28 +2580,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E52" t="n">
-        <v>3.063130140304565</v>
+        <v>467.0280684232712</v>
       </c>
       <c r="F52" t="n">
         <v>100</v>
       </c>
       <c r="G52" t="n">
-        <v>90.73369139894112</v>
+        <v>85.84998587345601</v>
       </c>
       <c r="H52" t="n">
-        <v>113.1193824293239</v>
+        <v>97.126155679452</v>
       </c>
       <c r="I52" t="n">
-        <v>90.73369139894112</v>
+        <v>85.84998587345601</v>
       </c>
       <c r="J52" t="n">
-        <v>113.1193824293239</v>
+        <v>97.126155679452</v>
       </c>
       <c r="K52" t="n">
-        <v>31.65814785826104</v>
+        <v>15.94691227126152</v>
       </c>
       <c r="L52" t="n">
-        <v>768.5112548511347</v>
+        <v>645.7179975388566</v>
       </c>
     </row>
     <row r="53">
@@ -2622,28 +2622,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E53" t="n">
-        <v>3.035805106163025</v>
+        <v>4.750369071960449</v>
       </c>
       <c r="F53" t="n">
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>133.2787803339714</v>
+        <v>104.8790602339446</v>
       </c>
       <c r="H53" t="n">
-        <v>152.9803108294141</v>
+        <v>125.5447688460301</v>
       </c>
       <c r="I53" t="n">
-        <v>133.2787803339714</v>
+        <v>104.8790602339446</v>
       </c>
       <c r="J53" t="n">
-        <v>152.9803108294141</v>
+        <v>125.5447688460301</v>
       </c>
       <c r="K53" t="n">
-        <v>27.86217162616227</v>
+        <v>29.22572539526174</v>
       </c>
       <c r="L53" t="n">
-        <v>555.4505130492655</v>
+        <v>437.9017907901905</v>
       </c>
     </row>
     <row r="54">
@@ -2664,28 +2664,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E54" t="n">
-        <v>0.861793041229248</v>
+        <v>1.371070981025696</v>
       </c>
       <c r="F54" t="n">
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>44.82790848591027</v>
+        <v>45.10722060186758</v>
       </c>
       <c r="H54" t="n">
-        <v>45.13497606419387</v>
+        <v>48.20397494551293</v>
       </c>
       <c r="I54" t="n">
-        <v>44.82790848591027</v>
+        <v>45.10722060186758</v>
       </c>
       <c r="J54" t="n">
-        <v>45.13497606419387</v>
+        <v>48.20397494551293</v>
       </c>
       <c r="K54" t="n">
-        <v>0.43425913377373</v>
+        <v>4.379471992121048</v>
       </c>
       <c r="L54" t="n">
-        <v>246.5386201492123</v>
+        <v>270.1018682178313</v>
       </c>
     </row>
     <row r="55">
@@ -2706,28 +2706,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E55" t="n">
-        <v>0.9446874856948853</v>
+        <v>1.506063938140869</v>
       </c>
       <c r="F55" t="n">
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>83.97923057846313</v>
+        <v>44.69314660602799</v>
       </c>
       <c r="H55" t="n">
-        <v>96.71780074624994</v>
+        <v>53.69198389024518</v>
       </c>
       <c r="I55" t="n">
-        <v>83.97923057846313</v>
+        <v>44.69314660602799</v>
       </c>
       <c r="J55" t="n">
-        <v>96.71780074624994</v>
+        <v>53.69198389024518</v>
       </c>
       <c r="K55" t="n">
-        <v>18.01505869652541</v>
+        <v>12.72627773292862</v>
       </c>
       <c r="L55" t="n">
-        <v>314.3914453855141</v>
+        <v>130.0455411333071</v>
       </c>
     </row>
     <row r="56">
@@ -2748,7 +2748,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E56" t="n">
-        <v>0.3939559459686279</v>
+        <v>0.7194430828094482</v>
       </c>
       <c r="F56" t="n">
         <v>100</v>
@@ -2790,7 +2790,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E57" t="n">
-        <v>0.4062560796737671</v>
+        <v>0.6846519708633423</v>
       </c>
       <c r="F57" t="n">
         <v>100</v>
@@ -2832,7 +2832,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E58" t="n">
-        <v>0.3397489786148071</v>
+        <v>0.5479069948196411</v>
       </c>
       <c r="F58" t="n">
         <v>100</v>
@@ -2874,7 +2874,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E59" t="n">
-        <v>0.3484299182891846</v>
+        <v>0.6053630113601685</v>
       </c>
       <c r="F59" t="n">
         <v>100</v>
@@ -2916,7 +2916,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E60" t="n">
-        <v>0.2005469799041748</v>
+        <v>0.3329730033874512</v>
       </c>
       <c r="F60" t="n">
         <v>100</v>
@@ -2958,7 +2958,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E61" t="n">
-        <v>0.198589563369751</v>
+        <v>0.3177584409713745</v>
       </c>
       <c r="F61" t="n">
         <v>100</v>
@@ -3000,7 +3000,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E62" t="n">
-        <v>0.5731929540634155</v>
+        <v>0.9197906255722046</v>
       </c>
       <c r="F62" t="n">
         <v>100</v>
@@ -3042,7 +3042,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E63" t="n">
-        <v>0.5691496133804321</v>
+        <v>0.8821635246276855</v>
       </c>
       <c r="F63" t="n">
         <v>100</v>
@@ -3084,7 +3084,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E64" t="n">
-        <v>0.4780590534210205</v>
+        <v>0.8245415687561035</v>
       </c>
       <c r="F64" t="n">
         <v>100</v>
@@ -3093,19 +3093,19 @@
         <v>24.82249030015713</v>
       </c>
       <c r="H64" t="n">
-        <v>25.98274676680382</v>
+        <v>24.82249030015713</v>
       </c>
       <c r="I64" t="n">
         <v>24.82249030015713</v>
       </c>
       <c r="J64" t="n">
-        <v>25.98274676680382</v>
+        <v>24.82249030015713</v>
       </c>
       <c r="K64" t="n">
-        <v>1.64085043096283</v>
+        <v>0</v>
       </c>
       <c r="L64" t="n">
-        <v>4.674214603839895</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -3126,7 +3126,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E65" t="n">
-        <v>0.4742070436477661</v>
+        <v>0.7692196369171143</v>
       </c>
       <c r="F65" t="n">
         <v>100</v>
@@ -3135,19 +3135,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H65" t="n">
-        <v>48.65032644645115</v>
+        <v>52.47888399062607</v>
       </c>
       <c r="I65" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J65" t="n">
-        <v>48.65032644645115</v>
+        <v>52.47888399062607</v>
       </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>5.414398003298002</v>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>7.869541324432776</v>
       </c>
     </row>
     <row r="66">
@@ -3168,7 +3168,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E66" t="n">
-        <v>0.2346640825271606</v>
+        <v>0.4185529947280884</v>
       </c>
       <c r="F66" t="n">
         <v>100</v>
@@ -3210,7 +3210,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E67" t="n">
-        <v>0.2884923219680786</v>
+        <v>0.4796780347824097</v>
       </c>
       <c r="F67" t="n">
         <v>100</v>
@@ -3252,7 +3252,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E68" t="n">
-        <v>0.1919745206832886</v>
+        <v>0.3050709962844849</v>
       </c>
       <c r="F68" t="n">
         <v>100</v>
@@ -3294,7 +3294,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E69" t="n">
-        <v>0.1975950002670288</v>
+        <v>0.316988468170166</v>
       </c>
       <c r="F69" t="n">
         <v>100</v>
@@ -3336,7 +3336,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E70" t="n">
-        <v>0.1522724628448486</v>
+        <v>0.2418564558029175</v>
       </c>
       <c r="F70" t="n">
         <v>100</v>
@@ -3378,7 +3378,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E71" t="n">
-        <v>0.1542540788650513</v>
+        <v>0.2447580099105835</v>
       </c>
       <c r="F71" t="n">
         <v>100</v>
@@ -3420,7 +3420,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E72" t="n">
-        <v>0.09960663318634033</v>
+        <v>0.1521104574203491</v>
       </c>
       <c r="F72" t="n">
         <v>100</v>
@@ -3462,7 +3462,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E73" t="n">
-        <v>0.1007434129714966</v>
+        <v>0.162079930305481</v>
       </c>
       <c r="F73" t="n">
         <v>100</v>
@@ -3504,7 +3504,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E74" t="n">
-        <v>0.6422369480133057</v>
+        <v>1.04652202129364</v>
       </c>
       <c r="F74" t="n">
         <v>100</v>
@@ -3546,7 +3546,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E75" t="n">
-        <v>0.649497389793396</v>
+        <v>1.099951505661011</v>
       </c>
       <c r="F75" t="n">
         <v>100</v>
@@ -3588,7 +3588,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E76" t="n">
-        <v>0.5644189119338989</v>
+        <v>0.8018379211425781</v>
       </c>
       <c r="F76" t="n">
         <v>100</v>
@@ -3597,19 +3597,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H76" t="n">
-        <v>30.95896547744237</v>
+        <v>35.03129664887638</v>
       </c>
       <c r="I76" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J76" t="n">
-        <v>30.95896547744237</v>
+        <v>35.03129664887638</v>
       </c>
       <c r="K76" t="n">
-        <v>0</v>
+        <v>5.759145973116683</v>
       </c>
       <c r="L76" t="n">
-        <v>0</v>
+        <v>13.15396399276078</v>
       </c>
     </row>
     <row r="77">
@@ -3630,7 +3630,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E77" t="n">
-        <v>0.5740125179290771</v>
+        <v>463.5480409860611</v>
       </c>
       <c r="F77" t="n">
         <v>100</v>
@@ -3639,19 +3639,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H77" t="n">
-        <v>42.27917555271888</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="I77" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J77" t="n">
-        <v>42.27917555271888</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="K77" t="n">
-        <v>5.759145973116689</v>
+        <v>0</v>
       </c>
       <c r="L77" t="n">
-        <v>10.65864307136757</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -3672,7 +3672,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E78" t="n">
-        <v>0.2824970483779907</v>
+        <v>0.4581534862518311</v>
       </c>
       <c r="F78" t="n">
         <v>100</v>
@@ -3714,7 +3714,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E79" t="n">
-        <v>0.2910028696060181</v>
+        <v>0.3675490617752075</v>
       </c>
       <c r="F79" t="n">
         <v>100</v>
@@ -3723,19 +3723,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H79" t="n">
-        <v>42.27917555271888</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="I79" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J79" t="n">
-        <v>42.27917555271888</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="K79" t="n">
-        <v>5.759145973116689</v>
+        <v>0</v>
       </c>
       <c r="L79" t="n">
-        <v>10.65864307136757</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -3756,7 +3756,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E80" t="n">
-        <v>0.9214990139007568</v>
+        <v>1.040823101997375</v>
       </c>
       <c r="F80" t="n">
         <v>100</v>
@@ -3798,28 +3798,28 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E81" t="n">
-        <v>0.8391155004501343</v>
+        <v>1.558430433273315</v>
       </c>
       <c r="F81" t="n">
         <v>100</v>
       </c>
       <c r="G81" t="n">
-        <v>18.17186472076723</v>
+        <v>19.29718019360264</v>
       </c>
       <c r="H81" t="n">
-        <v>20.77197819057553</v>
+        <v>19.83880259835954</v>
       </c>
       <c r="I81" t="n">
-        <v>18.17186472076723</v>
+        <v>19.29718019360264</v>
       </c>
       <c r="J81" t="n">
-        <v>20.77197819057553</v>
+        <v>19.83880259835954</v>
       </c>
       <c r="K81" t="n">
-        <v>3.677115732711864</v>
+        <v>0.7659697504923333</v>
       </c>
       <c r="L81" t="n">
-        <v>14.30845711082599</v>
+        <v>9.173180095751492</v>
       </c>
     </row>
     <row r="82">
@@ -3840,7 +3840,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E82" t="n">
-        <v>0.7322961091995239</v>
+        <v>1.132654070854187</v>
       </c>
       <c r="F82" t="n">
         <v>100</v>
@@ -3849,19 +3849,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H82" t="n">
-        <v>1.026285782096494</v>
+        <v>7.60232071121283</v>
       </c>
       <c r="I82" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J82" t="n">
-        <v>1.026285782096494</v>
+        <v>7.60232071121283</v>
       </c>
       <c r="K82" t="n">
-        <v>0</v>
+        <v>9.299917783395516</v>
       </c>
       <c r="L82" t="n">
-        <v>0</v>
+        <v>640.7605994192796</v>
       </c>
     </row>
     <row r="83">
@@ -3882,28 +3882,28 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E83" t="n">
-        <v>0.7135773897171021</v>
+        <v>1.190491080284119</v>
       </c>
       <c r="F83" t="n">
         <v>100</v>
       </c>
       <c r="G83" t="n">
-        <v>28.82591742481698</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="H83" t="n">
-        <v>28.82591742481698</v>
+        <v>23.49889107279211</v>
       </c>
       <c r="I83" t="n">
-        <v>28.82591742481698</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="J83" t="n">
-        <v>28.82591742481698</v>
+        <v>23.49889107279211</v>
       </c>
       <c r="K83" t="n">
-        <v>0</v>
+        <v>7.533552914152452</v>
       </c>
       <c r="L83" t="n">
-        <v>58.62938596430365</v>
+        <v>29.31469298215181</v>
       </c>
     </row>
     <row r="84">
@@ -3924,7 +3924,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E84" t="n">
-        <v>0.3349089622497559</v>
+        <v>0.5534210205078125</v>
       </c>
       <c r="F84" t="n">
         <v>100</v>
@@ -3966,7 +3966,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E85" t="n">
-        <v>0.3350690603256226</v>
+        <v>0.5380109548568726</v>
       </c>
       <c r="F85" t="n">
         <v>100</v>
@@ -3975,19 +3975,19 @@
         <v>18.17186472076723</v>
       </c>
       <c r="H85" t="n">
-        <v>18.99715010764876</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="I85" t="n">
         <v>18.17186472076723</v>
       </c>
       <c r="J85" t="n">
-        <v>18.99715010764876</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="K85" t="n">
-        <v>1.167129786956179</v>
+        <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>4.541555858812715</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -4008,7 +4008,7 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E86" t="n">
-        <v>1.028947114944458</v>
+        <v>1.662111639976501</v>
       </c>
       <c r="F86" t="n">
         <v>100</v>
@@ -4017,19 +4017,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="H86" t="n">
-        <v>46.9015153346644</v>
+        <v>47.98367170235787</v>
       </c>
       <c r="I86" t="n">
         <v>44.28900565726017</v>
       </c>
       <c r="J86" t="n">
-        <v>46.9015153346644</v>
+        <v>47.98367170235787</v>
       </c>
       <c r="K86" t="n">
-        <v>3.694646617616021</v>
+        <v>5.22504682941654</v>
       </c>
       <c r="L86" t="n">
-        <v>5.898776995856905</v>
+        <v>8.342174294202174</v>
       </c>
     </row>
     <row r="87">
@@ -4050,7 +4050,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E87" t="n">
-        <v>1.012732028961182</v>
+        <v>1.638383030891418</v>
       </c>
       <c r="F87" t="n">
         <v>100</v>
@@ -4059,19 +4059,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H87" t="n">
-        <v>51.02159306921135</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="I87" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J87" t="n">
-        <v>51.02159306921135</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="K87" t="n">
-        <v>0.685852634757563</v>
+        <v>0</v>
       </c>
       <c r="L87" t="n">
-        <v>0.9596427888217801</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -4092,28 +4092,28 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E88" t="n">
-        <v>0.8426909446716309</v>
+        <v>1.357137560844421</v>
       </c>
       <c r="F88" t="n">
         <v>100</v>
       </c>
       <c r="G88" t="n">
-        <v>46.45331839264711</v>
+        <v>46.57504147811616</v>
       </c>
       <c r="H88" t="n">
-        <v>52.51952133235241</v>
+        <v>48.0445332450924</v>
       </c>
       <c r="I88" t="n">
-        <v>46.45331839264711</v>
+        <v>46.57504147811616</v>
       </c>
       <c r="J88" t="n">
-        <v>52.51952133235241</v>
+        <v>48.0445332450924</v>
       </c>
       <c r="K88" t="n">
-        <v>8.578906469438772</v>
+        <v>2.078175186653398</v>
       </c>
       <c r="L88" t="n">
-        <v>18.58365423415876</v>
+        <v>8.479593371084396</v>
       </c>
     </row>
     <row r="89">
@@ -4134,7 +4134,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E89" t="n">
-        <v>0.9006506204605103</v>
+        <v>1.488242030143738</v>
       </c>
       <c r="F89" t="n">
         <v>100</v>
@@ -4143,19 +4143,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H89" t="n">
-        <v>55.86938097677704</v>
+        <v>56.85213063165645</v>
       </c>
       <c r="I89" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J89" t="n">
-        <v>55.86938097677704</v>
+        <v>56.85213063165645</v>
       </c>
       <c r="K89" t="n">
-        <v>7.541660041145253</v>
+        <v>8.931477931493188</v>
       </c>
       <c r="L89" t="n">
-        <v>10.55226634332121</v>
+        <v>12.49689504146619</v>
       </c>
     </row>
     <row r="90">
@@ -4176,7 +4176,7 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E90" t="n">
-        <v>0.3734534978866577</v>
+        <v>0.6456115245819092</v>
       </c>
       <c r="F90" t="n">
         <v>100</v>
@@ -4185,19 +4185,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="H90" t="n">
-        <v>47.41281383876989</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="I90" t="n">
         <v>44.28900565726017</v>
       </c>
       <c r="J90" t="n">
-        <v>47.41281383876989</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="K90" t="n">
-        <v>4.417731896543086</v>
+        <v>0</v>
       </c>
       <c r="L90" t="n">
-        <v>7.053236204226334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -4218,7 +4218,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E91" t="n">
-        <v>0.3774353265762329</v>
+        <v>0.5772280693054199</v>
       </c>
       <c r="F91" t="n">
         <v>100</v>
@@ -4227,19 +4227,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H91" t="n">
-        <v>54.23962095425221</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="I91" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J91" t="n">
-        <v>54.23962095425221</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="K91" t="n">
-        <v>5.236831313877156</v>
+        <v>0</v>
       </c>
       <c r="L91" t="n">
-        <v>7.327357440880465</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -4260,7 +4260,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E92" t="n">
-        <v>1.111896634101868</v>
+        <v>1.838971018791199</v>
       </c>
       <c r="F92" t="n">
         <v>100</v>
@@ -4269,19 +4269,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H92" t="n">
-        <v>47.33481367365937</v>
+        <v>48.95973811067714</v>
       </c>
       <c r="I92" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J92" t="n">
-        <v>47.33481367365937</v>
+        <v>48.95973811067714</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>2.297990176661993</v>
       </c>
       <c r="L92" t="n">
-        <v>0</v>
+        <v>3.432831590339601</v>
       </c>
     </row>
     <row r="93">
@@ -4302,28 +4302,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E93" t="n">
-        <v>1.124535083770752</v>
+        <v>1.901353478431702</v>
       </c>
       <c r="F93" t="n">
         <v>100</v>
       </c>
       <c r="G93" t="n">
-        <v>54.33806753213224</v>
+        <v>54.92280061922531</v>
       </c>
       <c r="H93" t="n">
-        <v>54.69948596909365</v>
+        <v>59.81646145512598</v>
       </c>
       <c r="I93" t="n">
-        <v>54.33806753213224</v>
+        <v>54.92280061922531</v>
       </c>
       <c r="J93" t="n">
-        <v>54.69948596909365</v>
+        <v>59.81646145512598</v>
       </c>
       <c r="K93" t="n">
-        <v>0.5111228552425087</v>
+        <v>6.920681523784783</v>
       </c>
       <c r="L93" t="n">
-        <v>0.6651293529120942</v>
+        <v>10.08205512600195</v>
       </c>
     </row>
     <row r="94">
@@ -4344,28 +4344,28 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E94" t="n">
-        <v>0.960055947303772</v>
+        <v>1.531654596328735</v>
       </c>
       <c r="F94" t="n">
         <v>100</v>
       </c>
       <c r="G94" t="n">
-        <v>54.13302706816542</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="H94" t="n">
-        <v>62.90266902155723</v>
+        <v>48.3305958815295</v>
       </c>
       <c r="I94" t="n">
-        <v>54.13302706816542</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="J94" t="n">
-        <v>62.90266902155723</v>
+        <v>48.3305958815295</v>
       </c>
       <c r="K94" t="n">
-        <v>12.40214658764278</v>
+        <v>1.408248703539775</v>
       </c>
       <c r="L94" t="n">
-        <v>32.88880665133151</v>
+        <v>2.103699435124772</v>
       </c>
     </row>
     <row r="95">
@@ -4386,28 +4386,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E95" t="n">
-        <v>0.9824579954147339</v>
+        <v>1.608596444129944</v>
       </c>
       <c r="F95" t="n">
         <v>100</v>
       </c>
       <c r="G95" t="n">
-        <v>54.90718637611567</v>
+        <v>54.92280061922531</v>
       </c>
       <c r="H95" t="n">
-        <v>59.88551334854085</v>
+        <v>68.06193224743592</v>
       </c>
       <c r="I95" t="n">
-        <v>54.90718637611567</v>
+        <v>54.92280061922531</v>
       </c>
       <c r="J95" t="n">
-        <v>59.88551334854085</v>
+        <v>68.06193224743592</v>
       </c>
       <c r="K95" t="n">
-        <v>7.040417522331478</v>
+        <v>18.58153814642073</v>
       </c>
       <c r="L95" t="n">
-        <v>10.20913342773588</v>
+        <v>25.25644605816763</v>
       </c>
     </row>
     <row r="96">
@@ -4428,7 +4428,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E96" t="n">
-        <v>0.4079614877700806</v>
+        <v>0.4611960649490356</v>
       </c>
       <c r="F96" t="n">
         <v>100</v>
@@ -4437,19 +4437,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H96" t="n">
-        <v>47.33481367365937</v>
+        <v>48.4074548964992</v>
       </c>
       <c r="I96" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J96" t="n">
-        <v>47.33481367365937</v>
+        <v>48.4074548964992</v>
       </c>
       <c r="K96" t="n">
-        <v>0</v>
+        <v>1.516943764900555</v>
       </c>
       <c r="L96" t="n">
-        <v>0</v>
+        <v>2.266072557578762</v>
       </c>
     </row>
     <row r="97">
@@ -4470,7 +4470,7 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E97" t="n">
-        <v>0.5309340953826904</v>
+        <v>463.4214724302292</v>
       </c>
       <c r="F97" t="n">
         <v>100</v>
@@ -4479,19 +4479,19 @@
         <v>54.49178556207163</v>
       </c>
       <c r="H97" t="n">
-        <v>59.67781294151883</v>
+        <v>63.47180641430181</v>
       </c>
       <c r="I97" t="n">
         <v>54.49178556207163</v>
       </c>
       <c r="J97" t="n">
-        <v>59.67781294151883</v>
+        <v>63.47180641430181</v>
       </c>
       <c r="K97" t="n">
-        <v>7.334150254852436</v>
+        <v>12.69966727961712</v>
       </c>
       <c r="L97" t="n">
-        <v>9.826896045261428</v>
+        <v>16.80909774122613</v>
       </c>
     </row>
     <row r="98">
@@ -4512,28 +4512,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E98" t="n">
-        <v>1.297523498535156</v>
+        <v>1.799224019050598</v>
       </c>
       <c r="F98" t="n">
         <v>100</v>
       </c>
       <c r="G98" t="n">
-        <v>1.670599491755848</v>
+        <v>0.9562267675903433</v>
       </c>
       <c r="H98" t="n">
-        <v>1.915805479516752</v>
+        <v>1.13135621019566</v>
       </c>
       <c r="I98" t="n">
-        <v>1.670599491755848</v>
+        <v>0.9562267675903433</v>
       </c>
       <c r="J98" t="n">
-        <v>1.915805479516752</v>
+        <v>1.13135621019566</v>
       </c>
       <c r="K98" t="n">
-        <v>0.3467736334665617</v>
+        <v>0.2476704329032791</v>
       </c>
       <c r="L98" t="n">
-        <v>1783.763544846556</v>
+        <v>1012.434225597853</v>
       </c>
     </row>
     <row r="99">
@@ -4554,28 +4554,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E99" t="n">
-        <v>1.275575399398804</v>
+        <v>1.985014081001282</v>
       </c>
       <c r="F99" t="n">
         <v>100</v>
       </c>
       <c r="G99" t="n">
-        <v>17.44082658478748</v>
+        <v>21.6799181202689</v>
       </c>
       <c r="H99" t="n">
-        <v>19.56037235252819</v>
+        <v>21.6799181202689</v>
       </c>
       <c r="I99" t="n">
-        <v>17.44082658478748</v>
+        <v>21.6799181202689</v>
       </c>
       <c r="J99" t="n">
-        <v>19.56037235252819</v>
+        <v>21.6799181202689</v>
       </c>
       <c r="K99" t="n">
-        <v>2.997490370809405</v>
+        <v>0</v>
       </c>
       <c r="L99" t="n">
-        <v>85.49645607981628</v>
+        <v>105.5966986175847</v>
       </c>
     </row>
     <row r="100">
@@ -4596,28 +4596,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E100" t="n">
-        <v>1.121787071228027</v>
+        <v>1.890044331550598</v>
       </c>
       <c r="F100" t="n">
         <v>100</v>
       </c>
       <c r="G100" t="n">
-        <v>20.7698829230452</v>
+        <v>14.56709750416335</v>
       </c>
       <c r="H100" t="n">
-        <v>22.43503327195231</v>
+        <v>20.82219388489576</v>
       </c>
       <c r="I100" t="n">
-        <v>20.7698829230452</v>
+        <v>14.56709750416335</v>
       </c>
       <c r="J100" t="n">
-        <v>22.43503327195231</v>
+        <v>20.82219388489576</v>
       </c>
       <c r="K100" t="n">
-        <v>2.354878206814734</v>
+        <v>8.846042135582641</v>
       </c>
       <c r="L100" t="n">
-        <v>21959.8063096592</v>
+        <v>20373.94173545611</v>
       </c>
     </row>
     <row r="101">
@@ -4638,28 +4638,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E101" t="n">
-        <v>1.19335401058197</v>
+        <v>1.848074913024902</v>
       </c>
       <c r="F101" t="n">
         <v>100</v>
       </c>
       <c r="G101" t="n">
-        <v>25.7972134058523</v>
+        <v>32.10475003054074</v>
       </c>
       <c r="H101" t="n">
-        <v>27.44191846171116</v>
+        <v>39.27796340232866</v>
       </c>
       <c r="I101" t="n">
-        <v>25.7972134058523</v>
+        <v>32.10475003054074</v>
       </c>
       <c r="J101" t="n">
-        <v>27.44191846171116</v>
+        <v>39.27796340232866</v>
       </c>
       <c r="K101" t="n">
-        <v>2.325964196099202</v>
+        <v>10.14445563617852</v>
       </c>
       <c r="L101" t="n">
-        <v>160.2393518352819</v>
+        <v>272.4838608311554</v>
       </c>
     </row>
     <row r="102">
@@ -4680,28 +4680,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E102" t="n">
-        <v>0.4553465843200684</v>
+        <v>0.7278029918670654</v>
       </c>
       <c r="F102" t="n">
         <v>100</v>
       </c>
       <c r="G102" t="n">
-        <v>0.9562267675903433</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="H102" t="n">
-        <v>6.640129470788645</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="I102" t="n">
-        <v>0.9562267675903433</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="J102" t="n">
-        <v>6.640129470788645</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="K102" t="n">
-        <v>8.038252290072135</v>
+        <v>0</v>
       </c>
       <c r="L102" t="n">
-        <v>6429.073000296497</v>
+        <v>1184.634620228945</v>
       </c>
     </row>
     <row r="103">
@@ -4722,28 +4722,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E103" t="n">
-        <v>0.4546098709106445</v>
+        <v>0.7243975400924683</v>
       </c>
       <c r="F103" t="n">
         <v>100</v>
       </c>
       <c r="G103" t="n">
-        <v>31.13769920038724</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="H103" t="n">
-        <v>37.83942582411279</v>
+        <v>13.39502578097015</v>
       </c>
       <c r="I103" t="n">
-        <v>31.13769920038724</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="J103" t="n">
-        <v>37.83942582411279</v>
+        <v>13.39502578097015</v>
       </c>
       <c r="K103" t="n">
-        <v>9.477672682589516</v>
+        <v>4.03071965583747</v>
       </c>
       <c r="L103" t="n">
-        <v>258.8418085282913</v>
+        <v>27.02875828161745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run #1 is completed
</commit_message>
<xml_diff>
--- a/results/graphs/benchmark_results.xlsx
+++ b/results/graphs/benchmark_results.xlsx
@@ -496,7 +496,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E2" t="n">
-        <v>0.07430966695149739</v>
+        <v>0.07327836990356446</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -538,7 +538,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E3" t="n">
-        <v>0.07017064094543457</v>
+        <v>0.06886888027191163</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -580,7 +580,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E4" t="n">
-        <v>0.03350504239400228</v>
+        <v>0.03294903993606568</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -622,7 +622,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03396288553873698</v>
+        <v>0.03346406936645508</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -664,7 +664,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E6" t="n">
-        <v>0.004328012466430664</v>
+        <v>0.002898759841918945</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -706,7 +706,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03433068593343099</v>
+        <v>0.03336961030960083</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -748,7 +748,7 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E8" t="n">
-        <v>1.024234056472778</v>
+        <v>1.022696838378906</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -757,19 +757,19 @@
         <v>12.04748748354309</v>
       </c>
       <c r="H8" t="n">
-        <v>13.0441713096798</v>
+        <v>13.40560809486521</v>
       </c>
       <c r="I8" t="n">
         <v>12.04748748354309</v>
       </c>
       <c r="J8" t="n">
-        <v>13.0441713096798</v>
+        <v>13.40560809486521</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8631535129754595</v>
+        <v>3.899462568235728</v>
       </c>
       <c r="L8" t="n">
-        <v>8.272960046633624</v>
+        <v>11.27306098617918</v>
       </c>
     </row>
     <row r="9">
@@ -790,7 +790,7 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9481183687845866</v>
+        <v>0.9244257020950317</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -799,19 +799,19 @@
         <v>53.31120138136255</v>
       </c>
       <c r="H9" t="n">
-        <v>64.94039716970791</v>
+        <v>66.44696065207982</v>
       </c>
       <c r="I9" t="n">
         <v>53.31120138136255</v>
       </c>
       <c r="J9" t="n">
-        <v>64.94039716970791</v>
+        <v>66.44696065207982</v>
       </c>
       <c r="K9" t="n">
-        <v>10.07312384576613</v>
+        <v>12.49186075768247</v>
       </c>
       <c r="L9" t="n">
-        <v>21.81379426277737</v>
+        <v>24.63977350041392</v>
       </c>
     </row>
     <row r="10">
@@ -832,28 +832,28 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7914830048878988</v>
+        <v>0.8140435528755188</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>20.03822060102891</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="H10" t="n">
-        <v>31.46852928911991</v>
+        <v>27.44428813559835</v>
       </c>
       <c r="I10" t="n">
-        <v>20.03822060102891</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="J10" t="n">
-        <v>31.46852928911991</v>
+        <v>27.44428813559835</v>
       </c>
       <c r="K10" t="n">
-        <v>11.18487885379429</v>
+        <v>13.91566858124934</v>
       </c>
       <c r="L10" t="n">
-        <v>161.2040836905291</v>
+        <v>127.8009267333736</v>
       </c>
     </row>
     <row r="11">
@@ -874,28 +874,28 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7033139864603678</v>
+        <v>0.7755626630783081</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>71.92554264065875</v>
+        <v>53.31120138136255</v>
       </c>
       <c r="H11" t="n">
-        <v>83.22512923974998</v>
+        <v>85.11152571728677</v>
       </c>
       <c r="I11" t="n">
-        <v>71.92554264065875</v>
+        <v>53.31120138136255</v>
       </c>
       <c r="J11" t="n">
-        <v>83.22512923974998</v>
+        <v>85.11152571728677</v>
       </c>
       <c r="K11" t="n">
-        <v>11.06172742990691</v>
+        <v>16.96516412925579</v>
       </c>
       <c r="L11" t="n">
-        <v>56.11189971953109</v>
+        <v>59.6503614848971</v>
       </c>
     </row>
     <row r="12">
@@ -916,7 +916,7 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E12" t="n">
-        <v>0.02570700645446777</v>
+        <v>0.02709391832351685</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
@@ -925,19 +925,19 @@
         <v>12.04748748354309</v>
       </c>
       <c r="H12" t="n">
-        <v>12.04748748354309</v>
+        <v>12.63358626965861</v>
       </c>
       <c r="I12" t="n">
         <v>12.04748748354309</v>
       </c>
       <c r="J12" t="n">
-        <v>12.04748748354309</v>
+        <v>12.63358626965861</v>
       </c>
       <c r="K12" t="n">
-        <v>2.175583928816829e-15</v>
+        <v>0.7945323924873762</v>
       </c>
       <c r="L12" t="n">
-        <v>-1.474462490064223e-14</v>
+        <v>4.864904710763374</v>
       </c>
     </row>
     <row r="13">
@@ -958,21 +958,29 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2778979937235515</v>
+        <v>0.2895361709594726</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>53.31120138136255</v>
+      </c>
+      <c r="H13" t="n">
+        <v>57.9647866961866</v>
+      </c>
       <c r="I13" t="n">
-        <v>41.21340348171624</v>
+        <v>20.87387904273287</v>
       </c>
       <c r="J13" t="n">
-        <v>60.32502810573148</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+        <v>57.37777681846475</v>
+      </c>
+      <c r="K13" t="n">
+        <v>9.307170629648098</v>
+      </c>
+      <c r="L13" t="n">
+        <v>8.729094813554379</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -992,7 +1000,7 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E14" t="n">
-        <v>1.127868334452311</v>
+        <v>1.133707711696625</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1001,19 +1009,19 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="H14" t="n">
-        <v>-3.68658624814832</v>
+        <v>-6.172254514210448</v>
       </c>
       <c r="I14" t="n">
         <v>-11.80593354076133</v>
       </c>
       <c r="J14" t="n">
-        <v>-3.68658624814832</v>
+        <v>-6.172254514210448</v>
       </c>
       <c r="K14" t="n">
-        <v>7.7904962918705</v>
+        <v>6.396806894390321</v>
       </c>
       <c r="L14" t="n">
-        <v>68.77344569643765</v>
+        <v>47.71904743576578</v>
       </c>
     </row>
     <row r="15">
@@ -1034,7 +1042,7 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E15" t="n">
-        <v>1.121533950169881</v>
+        <v>1.152146470546722</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1043,19 +1051,19 @@
         <v>13.7263575295875</v>
       </c>
       <c r="H15" t="n">
-        <v>24.14436939150308</v>
+        <v>28.34275111753655</v>
       </c>
       <c r="I15" t="n">
         <v>13.7263575295875</v>
       </c>
       <c r="J15" t="n">
-        <v>24.14436939150308</v>
+        <v>28.34275111753655</v>
       </c>
       <c r="K15" t="n">
-        <v>15.8473976684254</v>
+        <v>15.51730206809427</v>
       </c>
       <c r="L15" t="n">
-        <v>75.89786175581756</v>
+        <v>106.4841386831361</v>
       </c>
     </row>
     <row r="16">
@@ -1076,28 +1084,28 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E16" t="n">
-        <v>0.856292724609375</v>
+        <v>0.8907021689414978</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>-2.980862829573491</v>
+        <v>-11.80593354076133</v>
       </c>
       <c r="H16" t="n">
-        <v>10.22793880662019</v>
+        <v>21.96448947943182</v>
       </c>
       <c r="I16" t="n">
-        <v>-2.980862829573491</v>
+        <v>-11.80593354076133</v>
       </c>
       <c r="J16" t="n">
-        <v>10.22793880662019</v>
+        <v>21.96448947943182</v>
       </c>
       <c r="K16" t="n">
-        <v>12.54703248658785</v>
+        <v>18.06001986135499</v>
       </c>
       <c r="L16" t="n">
-        <v>186.6338843201773</v>
+        <v>286.0461894317541</v>
       </c>
     </row>
     <row r="17">
@@ -1118,28 +1126,28 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9117163022359213</v>
+        <v>0.9103633213043213</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>13.7263575295875</v>
+        <v>16.32499152035578</v>
       </c>
       <c r="H17" t="n">
-        <v>41.3286437616449</v>
+        <v>63.1528352743077</v>
       </c>
       <c r="I17" t="n">
-        <v>13.7263575295875</v>
+        <v>16.32499152035578</v>
       </c>
       <c r="J17" t="n">
-        <v>41.3286437616449</v>
+        <v>63.1528352743077</v>
       </c>
       <c r="K17" t="n">
-        <v>28.34769076076994</v>
+        <v>25.08369718326212</v>
       </c>
       <c r="L17" t="n">
-        <v>201.0896639735632</v>
+        <v>360.0844407424198</v>
       </c>
     </row>
     <row r="18">
@@ -1160,7 +1168,7 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E18" t="n">
-        <v>0.02763001124064128</v>
+        <v>0.02866180181503296</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1169,19 +1177,19 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="H18" t="n">
-        <v>-7.155137093216222</v>
+        <v>-8.416822271419015</v>
       </c>
       <c r="I18" t="n">
         <v>-11.80593354076133</v>
       </c>
       <c r="J18" t="n">
-        <v>-7.155137093216222</v>
+        <v>-8.416822271419015</v>
       </c>
       <c r="K18" t="n">
-        <v>4.203976542484646</v>
+        <v>4.084944442451147</v>
       </c>
       <c r="L18" t="n">
-        <v>39.39372038210874</v>
+        <v>28.70684692270224</v>
       </c>
     </row>
     <row r="19">
@@ -1202,28 +1210,28 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3275400002797444</v>
+        <v>0.3432621693611145</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="G19" t="n">
         <v>13.7263575295875</v>
       </c>
       <c r="H19" t="n">
-        <v>22.11782312175674</v>
+        <v>19.73167474435576</v>
       </c>
       <c r="I19" t="n">
         <v>13.7263575295875</v>
       </c>
       <c r="J19" t="n">
-        <v>22.11782312175674</v>
+        <v>27.85952743029948</v>
       </c>
       <c r="K19" t="n">
-        <v>12.35248719129619</v>
+        <v>5.777742686055614</v>
       </c>
       <c r="L19" t="n">
-        <v>61.13395760004957</v>
+        <v>43.75026077984378</v>
       </c>
     </row>
     <row r="20">
@@ -1244,28 +1252,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E20" t="n">
-        <v>1.307725667953491</v>
+        <v>1.330196940898895</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>-3.758716405667779</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="H20" t="n">
-        <v>0.8523860383297818</v>
+        <v>-0.456530469289016</v>
       </c>
       <c r="I20" t="n">
-        <v>-3.758716405667779</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="J20" t="n">
-        <v>0.8523860383297818</v>
+        <v>-0.456530469289016</v>
       </c>
       <c r="K20" t="n">
-        <v>4.285706219569787</v>
+        <v>7.725375342212417</v>
       </c>
       <c r="L20" t="n">
-        <v>109.0074039506273</v>
+        <v>95.17571362300437</v>
       </c>
     </row>
     <row r="21">
@@ -1286,28 +1294,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E21" t="n">
-        <v>1.228333314259847</v>
+        <v>1.250355911254883</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>18.7915703518064</v>
+        <v>15.06947538019221</v>
       </c>
       <c r="H21" t="n">
-        <v>31.01629489452317</v>
+        <v>33.32049410991213</v>
       </c>
       <c r="I21" t="n">
-        <v>18.7915703518064</v>
+        <v>15.06947538019221</v>
       </c>
       <c r="J21" t="n">
-        <v>31.01629489452317</v>
+        <v>33.32049410991213</v>
       </c>
       <c r="K21" t="n">
-        <v>10.7796405649257</v>
+        <v>15.2564804117167</v>
       </c>
       <c r="L21" t="n">
-        <v>105.8219952055661</v>
+        <v>121.1125023881697</v>
       </c>
     </row>
     <row r="22">
@@ -1328,28 +1336,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E22" t="n">
-        <v>1.041307051976522</v>
+        <v>1.025094621181488</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>30.95966696656225</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="H22" t="n">
-        <v>45.95598914311021</v>
+        <v>27.74100451441571</v>
       </c>
       <c r="I22" t="n">
-        <v>30.95966696656225</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="J22" t="n">
-        <v>45.95598914311021</v>
+        <v>27.74100451441571</v>
       </c>
       <c r="K22" t="n">
-        <v>14.62716201729563</v>
+        <v>18.16527609628692</v>
       </c>
       <c r="L22" t="n">
-        <v>585.6299136172461</v>
+        <v>393.1470277799702</v>
       </c>
     </row>
     <row r="23">
@@ -1370,28 +1378,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E23" t="n">
-        <v>0.9655170440673828</v>
+        <v>0.9708001184463501</v>
       </c>
       <c r="F23" t="n">
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>54.78201407506988</v>
+        <v>18.7915703518064</v>
       </c>
       <c r="H23" t="n">
-        <v>78.97117932923648</v>
+        <v>66.36045503319389</v>
       </c>
       <c r="I23" t="n">
-        <v>54.78201407506988</v>
+        <v>18.7915703518064</v>
       </c>
       <c r="J23" t="n">
-        <v>78.97117932923648</v>
+        <v>66.36045503319389</v>
       </c>
       <c r="K23" t="n">
-        <v>20.95786878323072</v>
+        <v>23.4849287479963</v>
       </c>
       <c r="L23" t="n">
-        <v>424.0473031532252</v>
+        <v>340.3634058848536</v>
       </c>
     </row>
     <row r="24">
@@ -1412,7 +1420,7 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E24" t="n">
-        <v>0.03166627883911133</v>
+        <v>0.03124053239822388</v>
       </c>
       <c r="F24" t="n">
         <v>100</v>
@@ -1421,19 +1429,19 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="H24" t="n">
-        <v>-6.858362900101219</v>
+        <v>-8.353630098055669</v>
       </c>
       <c r="I24" t="n">
         <v>-9.463170998014522</v>
       </c>
       <c r="J24" t="n">
-        <v>-6.858362900101219</v>
+        <v>-8.353630098055669</v>
       </c>
       <c r="K24" t="n">
-        <v>3.63647761841765</v>
+        <v>1.612896428302111</v>
       </c>
       <c r="L24" t="n">
-        <v>27.5257426761053</v>
+        <v>11.72483198487745</v>
       </c>
     </row>
     <row r="25">
@@ -1454,28 +1462,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3716853459676107</v>
+        <v>0.3714484190940857</v>
       </c>
       <c r="F25" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G25" t="n">
         <v>15.06947538019221</v>
       </c>
       <c r="H25" t="n">
-        <v>15.06947538019221</v>
+        <v>16.31256556421084</v>
       </c>
       <c r="I25" t="n">
         <v>15.06947538019221</v>
       </c>
       <c r="J25" t="n">
-        <v>15.06947538019221</v>
+        <v>17.29528846306434</v>
       </c>
       <c r="K25" t="n">
-        <v>2.175583928816829e-15</v>
+        <v>7.111149238948735</v>
       </c>
       <c r="L25" t="n">
-        <v>1.178778155565488e-14</v>
+        <v>8.249060784508734</v>
       </c>
     </row>
     <row r="26">
@@ -1496,7 +1504,7 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E26" t="n">
-        <v>1.327058394749959</v>
+        <v>1.342541608810425</v>
       </c>
       <c r="F26" t="n">
         <v>100</v>
@@ -1505,19 +1513,19 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="H26" t="n">
-        <v>-11.32473258383299</v>
+        <v>-9.118726815776981</v>
       </c>
       <c r="I26" t="n">
         <v>-21.96317396534843</v>
       </c>
       <c r="J26" t="n">
-        <v>-11.32473258383299</v>
+        <v>-9.118726815776981</v>
       </c>
       <c r="K26" t="n">
-        <v>11.38574060821172</v>
+        <v>10.09968384419952</v>
       </c>
       <c r="L26" t="n">
-        <v>48.43763200300577</v>
+        <v>58.48174389474077</v>
       </c>
     </row>
     <row r="27">
@@ -1538,28 +1546,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E27" t="n">
-        <v>1.340184370676677</v>
+        <v>1.280003888607025</v>
       </c>
       <c r="F27" t="n">
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>44.17887864393854</v>
+        <v>22.8444824168921</v>
       </c>
       <c r="H27" t="n">
-        <v>47.69973910434526</v>
+        <v>45.21017643725565</v>
       </c>
       <c r="I27" t="n">
-        <v>44.17887864393854</v>
+        <v>22.8444824168921</v>
       </c>
       <c r="J27" t="n">
-        <v>47.69973910434526</v>
+        <v>45.21017643725565</v>
       </c>
       <c r="K27" t="n">
-        <v>4.97494903619352</v>
+        <v>14.38390154180655</v>
       </c>
       <c r="L27" t="n">
-        <v>108.8020128180896</v>
+        <v>97.90413988029553</v>
       </c>
     </row>
     <row r="28">
@@ -1580,28 +1588,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E28" t="n">
-        <v>1.055155595143636</v>
+        <v>1.061874940395355</v>
       </c>
       <c r="F28" t="n">
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6842386946915235</v>
+        <v>-15.10741470745636</v>
       </c>
       <c r="H28" t="n">
-        <v>8.93572435724408</v>
+        <v>17.13999463659888</v>
       </c>
       <c r="I28" t="n">
-        <v>0.6842386946915235</v>
+        <v>-15.10741470745636</v>
       </c>
       <c r="J28" t="n">
-        <v>8.93572435724408</v>
+        <v>17.13999463659888</v>
       </c>
       <c r="K28" t="n">
-        <v>13.49914906424047</v>
+        <v>15.53470091067555</v>
       </c>
       <c r="L28" t="n">
-        <v>140.6850320055839</v>
+        <v>178.0396980128686</v>
       </c>
     </row>
     <row r="29">
@@ -1622,28 +1630,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E29" t="n">
-        <v>1.06733759244283</v>
+        <v>1.003616440296173</v>
       </c>
       <c r="F29" t="n">
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>27.83410683042805</v>
+        <v>30.82283888334696</v>
       </c>
       <c r="H29" t="n">
-        <v>67.45045524019105</v>
+        <v>72.88043326639564</v>
       </c>
       <c r="I29" t="n">
-        <v>27.83410683042805</v>
+        <v>30.82283888334696</v>
       </c>
       <c r="J29" t="n">
-        <v>67.45045524019105</v>
+        <v>72.88043326639564</v>
       </c>
       <c r="K29" t="n">
-        <v>34.34048737122436</v>
+        <v>24.97590585459614</v>
       </c>
       <c r="L29" t="n">
-        <v>195.2592840987965</v>
+        <v>219.02860365313</v>
       </c>
     </row>
     <row r="30">
@@ -1664,7 +1672,7 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E30" t="n">
-        <v>0.03626267115275065</v>
+        <v>0.03269515991210938</v>
       </c>
       <c r="F30" t="n">
         <v>100</v>
@@ -1673,19 +1681,19 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="H30" t="n">
-        <v>-19.7218609727848</v>
+        <v>-15.31961985730699</v>
       </c>
       <c r="I30" t="n">
         <v>-21.96317396534843</v>
       </c>
       <c r="J30" t="n">
-        <v>-19.7218609727848</v>
+        <v>-15.31961985730699</v>
       </c>
       <c r="K30" t="n">
-        <v>3.424860032465515</v>
+        <v>6.008245035560368</v>
       </c>
       <c r="L30" t="n">
-        <v>10.20486836784053</v>
+        <v>30.24860668372914</v>
       </c>
     </row>
     <row r="31">
@@ -1706,28 +1714,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E31" t="n">
-        <v>0.3648656209309896</v>
+        <v>0.3541808414459229</v>
       </c>
       <c r="F31" t="n">
-        <v>33.33333333333333</v>
+        <v>19</v>
       </c>
       <c r="G31" t="n">
-        <v>33.24561934539526</v>
+        <v>22.8444824168921</v>
       </c>
       <c r="H31" t="n">
-        <v>33.24561934539526</v>
+        <v>53.89122178801244</v>
       </c>
       <c r="I31" t="n">
-        <v>2.155613386802565</v>
+        <v>0.6757756268044144</v>
       </c>
       <c r="J31" t="n">
-        <v>13.96528906430626</v>
+        <v>45.11412415595805</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>21.27213375768284</v>
       </c>
       <c r="L31" t="n">
-        <v>45.53019297479096</v>
+        <v>135.9047616161493</v>
       </c>
     </row>
     <row r="32">
@@ -1748,28 +1756,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E32" t="n">
-        <v>1.596434990564982</v>
+        <v>1.613664419651031</v>
       </c>
       <c r="F32" t="n">
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>-3.772978658646409</v>
+        <v>-8.841290064295642</v>
       </c>
       <c r="H32" t="n">
-        <v>3.610944455278955</v>
+        <v>-1.611070971345694</v>
       </c>
       <c r="I32" t="n">
-        <v>-3.772978658646409</v>
+        <v>-8.841290064295642</v>
       </c>
       <c r="J32" t="n">
-        <v>3.610944455278955</v>
+        <v>-1.611070971345694</v>
       </c>
       <c r="K32" t="n">
-        <v>7.085332633945435</v>
+        <v>6.136021695447403</v>
       </c>
       <c r="L32" t="n">
-        <v>140.8418277086199</v>
+        <v>81.77787449987885</v>
       </c>
     </row>
     <row r="33">
@@ -1790,28 +1798,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E33" t="n">
-        <v>1.536899884541829</v>
+        <v>1.550020151138306</v>
       </c>
       <c r="F33" t="n">
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9171894075994231</v>
+        <v>-1.050704163143443</v>
       </c>
       <c r="H33" t="n">
-        <v>19.80218194676768</v>
+        <v>15.08362749843662</v>
       </c>
       <c r="I33" t="n">
-        <v>0.9171894075994231</v>
+        <v>-1.050704163143443</v>
       </c>
       <c r="J33" t="n">
-        <v>19.80218194676768</v>
+        <v>15.08362749843662</v>
       </c>
       <c r="K33" t="n">
-        <v>26.69484386102026</v>
+        <v>18.33548610329463</v>
       </c>
       <c r="L33" t="n">
-        <v>1984.658178903995</v>
+        <v>1535.57321152228</v>
       </c>
     </row>
     <row r="34">
@@ -1832,28 +1840,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E34" t="n">
-        <v>1.259856303532918</v>
+        <v>1.269640986919403</v>
       </c>
       <c r="F34" t="n">
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>12.07452446100671</v>
+        <v>-3.837456178543082</v>
       </c>
       <c r="H34" t="n">
-        <v>34.42636906030773</v>
+        <v>34.13584369839266</v>
       </c>
       <c r="I34" t="n">
-        <v>12.07452446100671</v>
+        <v>-3.837456178543082</v>
       </c>
       <c r="J34" t="n">
-        <v>34.42636906030773</v>
+        <v>34.13584369839266</v>
       </c>
       <c r="K34" t="n">
-        <v>21.59264976724075</v>
+        <v>19.94698979012258</v>
       </c>
       <c r="L34" t="n">
-        <v>489.3817396550983</v>
+        <v>486.095733203525</v>
       </c>
     </row>
     <row r="35">
@@ -1874,28 +1882,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E35" t="n">
-        <v>1.473158677419027</v>
+        <v>1.231335241794586</v>
       </c>
       <c r="F35" t="n">
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>86.60704220496189</v>
+        <v>-1.050704163143443</v>
       </c>
       <c r="H35" t="n">
-        <v>111.2004373910859</v>
+        <v>88.78119756767873</v>
       </c>
       <c r="I35" t="n">
-        <v>86.60704220496189</v>
+        <v>-1.050704163143443</v>
       </c>
       <c r="J35" t="n">
-        <v>111.2004373910859</v>
+        <v>88.78119756767873</v>
       </c>
       <c r="K35" t="n">
-        <v>41.09046363109742</v>
+        <v>39.1386972966944</v>
       </c>
       <c r="L35" t="n">
-        <v>10683.4202710687</v>
+        <v>8549.685523474815</v>
       </c>
     </row>
     <row r="36">
@@ -1916,28 +1924,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E36" t="n">
-        <v>0.03784370422363281</v>
+        <v>0.03667536973953247</v>
       </c>
       <c r="F36" t="n">
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>-4.653648487147549</v>
+        <v>-8.841290064295642</v>
       </c>
       <c r="H36" t="n">
-        <v>-0.9022275301783157</v>
+        <v>-1.022760056095839</v>
       </c>
       <c r="I36" t="n">
-        <v>-4.653648487147549</v>
+        <v>-8.841290064295642</v>
       </c>
       <c r="J36" t="n">
-        <v>-0.9022275301783157</v>
+        <v>-1.022760056095839</v>
       </c>
       <c r="K36" t="n">
-        <v>4.575881415531583</v>
+        <v>4.913939678384262</v>
       </c>
       <c r="L36" t="n">
-        <v>89.79529544198715</v>
+        <v>88.43200428152315</v>
       </c>
     </row>
     <row r="37">
@@ -1958,28 +1966,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4413469632466634</v>
+        <v>0.4356991195678711</v>
       </c>
       <c r="F37" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G37" t="n">
         <v>-1.050704163143443</v>
       </c>
       <c r="H37" t="n">
-        <v>0.2612248840184677</v>
+        <v>2.861817055460585</v>
       </c>
       <c r="I37" t="n">
-        <v>-1.050704163143443</v>
+        <v>-1.36824095017819</v>
       </c>
       <c r="J37" t="n">
-        <v>0.2612248840184677</v>
+        <v>8.68130175862124</v>
       </c>
       <c r="K37" t="n">
-        <v>1.136163882804928</v>
+        <v>3.26537734354274</v>
       </c>
       <c r="L37" t="n">
-        <v>124.8618872163739</v>
+        <v>372.3713444609134</v>
       </c>
     </row>
     <row r="38">
@@ -2000,7 +2008,7 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E38" t="n">
-        <v>1.603271007537842</v>
+        <v>1.5245334815979</v>
       </c>
       <c r="F38" t="n">
         <v>100</v>
@@ -2009,19 +2017,19 @@
         <v>9.383712874145662</v>
       </c>
       <c r="H38" t="n">
-        <v>18.04803245561795</v>
+        <v>19.87705880305042</v>
       </c>
       <c r="I38" t="n">
         <v>9.383712874145662</v>
       </c>
       <c r="J38" t="n">
-        <v>18.04803245561795</v>
+        <v>19.87705880305042</v>
       </c>
       <c r="K38" t="n">
-        <v>15.00704172812391</v>
+        <v>7.825259169072486</v>
       </c>
       <c r="L38" t="n">
-        <v>92.3335964950987</v>
+        <v>111.8250959896311</v>
       </c>
     </row>
     <row r="39">
@@ -2042,28 +2050,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E39" t="n">
-        <v>1.535286664962769</v>
+        <v>1.503237800598145</v>
       </c>
       <c r="F39" t="n">
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>37.75126003353604</v>
+        <v>26.21619167672251</v>
       </c>
       <c r="H39" t="n">
-        <v>50.75177968042362</v>
+        <v>45.3451481890507</v>
       </c>
       <c r="I39" t="n">
-        <v>37.75126003353604</v>
+        <v>26.21619167672251</v>
       </c>
       <c r="J39" t="n">
-        <v>50.75177968042362</v>
+        <v>45.3451481890507</v>
       </c>
       <c r="K39" t="n">
-        <v>11.25880134656047</v>
+        <v>10.07553664884598</v>
       </c>
       <c r="L39" t="n">
-        <v>93.58944390647854</v>
+        <v>72.96619107844286</v>
       </c>
     </row>
     <row r="40">
@@ -2084,28 +2092,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E40" t="n">
-        <v>1.223964055379232</v>
+        <v>1.212036910057068</v>
       </c>
       <c r="F40" t="n">
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>27.30475740433501</v>
+        <v>9.383712874145662</v>
       </c>
       <c r="H40" t="n">
-        <v>52.30775322753728</v>
+        <v>53.38852342948877</v>
       </c>
       <c r="I40" t="n">
-        <v>27.30475740433501</v>
+        <v>9.383712874145662</v>
       </c>
       <c r="J40" t="n">
-        <v>52.30775322753728</v>
+        <v>53.38852342948877</v>
       </c>
       <c r="K40" t="n">
-        <v>28.45744295857543</v>
+        <v>19.27559423170784</v>
       </c>
       <c r="L40" t="n">
-        <v>457.4313060202157</v>
+        <v>468.9488174407672</v>
       </c>
     </row>
     <row r="41">
@@ -2126,28 +2134,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E41" t="n">
-        <v>1.173933982849121</v>
+        <v>1.191228010654449</v>
       </c>
       <c r="F41" t="n">
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>34.50647568089784</v>
+        <v>37.10625335047498</v>
       </c>
       <c r="H41" t="n">
-        <v>52.21903460183123</v>
+        <v>71.94891164281708</v>
       </c>
       <c r="I41" t="n">
-        <v>34.50647568089784</v>
+        <v>37.10625335047498</v>
       </c>
       <c r="J41" t="n">
-        <v>52.21903460183123</v>
+        <v>71.94891164281708</v>
       </c>
       <c r="K41" t="n">
-        <v>16.71962479205288</v>
+        <v>18.98205376187818</v>
       </c>
       <c r="L41" t="n">
-        <v>99.18619472177865</v>
+        <v>174.4445590344874</v>
       </c>
     </row>
     <row r="42">
@@ -2168,28 +2176,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E42" t="n">
-        <v>0.03711732228597005</v>
+        <v>0.0367170786857605</v>
       </c>
       <c r="F42" t="n">
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>13.34718289413153</v>
+        <v>9.383712874145662</v>
       </c>
       <c r="H42" t="n">
-        <v>18.99742599107499</v>
+        <v>21.73273904659161</v>
       </c>
       <c r="I42" t="n">
-        <v>13.34718289413153</v>
+        <v>9.383712874145662</v>
       </c>
       <c r="J42" t="n">
-        <v>18.99742599107499</v>
+        <v>21.73273904659161</v>
       </c>
       <c r="K42" t="n">
-        <v>4.963841419479261</v>
+        <v>7.211201687054464</v>
       </c>
       <c r="L42" t="n">
-        <v>102.4510579753284</v>
+        <v>131.600639726205</v>
       </c>
     </row>
     <row r="43">
@@ -2210,28 +2218,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E43" t="n">
-        <v>0.4381202856699626</v>
+        <v>0.440082221031189</v>
       </c>
       <c r="F43" t="n">
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>30.23324412992315</v>
+        <v>26.21619167672251</v>
       </c>
       <c r="H43" t="n">
-        <v>34.6670786307083</v>
+        <v>33.37910592943111</v>
       </c>
       <c r="I43" t="n">
-        <v>30.23324412992315</v>
+        <v>26.21619167672251</v>
       </c>
       <c r="J43" t="n">
-        <v>34.6670786307083</v>
+        <v>33.37910592943111</v>
       </c>
       <c r="K43" t="n">
-        <v>4.037515475057447</v>
+        <v>4.433854171687641</v>
       </c>
       <c r="L43" t="n">
-        <v>32.23537216311009</v>
+        <v>27.32248200286306</v>
       </c>
     </row>
     <row r="44">
@@ -2252,7 +2260,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1535646915435791</v>
+        <v>0.1525745296478271</v>
       </c>
       <c r="F44" t="n">
         <v>100</v>
@@ -2270,7 +2278,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
@@ -2294,7 +2302,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1593592961629232</v>
+        <v>0.1590132713317871</v>
       </c>
       <c r="F45" t="n">
         <v>100</v>
@@ -2336,7 +2344,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1002607345581055</v>
+        <v>0.1001806473731995</v>
       </c>
       <c r="F46" t="n">
         <v>100</v>
@@ -2354,7 +2362,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2378,7 +2386,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1076070467631022</v>
+        <v>0.1049100112915039</v>
       </c>
       <c r="F47" t="n">
         <v>100</v>
@@ -2420,7 +2428,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E48" t="n">
-        <v>0.005750338236490886</v>
+        <v>0.005615382194519043</v>
       </c>
       <c r="F48" t="n">
         <v>100</v>
@@ -2438,7 +2446,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2462,7 +2470,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E49" t="n">
-        <v>0.06528528531392415</v>
+        <v>0.0654410195350647</v>
       </c>
       <c r="F49" t="n">
         <v>100</v>
@@ -2504,28 +2512,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E50" t="n">
-        <v>2.748978058497111</v>
+        <v>2.709939367771149</v>
       </c>
       <c r="F50" t="n">
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>16.21740924951783</v>
+        <v>13.02451543344857</v>
       </c>
       <c r="H50" t="n">
-        <v>30.67278476804103</v>
+        <v>39.04521578619128</v>
       </c>
       <c r="I50" t="n">
-        <v>16.21740924951783</v>
+        <v>13.02451543344857</v>
       </c>
       <c r="J50" t="n">
-        <v>30.67278476804103</v>
+        <v>39.04521578619128</v>
       </c>
       <c r="K50" t="n">
-        <v>17.57058234329859</v>
+        <v>13.16898458889659</v>
       </c>
       <c r="L50" t="n">
-        <v>135.5003909724696</v>
+        <v>199.7824831618559</v>
       </c>
     </row>
     <row r="51">
@@ -2546,28 +2554,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E51" t="n">
-        <v>2.64211901028951</v>
+        <v>2.690952260494232</v>
       </c>
       <c r="F51" t="n">
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>67.3989560678863</v>
+        <v>34.00523196803706</v>
       </c>
       <c r="H51" t="n">
-        <v>74.67647485726845</v>
+        <v>69.58762460982115</v>
       </c>
       <c r="I51" t="n">
-        <v>67.3989560678863</v>
+        <v>34.00523196803706</v>
       </c>
       <c r="J51" t="n">
-        <v>74.67647485726845</v>
+        <v>69.58762460982115</v>
       </c>
       <c r="K51" t="n">
-        <v>6.401332140338771</v>
+        <v>22.08933507509494</v>
       </c>
       <c r="L51" t="n">
-        <v>219.9544666403959</v>
+        <v>198.1510758155493</v>
       </c>
     </row>
     <row r="52">
@@ -2588,28 +2596,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E52" t="n">
-        <v>2.21771502494812</v>
+        <v>2.171270558834076</v>
       </c>
       <c r="F52" t="n">
         <v>100</v>
       </c>
       <c r="G52" t="n">
-        <v>85.20742621292536</v>
+        <v>35.51153901902885</v>
       </c>
       <c r="H52" t="n">
-        <v>98.25385469296543</v>
+        <v>107.4057204858784</v>
       </c>
       <c r="I52" t="n">
-        <v>85.20742621292536</v>
+        <v>35.51153901902885</v>
       </c>
       <c r="J52" t="n">
-        <v>98.25385469296543</v>
+        <v>107.4057204858784</v>
       </c>
       <c r="K52" t="n">
-        <v>19.59838172597339</v>
+        <v>26.86237323746136</v>
       </c>
       <c r="L52" t="n">
-        <v>654.3762775284318</v>
+        <v>724.6427364971073</v>
       </c>
     </row>
     <row r="53">
@@ -2630,28 +2638,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E53" t="n">
-        <v>2.196247259775797</v>
+        <v>2.09732195854187</v>
       </c>
       <c r="F53" t="n">
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>120.9043592566087</v>
+        <v>46.64785562333473</v>
       </c>
       <c r="H53" t="n">
-        <v>157.1176995349617</v>
+        <v>156.0186197263497</v>
       </c>
       <c r="I53" t="n">
-        <v>120.9043592566087</v>
+        <v>46.64785562333473</v>
       </c>
       <c r="J53" t="n">
-        <v>157.1176995349617</v>
+        <v>156.0186197263497</v>
       </c>
       <c r="K53" t="n">
-        <v>52.19746474244935</v>
+        <v>36.81240779489718</v>
       </c>
       <c r="L53" t="n">
-        <v>573.1773272715176</v>
+        <v>568.4682740572111</v>
       </c>
     </row>
     <row r="54">
@@ -2672,28 +2680,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E54" t="n">
-        <v>0.05488872528076172</v>
+        <v>0.05418124914169312</v>
       </c>
       <c r="F54" t="n">
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>28.23937792450594</v>
+        <v>23.00601802836938</v>
       </c>
       <c r="H54" t="n">
-        <v>32.55135255600849</v>
+        <v>41.22391773750977</v>
       </c>
       <c r="I54" t="n">
-        <v>28.23937792450594</v>
+        <v>23.00601802836938</v>
       </c>
       <c r="J54" t="n">
-        <v>32.55135255600849</v>
+        <v>41.22391773750977</v>
       </c>
       <c r="K54" t="n">
-        <v>3.735313818293337</v>
+        <v>9.54360599909379</v>
       </c>
       <c r="L54" t="n">
-        <v>149.9237128808077</v>
+        <v>216.510183800325</v>
       </c>
     </row>
     <row r="55">
@@ -2714,28 +2722,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E55" t="n">
-        <v>0.6151026089986166</v>
+        <v>0.6366844487190246</v>
       </c>
       <c r="F55" t="n">
-        <v>66.66666666666666</v>
+        <v>92</v>
       </c>
       <c r="G55" t="n">
-        <v>65.50623241031134</v>
+        <v>29.72035854397576</v>
       </c>
       <c r="H55" t="n">
-        <v>70.79377918328066</v>
+        <v>59.51424635828349</v>
       </c>
       <c r="I55" t="n">
-        <v>65.50623241031134</v>
+        <v>29.72035854397576</v>
       </c>
       <c r="J55" t="n">
-        <v>85.84825815137275</v>
+        <v>63.16416136922818</v>
       </c>
       <c r="K55" t="n">
-        <v>7.477720358015297</v>
+        <v>10.51583334519222</v>
       </c>
       <c r="L55" t="n">
-        <v>203.3188953192783</v>
+        <v>154.9912671623161</v>
       </c>
     </row>
     <row r="56">
@@ -2756,7 +2764,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2068752447764079</v>
+        <v>0.207843120098114</v>
       </c>
       <c r="F56" t="n">
         <v>100</v>
@@ -2774,7 +2782,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>3.570611593983174e-15</v>
       </c>
       <c r="L56" t="n">
         <v>0</v>
@@ -2798,7 +2806,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E57" t="n">
-        <v>0.212333599726359</v>
+        <v>0.2078845810890198</v>
       </c>
       <c r="F57" t="n">
         <v>100</v>
@@ -2807,19 +2815,19 @@
         <v>16.77327413265929</v>
       </c>
       <c r="H57" t="n">
-        <v>21.54204184322326</v>
+        <v>16.77327413265929</v>
       </c>
       <c r="I57" t="n">
         <v>16.77327413265929</v>
       </c>
       <c r="J57" t="n">
-        <v>21.54204184322326</v>
+        <v>16.77327413265929</v>
       </c>
       <c r="K57" t="n">
-        <v>8.259747964190705</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L57" t="n">
-        <v>28.43075044769397</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2840,7 +2848,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E58" t="n">
-        <v>0.146990696589152</v>
+        <v>0.1452521872520447</v>
       </c>
       <c r="F58" t="n">
         <v>100</v>
@@ -2858,7 +2866,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K58" t="n">
-        <v>0</v>
+        <v>3.570611593983174e-15</v>
       </c>
       <c r="L58" t="n">
         <v>0</v>
@@ -2882,7 +2890,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E59" t="n">
-        <v>0.1455210049947103</v>
+        <v>0.1462344884872437</v>
       </c>
       <c r="F59" t="n">
         <v>100</v>
@@ -2900,7 +2908,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L59" t="n">
         <v>0</v>
@@ -2924,7 +2932,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E60" t="n">
-        <v>0.02262369791666667</v>
+        <v>0.007531299591064453</v>
       </c>
       <c r="F60" t="n">
         <v>100</v>
@@ -2942,7 +2950,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>3.570611593983174e-15</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
@@ -2966,7 +2974,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E61" t="n">
-        <v>0.09221196174621582</v>
+        <v>0.08962120056152344</v>
       </c>
       <c r="F61" t="n">
         <v>100</v>
@@ -2984,7 +2992,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
@@ -3008,7 +3016,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E62" t="n">
-        <v>0.329405943552653</v>
+        <v>0.32591224193573</v>
       </c>
       <c r="F62" t="n">
         <v>100</v>
@@ -3026,7 +3034,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="K62" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L62" t="n">
         <v>-1.431247886831891e-14</v>
@@ -3050,7 +3058,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E63" t="n">
-        <v>0.3323976198832194</v>
+        <v>0.3320509099960327</v>
       </c>
       <c r="F63" t="n">
         <v>100</v>
@@ -3059,19 +3067,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H63" t="n">
-        <v>51.20269814256776</v>
+        <v>49.44269207730557</v>
       </c>
       <c r="I63" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J63" t="n">
-        <v>51.20269814256776</v>
+        <v>49.44269207730557</v>
       </c>
       <c r="K63" t="n">
-        <v>4.420837457474725</v>
+        <v>3.185952253599189</v>
       </c>
       <c r="L63" t="n">
-        <v>5.246360882955188</v>
+        <v>1.62869540397961</v>
       </c>
     </row>
     <row r="64">
@@ -3092,7 +3100,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E64" t="n">
-        <v>0.2426233291625977</v>
+        <v>0.2388650012016297</v>
       </c>
       <c r="F64" t="n">
         <v>100</v>
@@ -3101,19 +3109,19 @@
         <v>24.82249030015713</v>
       </c>
       <c r="H64" t="n">
-        <v>24.82249030015713</v>
+        <v>24.84569542949007</v>
       </c>
       <c r="I64" t="n">
         <v>24.82249030015713</v>
       </c>
       <c r="J64" t="n">
-        <v>24.82249030015713</v>
+        <v>24.84569542949007</v>
       </c>
       <c r="K64" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>0.2320512933293372</v>
       </c>
       <c r="L64" t="n">
-        <v>-1.431247886831891e-14</v>
+        <v>0.0934842920768082</v>
       </c>
     </row>
     <row r="65">
@@ -3134,7 +3142,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E65" t="n">
-        <v>0.2433927059173584</v>
+        <v>0.2409717726707458</v>
       </c>
       <c r="F65" t="n">
         <v>100</v>
@@ -3143,19 +3151,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H65" t="n">
-        <v>51.20269814256776</v>
+        <v>49.47614872262835</v>
       </c>
       <c r="I65" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J65" t="n">
-        <v>51.20269814256776</v>
+        <v>49.47614872262835</v>
       </c>
       <c r="K65" t="n">
-        <v>4.420837457474725</v>
+        <v>2.519496764162747</v>
       </c>
       <c r="L65" t="n">
-        <v>5.246360882955188</v>
+        <v>1.697465025411863</v>
       </c>
     </row>
     <row r="66">
@@ -3176,7 +3184,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E66" t="n">
-        <v>0.009020725886027018</v>
+        <v>0.008814167976379395</v>
       </c>
       <c r="F66" t="n">
         <v>100</v>
@@ -3194,7 +3202,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="K66" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L66" t="n">
         <v>-1.431247886831891e-14</v>
@@ -3218,7 +3226,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E67" t="n">
-        <v>0.1045376459757487</v>
+        <v>0.1046896910667419</v>
       </c>
       <c r="F67" t="n">
         <v>100</v>
@@ -3236,7 +3244,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>2.142366956389904e-14</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
@@ -3260,7 +3268,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E68" t="n">
-        <v>0.09198904037475586</v>
+        <v>0.09339206218719483</v>
       </c>
       <c r="F68" t="n">
         <v>100</v>
@@ -3278,7 +3286,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
@@ -3302,7 +3310,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E69" t="n">
-        <v>0.09185226758321126</v>
+        <v>0.09400078773498535</v>
       </c>
       <c r="F69" t="n">
         <v>100</v>
@@ -3320,7 +3328,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L69" t="n">
         <v>0</v>
@@ -3344,7 +3352,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E70" t="n">
-        <v>0.04980762799580892</v>
+        <v>0.05075753211975097</v>
       </c>
       <c r="F70" t="n">
         <v>100</v>
@@ -3362,7 +3370,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
@@ -3386,7 +3394,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E71" t="n">
-        <v>0.0497140089670817</v>
+        <v>0.05101221084594727</v>
       </c>
       <c r="F71" t="n">
         <v>100</v>
@@ -3404,7 +3412,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
@@ -3428,7 +3436,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E72" t="n">
-        <v>0.002295255661010742</v>
+        <v>0.002319879531860352</v>
       </c>
       <c r="F72" t="n">
         <v>100</v>
@@ -3446,7 +3454,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K72" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L72" t="n">
         <v>0</v>
@@ -3470,7 +3478,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E73" t="n">
-        <v>0.02660640080769857</v>
+        <v>0.0264729905128479</v>
       </c>
       <c r="F73" t="n">
         <v>100</v>
@@ -3488,7 +3496,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L73" t="n">
         <v>0</v>
@@ -3512,7 +3520,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E74" t="n">
-        <v>0.35843292872111</v>
+        <v>0.358566062450409</v>
       </c>
       <c r="F74" t="n">
         <v>100</v>
@@ -3521,19 +3529,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H74" t="n">
-        <v>30.95896547744237</v>
+        <v>31.06813056819737</v>
       </c>
       <c r="I74" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J74" t="n">
-        <v>30.95896547744237</v>
+        <v>31.06813056819737</v>
       </c>
       <c r="K74" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>0.8576863244551524</v>
       </c>
       <c r="L74" t="n">
-        <v>-1.147555683470468e-14</v>
+        <v>0.3526122048055629</v>
       </c>
     </row>
     <row r="75">
@@ -3554,7 +3562,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E75" t="n">
-        <v>0.368560791015625</v>
+        <v>0.3596773505210876</v>
       </c>
       <c r="F75" t="n">
         <v>100</v>
@@ -3563,19 +3571,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H75" t="n">
-        <v>38.20684438128487</v>
+        <v>40.19866139860349</v>
       </c>
       <c r="I75" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J75" t="n">
-        <v>38.20684438128487</v>
+        <v>40.19866139860349</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>3.298033702524826</v>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>5.213246604302893</v>
       </c>
     </row>
     <row r="76">
@@ -3596,7 +3604,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E76" t="n">
-        <v>0.2683002948760986</v>
+        <v>0.2759222602844238</v>
       </c>
       <c r="F76" t="n">
         <v>100</v>
@@ -3605,19 +3613,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H76" t="n">
-        <v>30.95896547744237</v>
+        <v>31.68225774080297</v>
       </c>
       <c r="I76" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J76" t="n">
-        <v>30.95896547744237</v>
+        <v>31.68225774080297</v>
       </c>
       <c r="K76" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>1.669414454809327</v>
       </c>
       <c r="L76" t="n">
-        <v>-1.147555683470468e-14</v>
+        <v>2.336293387734841</v>
       </c>
     </row>
     <row r="77">
@@ -3638,28 +3646,28 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E77" t="n">
-        <v>0.2679816881815593</v>
+        <v>0.2704894804954529</v>
       </c>
       <c r="F77" t="n">
         <v>100</v>
       </c>
       <c r="G77" t="n">
-        <v>40.11981949922859</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="H77" t="n">
-        <v>42.19704857420336</v>
+        <v>42.65164089282676</v>
       </c>
       <c r="I77" t="n">
-        <v>40.11981949922859</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="J77" t="n">
-        <v>42.19704857420336</v>
+        <v>42.65164089282676</v>
       </c>
       <c r="K77" t="n">
-        <v>3.597866296815593</v>
+        <v>6.570842334189233</v>
       </c>
       <c r="L77" t="n">
-        <v>10.44368949473629</v>
+        <v>11.63350855984097</v>
       </c>
     </row>
     <row r="78">
@@ -3680,7 +3688,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E78" t="n">
-        <v>0.01367831230163574</v>
+        <v>0.01343673944473267</v>
       </c>
       <c r="F78" t="n">
         <v>100</v>
@@ -3689,19 +3697,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H78" t="n">
-        <v>30.95896547744237</v>
+        <v>30.97669393536907</v>
       </c>
       <c r="I78" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J78" t="n">
-        <v>30.95896547744237</v>
+        <v>30.97669393536907</v>
       </c>
       <c r="K78" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>0.1772845792669813</v>
       </c>
       <c r="L78" t="n">
-        <v>-1.147555683470468e-14</v>
+        <v>0.05726437448181175</v>
       </c>
     </row>
     <row r="79">
@@ -3722,7 +3730,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E79" t="n">
-        <v>0.1614279747009277</v>
+        <v>0.1610432124137878</v>
       </c>
       <c r="F79" t="n">
         <v>100</v>
@@ -3740,7 +3748,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="K79" t="n">
-        <v>0</v>
+        <v>1.428244637593269e-14</v>
       </c>
       <c r="L79" t="n">
         <v>0</v>
@@ -3764,7 +3772,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E80" t="n">
-        <v>0.5383226871490479</v>
+        <v>0.532923948764801</v>
       </c>
       <c r="F80" t="n">
         <v>100</v>
@@ -3773,19 +3781,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H80" t="n">
-        <v>1.026285782096494</v>
+        <v>1.482212030891633</v>
       </c>
       <c r="I80" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J80" t="n">
-        <v>1.026285782096494</v>
+        <v>1.482212030891633</v>
       </c>
       <c r="K80" t="n">
-        <v>0</v>
+        <v>1.288251998500642</v>
       </c>
       <c r="L80" t="n">
-        <v>0</v>
+        <v>44.42488210874114</v>
       </c>
     </row>
     <row r="81">
@@ -3806,7 +3814,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E81" t="n">
-        <v>0.5029064019521078</v>
+        <v>0.5244971489906312</v>
       </c>
       <c r="F81" t="n">
         <v>100</v>
@@ -3815,19 +3823,19 @@
         <v>18.17186472076723</v>
       </c>
       <c r="H81" t="n">
-        <v>25.27456652346707</v>
+        <v>21.56787090188577</v>
       </c>
       <c r="I81" t="n">
         <v>18.17186472076723</v>
       </c>
       <c r="J81" t="n">
-        <v>25.27456652346707</v>
+        <v>21.56787090188577</v>
       </c>
       <c r="K81" t="n">
-        <v>6.151120196643584</v>
+        <v>3.977812161828188</v>
       </c>
       <c r="L81" t="n">
-        <v>39.08625730953579</v>
+        <v>18.68826470646959</v>
       </c>
     </row>
     <row r="82">
@@ -3848,28 +3856,28 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E82" t="n">
-        <v>0.4145996570587158</v>
+        <v>0.3955034112930298</v>
       </c>
       <c r="F82" t="n">
         <v>100</v>
       </c>
       <c r="G82" t="n">
-        <v>3.234846064445697</v>
+        <v>1.026285782096494</v>
       </c>
       <c r="H82" t="n">
-        <v>3.481706425519638</v>
+        <v>4.778366316858686</v>
       </c>
       <c r="I82" t="n">
-        <v>3.234846064445697</v>
+        <v>1.026285782096494</v>
       </c>
       <c r="J82" t="n">
-        <v>3.481706425519638</v>
+        <v>4.778366316858686</v>
       </c>
       <c r="K82" t="n">
-        <v>0.4275746877548641</v>
+        <v>5.270840478941794</v>
       </c>
       <c r="L82" t="n">
-        <v>239.2531092467458</v>
+        <v>365.5980234957023</v>
       </c>
     </row>
     <row r="83">
@@ -3890,7 +3898,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E83" t="n">
-        <v>0.405750036239624</v>
+        <v>0.3907591199874878</v>
       </c>
       <c r="F83" t="n">
         <v>100</v>
@@ -3899,19 +3907,19 @@
         <v>18.17186472076723</v>
       </c>
       <c r="H83" t="n">
-        <v>21.37266928489361</v>
+        <v>24.33509387540884</v>
       </c>
       <c r="I83" t="n">
         <v>18.17186472076723</v>
       </c>
       <c r="J83" t="n">
-        <v>21.37266928489361</v>
+        <v>24.33509387540884</v>
       </c>
       <c r="K83" t="n">
-        <v>5.543956130165241</v>
+        <v>5.927749011974221</v>
       </c>
       <c r="L83" t="n">
-        <v>17.6140677542488</v>
+        <v>33.91632751700012</v>
       </c>
     </row>
     <row r="84">
@@ -3932,7 +3940,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E84" t="n">
-        <v>0.01626936594645182</v>
+        <v>0.01594146013259888</v>
       </c>
       <c r="F84" t="n">
         <v>100</v>
@@ -3941,19 +3949,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H84" t="n">
-        <v>1.026285782096494</v>
+        <v>1.04109740376093</v>
       </c>
       <c r="I84" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J84" t="n">
-        <v>1.026285782096494</v>
+        <v>1.04109740376093</v>
       </c>
       <c r="K84" t="n">
-        <v>0</v>
+        <v>0.1042036791464984</v>
       </c>
       <c r="L84" t="n">
-        <v>0</v>
+        <v>1.443225846330945</v>
       </c>
     </row>
     <row r="85">
@@ -3974,7 +3982,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E85" t="n">
-        <v>0.1894310315450033</v>
+        <v>0.1967201089859009</v>
       </c>
       <c r="F85" t="n">
         <v>100</v>
@@ -3992,7 +4000,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="K85" t="n">
-        <v>0</v>
+        <v>3.570611593983174e-15</v>
       </c>
       <c r="L85" t="n">
         <v>0</v>
@@ -4016,7 +4024,7 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E86" t="n">
-        <v>0.6409023602803549</v>
+        <v>2.254394590854645</v>
       </c>
       <c r="F86" t="n">
         <v>100</v>
@@ -4025,19 +4033,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="H86" t="n">
-        <v>47.09298202339563</v>
+        <v>45.73137409085769</v>
       </c>
       <c r="I86" t="n">
         <v>44.28900565726017</v>
       </c>
       <c r="J86" t="n">
-        <v>47.09298202339563</v>
+        <v>45.73137409085769</v>
       </c>
       <c r="K86" t="n">
-        <v>3.172547040666831</v>
+        <v>2.844380686534761</v>
       </c>
       <c r="L86" t="n">
-        <v>6.331089001714381</v>
+        <v>3.256718935529046</v>
       </c>
     </row>
     <row r="87">
@@ -4058,7 +4066,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E87" t="n">
-        <v>0.6404439608256022</v>
+        <v>0.6372906613349915</v>
       </c>
       <c r="F87" t="n">
         <v>100</v>
@@ -4067,19 +4075,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H87" t="n">
-        <v>53.36624948003475</v>
+        <v>52.66253699384136</v>
       </c>
       <c r="I87" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J87" t="n">
-        <v>53.36624948003475</v>
+        <v>52.66253699384136</v>
       </c>
       <c r="K87" t="n">
-        <v>4.90105852678794</v>
+        <v>3.69088760159136</v>
       </c>
       <c r="L87" t="n">
-        <v>5.599162244400985</v>
+        <v>4.20668198343103</v>
       </c>
     </row>
     <row r="88">
@@ -4100,28 +4108,28 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E88" t="n">
-        <v>0.4898159503936768</v>
+        <v>0.4856209206581116</v>
       </c>
       <c r="F88" t="n">
         <v>100</v>
       </c>
       <c r="G88" t="n">
-        <v>49.51402501206863</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="H88" t="n">
-        <v>51.6899336950399</v>
+        <v>50.99879962602679</v>
       </c>
       <c r="I88" t="n">
-        <v>49.51402501206863</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="J88" t="n">
-        <v>51.6899336950399</v>
+        <v>50.99879962602679</v>
       </c>
       <c r="K88" t="n">
-        <v>1.884392195768267</v>
+        <v>4.689307717249227</v>
       </c>
       <c r="L88" t="n">
-        <v>16.71053104026173</v>
+        <v>15.15002170220705</v>
       </c>
     </row>
     <row r="89">
@@ -4142,7 +4150,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E89" t="n">
-        <v>0.4775613149007161</v>
+        <v>0.4766767072677612</v>
       </c>
       <c r="F89" t="n">
         <v>100</v>
@@ -4151,19 +4159,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H89" t="n">
-        <v>55.47395393224307</v>
+        <v>57.61343046341774</v>
       </c>
       <c r="I89" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J89" t="n">
-        <v>55.47395393224307</v>
+        <v>57.61343046341774</v>
       </c>
       <c r="K89" t="n">
-        <v>4.275854862675949</v>
+        <v>4.991667725708012</v>
       </c>
       <c r="L89" t="n">
-        <v>9.769809921173946</v>
+        <v>14.00332701362253</v>
       </c>
     </row>
     <row r="90">
@@ -4184,7 +4192,7 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E90" t="n">
-        <v>0.01843627293904622</v>
+        <v>0.01850558996200562</v>
       </c>
       <c r="F90" t="n">
         <v>100</v>
@@ -4193,19 +4201,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="H90" t="n">
-        <v>44.28900565726017</v>
+        <v>45.44935890994204</v>
       </c>
       <c r="I90" t="n">
         <v>44.28900565726017</v>
       </c>
       <c r="J90" t="n">
-        <v>44.28900565726017</v>
+        <v>45.44935890994204</v>
       </c>
       <c r="K90" t="n">
-        <v>0</v>
+        <v>1.704561875361765</v>
       </c>
       <c r="L90" t="n">
-        <v>0</v>
+        <v>2.61995778740555</v>
       </c>
     </row>
     <row r="91">
@@ -4226,7 +4234,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E91" t="n">
-        <v>0.2154332796732585</v>
+        <v>0.2175374698638916</v>
       </c>
       <c r="F91" t="n">
         <v>100</v>
@@ -4244,10 +4252,10 @@
         <v>50.53662202027962</v>
       </c>
       <c r="K91" t="n">
-        <v>0</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L91" t="n">
-        <v>0</v>
+        <v>1.405995706390842e-14</v>
       </c>
     </row>
     <row r="92">
@@ -4268,7 +4276,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E92" t="n">
-        <v>0.6909650166829427</v>
+        <v>0.6990683484077453</v>
       </c>
       <c r="F92" t="n">
         <v>100</v>
@@ -4277,19 +4285,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H92" t="n">
-        <v>47.33481367365937</v>
+        <v>48.17965504840349</v>
       </c>
       <c r="I92" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J92" t="n">
-        <v>47.33481367365937</v>
+        <v>48.17965504840349</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>2.660085952667409</v>
       </c>
       <c r="L92" t="n">
-        <v>0</v>
+        <v>1.784820323934757</v>
       </c>
     </row>
     <row r="93">
@@ -4310,28 +4318,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E93" t="n">
-        <v>0.6926216284434</v>
+        <v>0.6919659090042114</v>
       </c>
       <c r="F93" t="n">
         <v>100</v>
       </c>
       <c r="G93" t="n">
-        <v>55.07651864916471</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="H93" t="n">
-        <v>61.49892107707267</v>
+        <v>58.47879925218077</v>
       </c>
       <c r="I93" t="n">
-        <v>55.07651864916471</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="J93" t="n">
-        <v>61.49892107707267</v>
+        <v>58.47879925218077</v>
       </c>
       <c r="K93" t="n">
-        <v>5.561963655895149</v>
+        <v>5.012389607812267</v>
       </c>
       <c r="L93" t="n">
-        <v>13.17833679069638</v>
+        <v>7.620314648841625</v>
       </c>
     </row>
     <row r="94">
@@ -4352,28 +4360,28 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E94" t="n">
-        <v>0.5527960459391276</v>
+        <v>0.5555941009521485</v>
       </c>
       <c r="F94" t="n">
         <v>100</v>
       </c>
       <c r="G94" t="n">
-        <v>48.59309813195462</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="H94" t="n">
-        <v>57.16959076061679</v>
+        <v>55.16478562210857</v>
       </c>
       <c r="I94" t="n">
-        <v>48.59309813195462</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="J94" t="n">
-        <v>57.16959076061679</v>
+        <v>55.16478562210857</v>
       </c>
       <c r="K94" t="n">
-        <v>8.108299974954489</v>
+        <v>8.426754492484168</v>
       </c>
       <c r="L94" t="n">
-        <v>20.77704827309847</v>
+        <v>16.54167691972217</v>
       </c>
     </row>
     <row r="95">
@@ -4394,28 +4402,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E95" t="n">
-        <v>0.5557576020558676</v>
+        <v>0.5420695209503174</v>
       </c>
       <c r="F95" t="n">
         <v>100</v>
       </c>
       <c r="G95" t="n">
-        <v>69.75620930338751</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="H95" t="n">
-        <v>78.10890153459694</v>
+        <v>66.54862656309342</v>
       </c>
       <c r="I95" t="n">
-        <v>69.75620930338751</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="J95" t="n">
-        <v>78.10890153459694</v>
+        <v>66.54862656309342</v>
       </c>
       <c r="K95" t="n">
-        <v>9.102741062096232</v>
+        <v>8.932622953389657</v>
       </c>
       <c r="L95" t="n">
-        <v>43.74618951696812</v>
+        <v>22.47146353473206</v>
       </c>
     </row>
     <row r="96">
@@ -4436,28 +4444,28 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E96" t="n">
-        <v>0.02321434020996094</v>
+        <v>0.02307023048400879</v>
       </c>
       <c r="F96" t="n">
         <v>100</v>
       </c>
       <c r="G96" t="n">
-        <v>47.48853170359875</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="H96" t="n">
-        <v>51.33415315259479</v>
+        <v>49.06946089259275</v>
       </c>
       <c r="I96" t="n">
-        <v>47.48853170359875</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="J96" t="n">
-        <v>51.33415315259479</v>
+        <v>49.06946089259275</v>
       </c>
       <c r="K96" t="n">
-        <v>3.51225657220097</v>
+        <v>2.270751167183505</v>
       </c>
       <c r="L96" t="n">
-        <v>8.449044516173833</v>
+        <v>3.664633034984714</v>
       </c>
     </row>
     <row r="97">
@@ -4478,7 +4486,7 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E97" t="n">
-        <v>0.2747716903686523</v>
+        <v>0.2737784099578857</v>
       </c>
       <c r="F97" t="n">
         <v>100</v>
@@ -4487,19 +4495,19 @@
         <v>54.33806753213224</v>
       </c>
       <c r="H97" t="n">
-        <v>54.33806753213224</v>
+        <v>54.34114189273103</v>
       </c>
       <c r="I97" t="n">
         <v>54.33806753213224</v>
       </c>
       <c r="J97" t="n">
-        <v>54.33806753213224</v>
+        <v>54.34114189273103</v>
       </c>
       <c r="K97" t="n">
-        <v>0</v>
+        <v>0.02162894061667199</v>
       </c>
       <c r="L97" t="n">
-        <v>0</v>
+        <v>0.005657839408753304</v>
       </c>
     </row>
     <row r="98">
@@ -4520,7 +4528,7 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8823420206705729</v>
+        <v>0.8661245393753052</v>
       </c>
       <c r="F98" t="n">
         <v>100</v>
@@ -4529,19 +4537,19 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="H98" t="n">
-        <v>0.9048907529052066</v>
+        <v>2.085010959758808</v>
       </c>
       <c r="I98" t="n">
         <v>0.1017009531136672</v>
       </c>
       <c r="J98" t="n">
-        <v>0.9048907529052066</v>
+        <v>2.085010959758808</v>
       </c>
       <c r="K98" t="n">
-        <v>0.6955827706800103</v>
+        <v>2.912846636412049</v>
       </c>
       <c r="L98" t="n">
-        <v>789.7564134859633</v>
+        <v>1950.139055657101</v>
       </c>
     </row>
     <row r="99">
@@ -4562,7 +4570,7 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E99" t="n">
-        <v>0.8303689956665039</v>
+        <v>0.8166107010841369</v>
       </c>
       <c r="F99" t="n">
         <v>100</v>
@@ -4571,19 +4579,19 @@
         <v>10.54487657926557</v>
       </c>
       <c r="H99" t="n">
-        <v>14.25655709293335</v>
+        <v>19.80986964450671</v>
       </c>
       <c r="I99" t="n">
         <v>10.54487657926557</v>
       </c>
       <c r="J99" t="n">
-        <v>14.25655709293335</v>
+        <v>19.80986964450671</v>
       </c>
       <c r="K99" t="n">
-        <v>6.428819231135939</v>
+        <v>6.532783985572673</v>
       </c>
       <c r="L99" t="n">
-        <v>35.19889953919489</v>
+        <v>87.86250835271922</v>
       </c>
     </row>
     <row r="100">
@@ -4604,28 +4612,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E100" t="n">
-        <v>0.6474260489145914</v>
+        <v>0.6621059823036194</v>
       </c>
       <c r="F100" t="n">
         <v>100</v>
       </c>
       <c r="G100" t="n">
-        <v>0.9562267675903433</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="H100" t="n">
-        <v>4.466252659464188</v>
+        <v>10.41332765203487</v>
       </c>
       <c r="I100" t="n">
-        <v>0.9562267675903433</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="J100" t="n">
-        <v>4.466252659464188</v>
+        <v>10.41332765203487</v>
       </c>
       <c r="K100" t="n">
-        <v>3.357874487251162</v>
+        <v>8.134361461979164</v>
       </c>
       <c r="L100" t="n">
-        <v>4291.55437852429</v>
+        <v>10139.1642685947</v>
       </c>
     </row>
     <row r="101">
@@ -4646,28 +4654,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E101" t="n">
-        <v>0.6506377855936686</v>
+        <v>0.6329903674125671</v>
       </c>
       <c r="F101" t="n">
         <v>100</v>
       </c>
       <c r="G101" t="n">
-        <v>17.67202855799388</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="H101" t="n">
-        <v>26.56685283806384</v>
+        <v>31.96446820773227</v>
       </c>
       <c r="I101" t="n">
-        <v>17.67202855799388</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="J101" t="n">
-        <v>26.56685283806384</v>
+        <v>31.96446820773227</v>
       </c>
       <c r="K101" t="n">
-        <v>8.678924239452842</v>
+        <v>14.36505863199191</v>
       </c>
       <c r="L101" t="n">
-        <v>151.9408609324299</v>
+        <v>203.1279500282074</v>
       </c>
     </row>
     <row r="102">
@@ -4688,28 +4696,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E102" t="n">
-        <v>0.02623438835144043</v>
+        <v>0.0265893292427063</v>
       </c>
       <c r="F102" t="n">
         <v>100</v>
       </c>
       <c r="G102" t="n">
-        <v>3.940167061999031</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="H102" t="n">
-        <v>5.960138909456727</v>
+        <v>3.917027155943254</v>
       </c>
       <c r="I102" t="n">
-        <v>3.940167061999031</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="J102" t="n">
-        <v>5.960138909456727</v>
+        <v>3.917027155943254</v>
       </c>
       <c r="K102" t="n">
-        <v>1.876035790708683</v>
+        <v>4.076786859968062</v>
       </c>
       <c r="L102" t="n">
-        <v>5760.455312346296</v>
+        <v>3751.51469678494</v>
       </c>
     </row>
     <row r="103">
@@ -4730,28 +4738,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E103" t="n">
-        <v>0.292155663172404</v>
+        <v>0.2968737006187439</v>
       </c>
       <c r="F103" t="n">
-        <v>66.66666666666666</v>
+        <v>81</v>
       </c>
       <c r="G103" t="n">
         <v>10.54487657926557</v>
       </c>
       <c r="H103" t="n">
-        <v>10.54487657926557</v>
+        <v>18.80629214001168</v>
       </c>
       <c r="I103" t="n">
-        <v>10.54487657926557</v>
+        <v>2.525125306232527</v>
       </c>
       <c r="J103" t="n">
-        <v>30.56372180302802</v>
+        <v>23.64187151603962</v>
       </c>
       <c r="K103" t="n">
-        <v>0</v>
+        <v>24.79844328455565</v>
       </c>
       <c r="L103" t="n">
-        <v>0</v>
+        <v>78.3453035096737</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run #2: with Simulated Quantum Annealers
</commit_message>
<xml_diff>
--- a/results/graphs/benchmark_results.xlsx
+++ b/results/graphs/benchmark_results.xlsx
@@ -496,7 +496,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E2" t="n">
-        <v>0.07327836990356446</v>
+        <v>0.1879293123881022</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -538,7 +538,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06886888027191163</v>
+        <v>0.2010863622029622</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -580,7 +580,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E4" t="n">
-        <v>0.03294903993606568</v>
+        <v>0.1523040135701497</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -622,7 +622,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03346406936645508</v>
+        <v>0.1542932192484538</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -664,7 +664,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E6" t="n">
-        <v>0.002898759841918945</v>
+        <v>0.6868889331817627</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -706,7 +706,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03336961030960083</v>
+        <v>7.052044312159221</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -748,7 +748,7 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E8" t="n">
-        <v>1.022696838378906</v>
+        <v>1.463008006413778</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -757,19 +757,19 @@
         <v>12.04748748354309</v>
       </c>
       <c r="H8" t="n">
-        <v>13.40560809486521</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="I8" t="n">
         <v>12.04748748354309</v>
       </c>
       <c r="J8" t="n">
-        <v>13.40560809486521</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="K8" t="n">
-        <v>3.899462568235728</v>
+        <v>2.175583928816829e-15</v>
       </c>
       <c r="L8" t="n">
-        <v>11.27306098617918</v>
+        <v>-1.474462490064223e-14</v>
       </c>
     </row>
     <row r="9">
@@ -790,7 +790,7 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9244257020950317</v>
+        <v>1.401365677515666</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -799,19 +799,19 @@
         <v>53.31120138136255</v>
       </c>
       <c r="H9" t="n">
-        <v>66.44696065207982</v>
+        <v>74.68741544755886</v>
       </c>
       <c r="I9" t="n">
         <v>53.31120138136255</v>
       </c>
       <c r="J9" t="n">
-        <v>66.44696065207982</v>
+        <v>74.68741544755886</v>
       </c>
       <c r="K9" t="n">
-        <v>12.49186075768247</v>
+        <v>23.71273295981149</v>
       </c>
       <c r="L9" t="n">
-        <v>24.63977350041392</v>
+        <v>40.09704060743486</v>
       </c>
     </row>
     <row r="10">
@@ -832,7 +832,7 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8140435528755188</v>
+        <v>1.283445119857788</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -841,19 +841,19 @@
         <v>12.04748748354309</v>
       </c>
       <c r="H10" t="n">
-        <v>27.44428813559835</v>
+        <v>21.98188464172121</v>
       </c>
       <c r="I10" t="n">
         <v>12.04748748354309</v>
       </c>
       <c r="J10" t="n">
-        <v>27.44428813559835</v>
+        <v>21.98188464172121</v>
       </c>
       <c r="K10" t="n">
-        <v>13.91566858124934</v>
+        <v>12.02269175057124</v>
       </c>
       <c r="L10" t="n">
-        <v>127.8009267333736</v>
+        <v>82.46032354670251</v>
       </c>
     </row>
     <row r="11">
@@ -874,28 +874,28 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7755626630783081</v>
+        <v>1.17594838142395</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>53.31120138136255</v>
+        <v>70.55706073287621</v>
       </c>
       <c r="H11" t="n">
-        <v>85.11152571728677</v>
+        <v>84.6847268524665</v>
       </c>
       <c r="I11" t="n">
-        <v>53.31120138136255</v>
+        <v>70.55706073287621</v>
       </c>
       <c r="J11" t="n">
-        <v>85.11152571728677</v>
+        <v>84.6847268524665</v>
       </c>
       <c r="K11" t="n">
-        <v>16.96516412925579</v>
+        <v>12.39306178552477</v>
       </c>
       <c r="L11" t="n">
-        <v>59.6503614848971</v>
+        <v>58.84978139335656</v>
       </c>
     </row>
     <row r="12">
@@ -916,28 +916,28 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E12" t="n">
-        <v>0.02709391832351685</v>
+        <v>1.115394592285156</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>12.04748748354309</v>
+        <v>19.45696800172116</v>
       </c>
       <c r="H12" t="n">
-        <v>12.63358626965861</v>
+        <v>20.62873454896448</v>
       </c>
       <c r="I12" t="n">
-        <v>12.04748748354309</v>
+        <v>19.45696800172116</v>
       </c>
       <c r="J12" t="n">
-        <v>12.63358626965861</v>
+        <v>20.62873454896448</v>
       </c>
       <c r="K12" t="n">
-        <v>0.7945323924873762</v>
+        <v>1.553604857683085</v>
       </c>
       <c r="L12" t="n">
-        <v>4.864904710763374</v>
+        <v>71.22852027979616</v>
       </c>
     </row>
     <row r="13">
@@ -958,29 +958,21 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2895361709594726</v>
+        <v>8.618704001108805</v>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" t="n">
-        <v>53.31120138136255</v>
-      </c>
-      <c r="H13" t="n">
-        <v>57.9647866961866</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>20.87387904273287</v>
+        <v>47.57847490964248</v>
       </c>
       <c r="J13" t="n">
-        <v>57.37777681846475</v>
-      </c>
-      <c r="K13" t="n">
-        <v>9.307170629648098</v>
-      </c>
-      <c r="L13" t="n">
-        <v>8.729094813554379</v>
-      </c>
+        <v>79.50395106466219</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1000,7 +992,7 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E14" t="n">
-        <v>1.133707711696625</v>
+        <v>1.610737323760986</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1009,19 +1001,19 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="H14" t="n">
-        <v>-6.172254514210448</v>
+        <v>-0.2852081487284537</v>
       </c>
       <c r="I14" t="n">
         <v>-11.80593354076133</v>
       </c>
       <c r="J14" t="n">
-        <v>-6.172254514210448</v>
+        <v>-0.2852081487284537</v>
       </c>
       <c r="K14" t="n">
-        <v>6.396806894390321</v>
+        <v>10.04646731912484</v>
       </c>
       <c r="L14" t="n">
-        <v>47.71904743576578</v>
+        <v>97.58419655892742</v>
       </c>
     </row>
     <row r="15">
@@ -1042,7 +1034,7 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E15" t="n">
-        <v>1.152146470546722</v>
+        <v>1.612162351608276</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1051,19 +1043,19 @@
         <v>13.7263575295875</v>
       </c>
       <c r="H15" t="n">
-        <v>28.34275111753655</v>
+        <v>18.97706366014659</v>
       </c>
       <c r="I15" t="n">
         <v>13.7263575295875</v>
       </c>
       <c r="J15" t="n">
-        <v>28.34275111753655</v>
+        <v>18.97706366014659</v>
       </c>
       <c r="K15" t="n">
-        <v>15.51730206809427</v>
+        <v>4.850132045736043</v>
       </c>
       <c r="L15" t="n">
-        <v>106.4841386831361</v>
+        <v>38.25272742051967</v>
       </c>
     </row>
     <row r="16">
@@ -1084,28 +1076,28 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8907021689414978</v>
+        <v>1.638352394104004</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>-11.80593354076133</v>
+        <v>4.297797156658406</v>
       </c>
       <c r="H16" t="n">
-        <v>21.96448947943182</v>
+        <v>21.84179742087983</v>
       </c>
       <c r="I16" t="n">
-        <v>-11.80593354076133</v>
+        <v>4.297797156658406</v>
       </c>
       <c r="J16" t="n">
-        <v>21.96448947943182</v>
+        <v>21.84179742087983</v>
       </c>
       <c r="K16" t="n">
-        <v>18.06001986135499</v>
+        <v>15.86367097427612</v>
       </c>
       <c r="L16" t="n">
-        <v>286.0461894317541</v>
+        <v>285.0069487979797</v>
       </c>
     </row>
     <row r="17">
@@ -1126,28 +1118,28 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9103633213043213</v>
+        <v>1.431125720342</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>16.32499152035578</v>
+        <v>64.48172630257449</v>
       </c>
       <c r="H17" t="n">
-        <v>63.1528352743077</v>
+        <v>70.66150778251817</v>
       </c>
       <c r="I17" t="n">
-        <v>16.32499152035578</v>
+        <v>64.48172630257449</v>
       </c>
       <c r="J17" t="n">
-        <v>63.1528352743077</v>
+        <v>70.66150778251817</v>
       </c>
       <c r="K17" t="n">
-        <v>25.08369718326212</v>
+        <v>8.18443166056025</v>
       </c>
       <c r="L17" t="n">
-        <v>360.0844407424198</v>
+        <v>414.7870265669938</v>
       </c>
     </row>
     <row r="18">
@@ -1168,28 +1160,30 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E18" t="n">
-        <v>0.02866180181503296</v>
+        <v>0.9904703299204508</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G18" t="n">
-        <v>-11.80593354076133</v>
+        <v>4.896138561360734</v>
       </c>
       <c r="H18" t="n">
-        <v>-8.416822271419015</v>
+        <v>10.69764543237702</v>
       </c>
       <c r="I18" t="n">
-        <v>-11.80593354076133</v>
-      </c>
-      <c r="J18" t="n">
-        <v>-8.416822271419015</v>
+        <v>4.896138561360734</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K18" t="n">
-        <v>4.084944442451147</v>
+        <v>8.204569699191927</v>
       </c>
       <c r="L18" t="n">
-        <v>28.70684692270224</v>
+        <v>190.6124483543989</v>
       </c>
     </row>
     <row r="19">
@@ -1210,29 +1204,21 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3432621693611145</v>
+        <v>8.696507374445597</v>
       </c>
       <c r="F19" t="n">
-        <v>79</v>
-      </c>
-      <c r="G19" t="n">
-        <v>13.7263575295875</v>
-      </c>
-      <c r="H19" t="n">
-        <v>19.73167474435576</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>13.7263575295875</v>
+        <v>27.99504865350196</v>
       </c>
       <c r="J19" t="n">
-        <v>27.85952743029948</v>
-      </c>
-      <c r="K19" t="n">
-        <v>5.777742686055614</v>
-      </c>
-      <c r="L19" t="n">
-        <v>43.75026077984378</v>
-      </c>
+        <v>92.18875943360921</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1252,28 +1238,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E20" t="n">
-        <v>1.330196940898895</v>
+        <v>1.927209297815959</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>-9.463170998014522</v>
+        <v>-3.758716405667779</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.456530469289016</v>
+        <v>0.770409565324441</v>
       </c>
       <c r="I20" t="n">
-        <v>-9.463170998014522</v>
+        <v>-3.758716405667779</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.456530469289016</v>
+        <v>0.770409565324441</v>
       </c>
       <c r="K20" t="n">
-        <v>7.725375342212417</v>
+        <v>4.266504127476306</v>
       </c>
       <c r="L20" t="n">
-        <v>95.17571362300437</v>
+        <v>108.1411354131304</v>
       </c>
     </row>
     <row r="21">
@@ -1294,28 +1280,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E21" t="n">
-        <v>1.250355911254883</v>
+        <v>1.770529349644979</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>15.06947538019221</v>
+        <v>24.95684465099749</v>
       </c>
       <c r="H21" t="n">
-        <v>33.32049410991213</v>
+        <v>33.36420076015548</v>
       </c>
       <c r="I21" t="n">
-        <v>15.06947538019221</v>
+        <v>24.95684465099749</v>
       </c>
       <c r="J21" t="n">
-        <v>33.32049410991213</v>
+        <v>33.36420076015548</v>
       </c>
       <c r="K21" t="n">
-        <v>15.2564804117167</v>
+        <v>7.447466314686423</v>
       </c>
       <c r="L21" t="n">
-        <v>121.1125023881697</v>
+        <v>121.4025367068215</v>
       </c>
     </row>
     <row r="22">
@@ -1336,28 +1322,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E22" t="n">
-        <v>1.025094621181488</v>
+        <v>1.59409236907959</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>-9.463170998014522</v>
+        <v>7.060641592855646</v>
       </c>
       <c r="H22" t="n">
-        <v>27.74100451441571</v>
+        <v>27.07035246089511</v>
       </c>
       <c r="I22" t="n">
-        <v>-9.463170998014522</v>
+        <v>7.060641592855646</v>
       </c>
       <c r="J22" t="n">
-        <v>27.74100451441571</v>
+        <v>27.07035246089511</v>
       </c>
       <c r="K22" t="n">
-        <v>18.16527609628692</v>
+        <v>22.78881140942149</v>
       </c>
       <c r="L22" t="n">
-        <v>393.1470277799702</v>
+        <v>386.0600581620555</v>
       </c>
     </row>
     <row r="23">
@@ -1378,28 +1364,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E23" t="n">
-        <v>0.9708001184463501</v>
+        <v>1.520270983378093</v>
       </c>
       <c r="F23" t="n">
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>18.7915703518064</v>
+        <v>42.03499384317907</v>
       </c>
       <c r="H23" t="n">
-        <v>66.36045503319389</v>
+        <v>66.78404275042151</v>
       </c>
       <c r="I23" t="n">
-        <v>18.7915703518064</v>
+        <v>42.03499384317907</v>
       </c>
       <c r="J23" t="n">
-        <v>66.36045503319389</v>
+        <v>66.78404275042151</v>
       </c>
       <c r="K23" t="n">
-        <v>23.4849287479963</v>
+        <v>29.05257162586466</v>
       </c>
       <c r="L23" t="n">
-        <v>340.3634058848536</v>
+        <v>343.1743047817349</v>
       </c>
     </row>
     <row r="24">
@@ -1420,28 +1406,30 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E24" t="n">
-        <v>0.03124053239822388</v>
+        <v>1.160794019699097</v>
       </c>
       <c r="F24" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G24" t="n">
-        <v>-9.463170998014522</v>
+        <v>27.0642714807036</v>
       </c>
       <c r="H24" t="n">
-        <v>-8.353630098055669</v>
+        <v>31.35686774303407</v>
       </c>
       <c r="I24" t="n">
-        <v>-9.463170998014522</v>
-      </c>
-      <c r="J24" t="n">
-        <v>-8.353630098055669</v>
+        <v>27.0642714807036</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K24" t="n">
-        <v>1.612896428302111</v>
+        <v>6.070647851979807</v>
       </c>
       <c r="L24" t="n">
-        <v>11.72483198487745</v>
+        <v>431.3568755083585</v>
       </c>
     </row>
     <row r="25">
@@ -1462,28 +1450,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3714484190940857</v>
+        <v>9.525638659795126</v>
       </c>
       <c r="F25" t="n">
-        <v>99</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="G25" t="n">
-        <v>15.06947538019221</v>
+        <v>189.0690162466089</v>
       </c>
       <c r="H25" t="n">
-        <v>16.31256556421084</v>
+        <v>189.0690162466089</v>
       </c>
       <c r="I25" t="n">
-        <v>15.06947538019221</v>
+        <v>11.71921242943418</v>
       </c>
       <c r="J25" t="n">
-        <v>17.29528846306434</v>
+        <v>104.6340857300811</v>
       </c>
       <c r="K25" t="n">
-        <v>7.111149238948735</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>8.249060784508734</v>
+        <v>1154.648960740379</v>
       </c>
     </row>
     <row r="26">
@@ -1504,28 +1492,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E26" t="n">
-        <v>1.342541608810425</v>
+        <v>1.994977712631226</v>
       </c>
       <c r="F26" t="n">
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>-21.96317396534843</v>
+        <v>-12.26324715798393</v>
       </c>
       <c r="H26" t="n">
-        <v>-9.118726815776981</v>
+        <v>-5.828972495513599</v>
       </c>
       <c r="I26" t="n">
-        <v>-21.96317396534843</v>
+        <v>-12.26324715798393</v>
       </c>
       <c r="J26" t="n">
-        <v>-9.118726815776981</v>
+        <v>-5.828972495513599</v>
       </c>
       <c r="K26" t="n">
-        <v>10.09968384419952</v>
+        <v>5.572246791414693</v>
       </c>
       <c r="L26" t="n">
-        <v>58.48174389474077</v>
+        <v>73.46024529646743</v>
       </c>
     </row>
     <row r="27">
@@ -1546,28 +1534,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E27" t="n">
-        <v>1.280003888607025</v>
+        <v>1.867767731348674</v>
       </c>
       <c r="F27" t="n">
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>22.8444824168921</v>
+        <v>41.59734965676242</v>
       </c>
       <c r="H27" t="n">
-        <v>45.21017643725565</v>
+        <v>48.24650341074641</v>
       </c>
       <c r="I27" t="n">
-        <v>22.8444824168921</v>
+        <v>41.59734965676242</v>
       </c>
       <c r="J27" t="n">
-        <v>45.21017643725565</v>
+        <v>48.24650341074641</v>
       </c>
       <c r="K27" t="n">
-        <v>14.38390154180655</v>
+        <v>11.51667212923761</v>
       </c>
       <c r="L27" t="n">
-        <v>97.90413988029553</v>
+        <v>111.195432359943</v>
       </c>
     </row>
     <row r="28">
@@ -1588,28 +1576,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E28" t="n">
-        <v>1.061874940395355</v>
+        <v>1.640861590703328</v>
       </c>
       <c r="F28" t="n">
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>-15.10741470745636</v>
+        <v>-8.638095787128815</v>
       </c>
       <c r="H28" t="n">
-        <v>17.13999463659888</v>
+        <v>5.831544285723369</v>
       </c>
       <c r="I28" t="n">
-        <v>-15.10741470745636</v>
+        <v>-8.638095787128815</v>
       </c>
       <c r="J28" t="n">
-        <v>17.13999463659888</v>
+        <v>5.831544285723369</v>
       </c>
       <c r="K28" t="n">
-        <v>15.53470091067555</v>
+        <v>13.8823299483488</v>
       </c>
       <c r="L28" t="n">
-        <v>178.0396980128686</v>
+        <v>126.5514642597826</v>
       </c>
     </row>
     <row r="29">
@@ -1630,28 +1618,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E29" t="n">
-        <v>1.003616440296173</v>
+        <v>1.627530336380005</v>
       </c>
       <c r="F29" t="n">
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>30.82283888334696</v>
+        <v>82.49122720406568</v>
       </c>
       <c r="H29" t="n">
-        <v>72.88043326639564</v>
+        <v>99.34603813998324</v>
       </c>
       <c r="I29" t="n">
-        <v>30.82283888334696</v>
+        <v>82.49122720406568</v>
       </c>
       <c r="J29" t="n">
-        <v>72.88043326639564</v>
+        <v>99.34603813998324</v>
       </c>
       <c r="K29" t="n">
-        <v>24.97590585459614</v>
+        <v>20.90248942691398</v>
       </c>
       <c r="L29" t="n">
-        <v>219.02860365313</v>
+        <v>334.8797942846932</v>
       </c>
     </row>
     <row r="30">
@@ -1672,28 +1660,30 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E30" t="n">
-        <v>0.03269515991210938</v>
+        <v>1.153596003850301</v>
       </c>
       <c r="F30" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G30" t="n">
-        <v>-21.96317396534843</v>
+        <v>25.60736840705994</v>
       </c>
       <c r="H30" t="n">
-        <v>-15.31961985730699</v>
+        <v>33.95232120936691</v>
       </c>
       <c r="I30" t="n">
-        <v>-21.96317396534843</v>
-      </c>
-      <c r="J30" t="n">
-        <v>-15.31961985730699</v>
+        <v>25.60736840705994</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K30" t="n">
-        <v>6.008245035560368</v>
+        <v>11.80154543038589</v>
       </c>
       <c r="L30" t="n">
-        <v>30.24860668372914</v>
+        <v>254.5874984323027</v>
       </c>
     </row>
     <row r="31">
@@ -1714,29 +1704,21 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E31" t="n">
-        <v>0.3541808414459229</v>
+        <v>10.18371327718099</v>
       </c>
       <c r="F31" t="n">
-        <v>19</v>
-      </c>
-      <c r="G31" t="n">
-        <v>22.8444824168921</v>
-      </c>
-      <c r="H31" t="n">
-        <v>53.89122178801244</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>0.6757756268044144</v>
+        <v>50.13618324377208</v>
       </c>
       <c r="J31" t="n">
-        <v>45.11412415595805</v>
-      </c>
-      <c r="K31" t="n">
-        <v>21.27213375768284</v>
-      </c>
-      <c r="L31" t="n">
-        <v>135.9047616161493</v>
-      </c>
+        <v>161.4826535735259</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1756,28 +1738,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E32" t="n">
-        <v>1.613664419651031</v>
+        <v>2.323824008305868</v>
       </c>
       <c r="F32" t="n">
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>-8.841290064295642</v>
+        <v>-7.873400703841429</v>
       </c>
       <c r="H32" t="n">
-        <v>-1.611070971345694</v>
+        <v>-2.774184083904669</v>
       </c>
       <c r="I32" t="n">
-        <v>-8.841290064295642</v>
+        <v>-7.873400703841429</v>
       </c>
       <c r="J32" t="n">
-        <v>-1.611070971345694</v>
+        <v>-2.774184083904669</v>
       </c>
       <c r="K32" t="n">
-        <v>6.136021695447403</v>
+        <v>4.690364302942437</v>
       </c>
       <c r="L32" t="n">
-        <v>81.77787449987885</v>
+        <v>68.62240619038347</v>
       </c>
     </row>
     <row r="33">
@@ -1798,28 +1780,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E33" t="n">
-        <v>1.550020151138306</v>
+        <v>2.154251654942831</v>
       </c>
       <c r="F33" t="n">
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>-1.050704163143443</v>
+        <v>-0.08281480268923147</v>
       </c>
       <c r="H33" t="n">
-        <v>15.08362749843662</v>
+        <v>21.83548256033676</v>
       </c>
       <c r="I33" t="n">
-        <v>-1.050704163143443</v>
+        <v>-0.08281480268923147</v>
       </c>
       <c r="J33" t="n">
-        <v>15.08362749843662</v>
+        <v>21.83548256033676</v>
       </c>
       <c r="K33" t="n">
-        <v>18.33548610329463</v>
+        <v>35.05637043329526</v>
       </c>
       <c r="L33" t="n">
-        <v>1535.57321152228</v>
+        <v>2178.176077175755</v>
       </c>
     </row>
     <row r="34">
@@ -1840,28 +1822,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E34" t="n">
-        <v>1.269640986919403</v>
+        <v>1.864962259928385</v>
       </c>
       <c r="F34" t="n">
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>-3.837456178543082</v>
+        <v>18.40332392589283</v>
       </c>
       <c r="H34" t="n">
-        <v>34.13584369839266</v>
+        <v>36.17862124687474</v>
       </c>
       <c r="I34" t="n">
-        <v>-3.837456178543082</v>
+        <v>18.40332392589283</v>
       </c>
       <c r="J34" t="n">
-        <v>34.13584369839266</v>
+        <v>36.17862124687474</v>
       </c>
       <c r="K34" t="n">
-        <v>19.94698979012258</v>
+        <v>18.01661396749524</v>
       </c>
       <c r="L34" t="n">
-        <v>486.095733203525</v>
+        <v>509.2007046910182</v>
       </c>
     </row>
     <row r="35">
@@ -1882,28 +1864,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E35" t="n">
-        <v>1.231335241794586</v>
+        <v>1.850282351175944</v>
       </c>
       <c r="F35" t="n">
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>-1.050704163143443</v>
+        <v>10.11440880163737</v>
       </c>
       <c r="H35" t="n">
-        <v>88.78119756767873</v>
+        <v>60.40349913801371</v>
       </c>
       <c r="I35" t="n">
-        <v>-1.050704163143443</v>
+        <v>10.11440880163737</v>
       </c>
       <c r="J35" t="n">
-        <v>88.78119756767873</v>
+        <v>60.40349913801371</v>
       </c>
       <c r="K35" t="n">
-        <v>39.1386972966944</v>
+        <v>46.25775095134383</v>
       </c>
       <c r="L35" t="n">
-        <v>8549.685523474815</v>
+        <v>5848.858837420192</v>
       </c>
     </row>
     <row r="36">
@@ -1924,28 +1906,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E36" t="n">
-        <v>0.03667536973953247</v>
+        <v>1.310578346252441</v>
       </c>
       <c r="F36" t="n">
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>-8.841290064295642</v>
+        <v>19.44669875577845</v>
       </c>
       <c r="H36" t="n">
-        <v>-1.022760056095839</v>
+        <v>54.48244429275157</v>
       </c>
       <c r="I36" t="n">
-        <v>-8.841290064295642</v>
+        <v>19.44669875577845</v>
       </c>
       <c r="J36" t="n">
-        <v>-1.022760056095839</v>
+        <v>54.48244429275157</v>
       </c>
       <c r="K36" t="n">
-        <v>4.913939678384262</v>
+        <v>45.06483211228916</v>
       </c>
       <c r="L36" t="n">
-        <v>88.43200428152315</v>
+        <v>716.2273140745781</v>
       </c>
     </row>
     <row r="37">
@@ -1966,29 +1948,23 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4356991195678711</v>
+        <v>9.690512975056967</v>
       </c>
       <c r="F37" t="n">
-        <v>90</v>
-      </c>
-      <c r="G37" t="n">
-        <v>-1.050704163143443</v>
-      </c>
-      <c r="H37" t="n">
-        <v>2.861817055460585</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="n">
-        <v>-1.36824095017819</v>
-      </c>
-      <c r="J37" t="n">
-        <v>8.68130175862124</v>
-      </c>
-      <c r="K37" t="n">
-        <v>3.26537734354274</v>
-      </c>
-      <c r="L37" t="n">
-        <v>372.3713444609134</v>
-      </c>
+        <v>60.09728936452053</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2008,7 +1984,7 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E38" t="n">
-        <v>1.5245334815979</v>
+        <v>2.47080667813619</v>
       </c>
       <c r="F38" t="n">
         <v>100</v>
@@ -2017,19 +1993,19 @@
         <v>9.383712874145662</v>
       </c>
       <c r="H38" t="n">
-        <v>19.87705880305042</v>
+        <v>19.64053134499601</v>
       </c>
       <c r="I38" t="n">
         <v>9.383712874145662</v>
       </c>
       <c r="J38" t="n">
-        <v>19.87705880305042</v>
+        <v>19.64053134499601</v>
       </c>
       <c r="K38" t="n">
-        <v>7.825259169072486</v>
+        <v>9.145696988089208</v>
       </c>
       <c r="L38" t="n">
-        <v>111.8250959896311</v>
+        <v>109.3044790310059</v>
       </c>
     </row>
     <row r="39">
@@ -2050,28 +2026,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E39" t="n">
-        <v>1.503237800598145</v>
+        <v>2.155666987101237</v>
       </c>
       <c r="F39" t="n">
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>26.21619167672251</v>
+        <v>41.34874866528129</v>
       </c>
       <c r="H39" t="n">
-        <v>45.3451481890507</v>
+        <v>53.77413253383622</v>
       </c>
       <c r="I39" t="n">
-        <v>26.21619167672251</v>
+        <v>41.34874866528129</v>
       </c>
       <c r="J39" t="n">
-        <v>45.3451481890507</v>
+        <v>53.77413253383622</v>
       </c>
       <c r="K39" t="n">
-        <v>10.07553664884598</v>
+        <v>16.47205155000465</v>
       </c>
       <c r="L39" t="n">
-        <v>72.96619107844286</v>
+        <v>105.1180171282564</v>
       </c>
     </row>
     <row r="40">
@@ -2092,28 +2068,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E40" t="n">
-        <v>1.212036910057068</v>
+        <v>1.869088729222615</v>
       </c>
       <c r="F40" t="n">
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>9.383712874145662</v>
+        <v>41.43632650113572</v>
       </c>
       <c r="H40" t="n">
-        <v>53.38852342948877</v>
+        <v>47.11875873930884</v>
       </c>
       <c r="I40" t="n">
-        <v>9.383712874145662</v>
+        <v>41.43632650113572</v>
       </c>
       <c r="J40" t="n">
-        <v>53.38852342948877</v>
+        <v>47.11875873930884</v>
       </c>
       <c r="K40" t="n">
-        <v>19.27559423170784</v>
+        <v>5.824129165080397</v>
       </c>
       <c r="L40" t="n">
-        <v>468.9488174407672</v>
+        <v>402.1334238511507</v>
       </c>
     </row>
     <row r="41">
@@ -2134,28 +2110,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E41" t="n">
-        <v>1.191228010654449</v>
+        <v>1.82608699798584</v>
       </c>
       <c r="F41" t="n">
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>37.10625335047498</v>
+        <v>46.08755662137803</v>
       </c>
       <c r="H41" t="n">
-        <v>71.94891164281708</v>
+        <v>61.9756856565895</v>
       </c>
       <c r="I41" t="n">
-        <v>37.10625335047498</v>
+        <v>46.08755662137803</v>
       </c>
       <c r="J41" t="n">
-        <v>71.94891164281708</v>
+        <v>61.9756856565895</v>
       </c>
       <c r="K41" t="n">
-        <v>18.98205376187818</v>
+        <v>20.23663457870682</v>
       </c>
       <c r="L41" t="n">
-        <v>174.4445590344874</v>
+        <v>136.4023212098271</v>
       </c>
     </row>
     <row r="42">
@@ -2176,28 +2152,30 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0367170786857605</v>
+        <v>1.131096998850505</v>
       </c>
       <c r="F42" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G42" t="n">
-        <v>9.383712874145662</v>
+        <v>29.0643863437334</v>
       </c>
       <c r="H42" t="n">
-        <v>21.73273904659161</v>
+        <v>44.47247064366387</v>
       </c>
       <c r="I42" t="n">
-        <v>9.383712874145662</v>
-      </c>
-      <c r="J42" t="n">
-        <v>21.73273904659161</v>
+        <v>29.0643863437334</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K42" t="n">
-        <v>7.211201687054464</v>
+        <v>21.79032178714962</v>
       </c>
       <c r="L42" t="n">
-        <v>131.600639726205</v>
+        <v>373.932559959246</v>
       </c>
     </row>
     <row r="43">
@@ -2218,28 +2196,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E43" t="n">
-        <v>0.440082221031189</v>
+        <v>10.01489273707072</v>
       </c>
       <c r="F43" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G43" t="n">
-        <v>26.21619167672251</v>
+        <v>65.2667442259319</v>
       </c>
       <c r="H43" t="n">
-        <v>33.37910592943111</v>
+        <v>71.57931473911299</v>
       </c>
       <c r="I43" t="n">
-        <v>26.21619167672251</v>
+        <v>24.30247503222626</v>
       </c>
       <c r="J43" t="n">
-        <v>33.37910592943111</v>
+        <v>55.82036817015075</v>
       </c>
       <c r="K43" t="n">
-        <v>4.433854171687641</v>
+        <v>8.927322833177191</v>
       </c>
       <c r="L43" t="n">
-        <v>27.32248200286306</v>
+        <v>173.0347550924745</v>
       </c>
     </row>
     <row r="44">
@@ -2260,7 +2238,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1525745296478271</v>
+        <v>0.3895590305328369</v>
       </c>
       <c r="F44" t="n">
         <v>100</v>
@@ -2278,7 +2256,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K44" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
@@ -2302,7 +2280,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1590132713317871</v>
+        <v>0.4008009433746338</v>
       </c>
       <c r="F45" t="n">
         <v>100</v>
@@ -2344,7 +2322,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1001806473731995</v>
+        <v>0.3364046414693196</v>
       </c>
       <c r="F46" t="n">
         <v>100</v>
@@ -2362,7 +2340,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K46" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2386,7 +2364,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1049100112915039</v>
+        <v>0.3455493450164795</v>
       </c>
       <c r="F47" t="n">
         <v>100</v>
@@ -2428,7 +2406,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E48" t="n">
-        <v>0.005615382194519043</v>
+        <v>0.8248132864634196</v>
       </c>
       <c r="F48" t="n">
         <v>100</v>
@@ -2446,7 +2424,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K48" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2470,7 +2448,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E49" t="n">
-        <v>0.0654410195350647</v>
+        <v>7.259474595387776</v>
       </c>
       <c r="F49" t="n">
         <v>100</v>
@@ -2512,28 +2490,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E50" t="n">
-        <v>2.709939367771149</v>
+        <v>3.528955618540446</v>
       </c>
       <c r="F50" t="n">
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>13.02451543344857</v>
+        <v>30.27537186972479</v>
       </c>
       <c r="H50" t="n">
-        <v>39.04521578619128</v>
+        <v>47.59417951446528</v>
       </c>
       <c r="I50" t="n">
-        <v>13.02451543344857</v>
+        <v>30.27537186972479</v>
       </c>
       <c r="J50" t="n">
-        <v>39.04521578619128</v>
+        <v>47.59417951446528</v>
       </c>
       <c r="K50" t="n">
-        <v>13.16898458889659</v>
+        <v>15.00319976160127</v>
       </c>
       <c r="L50" t="n">
-        <v>199.7824831618559</v>
+        <v>265.4199632812253</v>
       </c>
     </row>
     <row r="51">
@@ -2554,28 +2532,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E51" t="n">
-        <v>2.690952260494232</v>
+        <v>3.546395381291708</v>
       </c>
       <c r="F51" t="n">
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>34.00523196803706</v>
+        <v>37.60618409062889</v>
       </c>
       <c r="H51" t="n">
-        <v>69.58762460982115</v>
+        <v>68.09142119442838</v>
       </c>
       <c r="I51" t="n">
-        <v>34.00523196803706</v>
+        <v>37.60618409062889</v>
       </c>
       <c r="J51" t="n">
-        <v>69.58762460982115</v>
+        <v>68.09142119442838</v>
       </c>
       <c r="K51" t="n">
-        <v>22.08933507509494</v>
+        <v>29.11079206897703</v>
       </c>
       <c r="L51" t="n">
-        <v>198.1510758155493</v>
+        <v>191.7405299686475</v>
       </c>
     </row>
     <row r="52">
@@ -2596,28 +2574,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E52" t="n">
-        <v>2.171270558834076</v>
+        <v>3.003234624862671</v>
       </c>
       <c r="F52" t="n">
         <v>100</v>
       </c>
       <c r="G52" t="n">
-        <v>35.51153901902885</v>
+        <v>89.20867358878883</v>
       </c>
       <c r="H52" t="n">
-        <v>107.4057204858784</v>
+        <v>94.29226409484549</v>
       </c>
       <c r="I52" t="n">
-        <v>35.51153901902885</v>
+        <v>89.20867358878883</v>
       </c>
       <c r="J52" t="n">
-        <v>107.4057204858784</v>
+        <v>94.29226409484549</v>
       </c>
       <c r="K52" t="n">
-        <v>26.86237323746136</v>
+        <v>4.922387598102157</v>
       </c>
       <c r="L52" t="n">
-        <v>724.6427364971073</v>
+        <v>623.9598630494249</v>
       </c>
     </row>
     <row r="53">
@@ -2638,28 +2616,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E53" t="n">
-        <v>2.09732195854187</v>
+        <v>2.980710983276367</v>
       </c>
       <c r="F53" t="n">
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>46.64785562333473</v>
+        <v>152.3677802137354</v>
       </c>
       <c r="H53" t="n">
-        <v>156.0186197263497</v>
+        <v>167.2062146222932</v>
       </c>
       <c r="I53" t="n">
-        <v>46.64785562333473</v>
+        <v>152.3677802137354</v>
       </c>
       <c r="J53" t="n">
-        <v>156.0186197263497</v>
+        <v>167.2062146222932</v>
       </c>
       <c r="K53" t="n">
-        <v>36.81240779489718</v>
+        <v>12.88274822662302</v>
       </c>
       <c r="L53" t="n">
-        <v>568.4682740572111</v>
+        <v>616.401990328126</v>
       </c>
     </row>
     <row r="54">
@@ -2680,29 +2658,25 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E54" t="n">
-        <v>0.05418124914169312</v>
+        <v>1.320327361424764</v>
       </c>
       <c r="F54" t="n">
-        <v>100</v>
-      </c>
-      <c r="G54" t="n">
-        <v>23.00601802836938</v>
-      </c>
-      <c r="H54" t="n">
-        <v>41.22391773750977</v>
-      </c>
-      <c r="I54" t="n">
-        <v>23.00601802836938</v>
-      </c>
-      <c r="J54" t="n">
-        <v>41.22391773750977</v>
-      </c>
-      <c r="K54" t="n">
-        <v>9.54360599909379</v>
-      </c>
-      <c r="L54" t="n">
-        <v>216.510183800325</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2722,29 +2696,25 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E55" t="n">
-        <v>0.6366844487190246</v>
+        <v>9.390654961268107</v>
       </c>
       <c r="F55" t="n">
-        <v>92</v>
-      </c>
-      <c r="G55" t="n">
-        <v>29.72035854397576</v>
-      </c>
-      <c r="H55" t="n">
-        <v>59.51424635828349</v>
-      </c>
-      <c r="I55" t="n">
-        <v>29.72035854397576</v>
-      </c>
-      <c r="J55" t="n">
-        <v>63.16416136922818</v>
-      </c>
-      <c r="K55" t="n">
-        <v>10.51583334519222</v>
-      </c>
-      <c r="L55" t="n">
-        <v>154.9912671623161</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2764,7 +2734,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E56" t="n">
-        <v>0.207843120098114</v>
+        <v>0.414016326268514</v>
       </c>
       <c r="F56" t="n">
         <v>100</v>
@@ -2782,7 +2752,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K56" t="n">
-        <v>3.570611593983174e-15</v>
+        <v>0</v>
       </c>
       <c r="L56" t="n">
         <v>0</v>
@@ -2806,7 +2776,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E57" t="n">
-        <v>0.2078845810890198</v>
+        <v>0.4078160127003987</v>
       </c>
       <c r="F57" t="n">
         <v>100</v>
@@ -2824,7 +2794,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K57" t="n">
-        <v>7.141223187966347e-15</v>
+        <v>0</v>
       </c>
       <c r="L57" t="n">
         <v>0</v>
@@ -2848,7 +2818,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E58" t="n">
-        <v>0.1452521872520447</v>
+        <v>0.3458969593048096</v>
       </c>
       <c r="F58" t="n">
         <v>100</v>
@@ -2866,7 +2836,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K58" t="n">
-        <v>3.570611593983174e-15</v>
+        <v>0</v>
       </c>
       <c r="L58" t="n">
         <v>0</v>
@@ -2890,7 +2860,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E59" t="n">
-        <v>0.1462344884872437</v>
+        <v>0.3465774059295654</v>
       </c>
       <c r="F59" t="n">
         <v>100</v>
@@ -2908,7 +2878,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K59" t="n">
-        <v>7.141223187966347e-15</v>
+        <v>0</v>
       </c>
       <c r="L59" t="n">
         <v>0</v>
@@ -2932,7 +2902,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E60" t="n">
-        <v>0.007531299591064453</v>
+        <v>0.8312124411265055</v>
       </c>
       <c r="F60" t="n">
         <v>100</v>
@@ -2941,19 +2911,19 @@
         <v>13.90826436045291</v>
       </c>
       <c r="H60" t="n">
-        <v>13.90826436045291</v>
+        <v>18.68256530384832</v>
       </c>
       <c r="I60" t="n">
         <v>13.90826436045291</v>
       </c>
       <c r="J60" t="n">
-        <v>13.90826436045291</v>
+        <v>18.68256530384832</v>
       </c>
       <c r="K60" t="n">
-        <v>3.570611593983174e-15</v>
+        <v>5.962790698516184</v>
       </c>
       <c r="L60" t="n">
-        <v>0</v>
+        <v>34.32707935125806</v>
       </c>
     </row>
     <row r="61">
@@ -2974,7 +2944,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E61" t="n">
-        <v>0.08962120056152344</v>
+        <v>7.960235754648845</v>
       </c>
       <c r="F61" t="n">
         <v>100</v>
@@ -2992,7 +2962,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K61" t="n">
-        <v>7.141223187966347e-15</v>
+        <v>0</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
@@ -3016,7 +2986,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E62" t="n">
-        <v>0.32591224193573</v>
+        <v>0.5718727111816406</v>
       </c>
       <c r="F62" t="n">
         <v>100</v>
@@ -3034,7 +3004,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="K62" t="n">
-        <v>7.141223187966347e-15</v>
+        <v>4.351167857633658e-15</v>
       </c>
       <c r="L62" t="n">
         <v>-1.431247886831891e-14</v>
@@ -3058,7 +3028,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E63" t="n">
-        <v>0.3320509099960327</v>
+        <v>0.5649979909261068</v>
       </c>
       <c r="F63" t="n">
         <v>100</v>
@@ -3067,19 +3037,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H63" t="n">
-        <v>49.44269207730557</v>
+        <v>48.65032644645115</v>
       </c>
       <c r="I63" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J63" t="n">
-        <v>49.44269207730557</v>
+        <v>48.65032644645115</v>
       </c>
       <c r="K63" t="n">
-        <v>3.185952253599189</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>1.62869540397961</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -3100,7 +3070,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E64" t="n">
-        <v>0.2388650012016297</v>
+        <v>0.4589842955271403</v>
       </c>
       <c r="F64" t="n">
         <v>100</v>
@@ -3109,19 +3079,19 @@
         <v>24.82249030015713</v>
       </c>
       <c r="H64" t="n">
-        <v>24.84569542949007</v>
+        <v>24.82249030015713</v>
       </c>
       <c r="I64" t="n">
         <v>24.82249030015713</v>
       </c>
       <c r="J64" t="n">
-        <v>24.84569542949007</v>
+        <v>24.82249030015713</v>
       </c>
       <c r="K64" t="n">
-        <v>0.2320512933293372</v>
+        <v>4.351167857633658e-15</v>
       </c>
       <c r="L64" t="n">
-        <v>0.0934842920768082</v>
+        <v>-1.431247886831891e-14</v>
       </c>
     </row>
     <row r="65">
@@ -3142,7 +3112,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E65" t="n">
-        <v>0.2409717726707458</v>
+        <v>0.520045280456543</v>
       </c>
       <c r="F65" t="n">
         <v>100</v>
@@ -3151,19 +3121,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H65" t="n">
-        <v>49.47614872262835</v>
+        <v>51.20269814256776</v>
       </c>
       <c r="I65" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J65" t="n">
-        <v>49.47614872262835</v>
+        <v>51.20269814256776</v>
       </c>
       <c r="K65" t="n">
-        <v>2.519496764162747</v>
+        <v>4.420837457474725</v>
       </c>
       <c r="L65" t="n">
-        <v>1.697465025411863</v>
+        <v>5.246360882955188</v>
       </c>
     </row>
     <row r="66">
@@ -3184,7 +3154,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E66" t="n">
-        <v>0.008814167976379395</v>
+        <v>0.8588020006815592</v>
       </c>
       <c r="F66" t="n">
         <v>100</v>
@@ -3193,19 +3163,19 @@
         <v>24.82249030015713</v>
       </c>
       <c r="H66" t="n">
-        <v>24.82249030015713</v>
+        <v>26.99605343621456</v>
       </c>
       <c r="I66" t="n">
         <v>24.82249030015713</v>
       </c>
       <c r="J66" t="n">
-        <v>24.82249030015713</v>
+        <v>26.99605343621456</v>
       </c>
       <c r="K66" t="n">
-        <v>7.141223187966347e-15</v>
+        <v>3.764721785110208</v>
       </c>
       <c r="L66" t="n">
-        <v>-1.431247886831891e-14</v>
+        <v>8.756426570317439</v>
       </c>
     </row>
     <row r="67">
@@ -3226,7 +3196,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E67" t="n">
-        <v>0.1046896910667419</v>
+        <v>7.666666984558105</v>
       </c>
       <c r="F67" t="n">
         <v>100</v>
@@ -3244,7 +3214,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="K67" t="n">
-        <v>2.142366956389904e-14</v>
+        <v>0</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
@@ -3268,7 +3238,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E68" t="n">
-        <v>0.09339206218719483</v>
+        <v>0.1903249422709147</v>
       </c>
       <c r="F68" t="n">
         <v>100</v>
@@ -3286,7 +3256,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K68" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
@@ -3310,7 +3280,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E69" t="n">
-        <v>0.09400078773498535</v>
+        <v>0.2013113498687744</v>
       </c>
       <c r="F69" t="n">
         <v>100</v>
@@ -3328,7 +3298,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K69" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L69" t="n">
         <v>0</v>
@@ -3352,7 +3322,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E70" t="n">
-        <v>0.05075753211975097</v>
+        <v>0.1571446259816488</v>
       </c>
       <c r="F70" t="n">
         <v>100</v>
@@ -3370,7 +3340,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K70" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
@@ -3394,7 +3364,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E71" t="n">
-        <v>0.05101221084594727</v>
+        <v>0.1580249468485514</v>
       </c>
       <c r="F71" t="n">
         <v>100</v>
@@ -3412,7 +3382,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K71" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
@@ -3436,7 +3406,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E72" t="n">
-        <v>0.002319879531860352</v>
+        <v>0.9425457318623861</v>
       </c>
       <c r="F72" t="n">
         <v>100</v>
@@ -3454,7 +3424,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K72" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L72" t="n">
         <v>0</v>
@@ -3478,7 +3448,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E73" t="n">
-        <v>0.0264729905128479</v>
+        <v>7.38074803352356</v>
       </c>
       <c r="F73" t="n">
         <v>100</v>
@@ -3496,7 +3466,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K73" t="n">
-        <v>1.785305796991587e-15</v>
+        <v>0</v>
       </c>
       <c r="L73" t="n">
         <v>0</v>
@@ -3520,7 +3490,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E74" t="n">
-        <v>0.358566062450409</v>
+        <v>0.6762966314951578</v>
       </c>
       <c r="F74" t="n">
         <v>100</v>
@@ -3529,19 +3499,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H74" t="n">
-        <v>31.06813056819737</v>
+        <v>30.95896547744237</v>
       </c>
       <c r="I74" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J74" t="n">
-        <v>31.06813056819737</v>
+        <v>30.95896547744237</v>
       </c>
       <c r="K74" t="n">
-        <v>0.8576863244551524</v>
+        <v>4.351167857633658e-15</v>
       </c>
       <c r="L74" t="n">
-        <v>0.3526122048055629</v>
+        <v>-1.147555683470468e-14</v>
       </c>
     </row>
     <row r="75">
@@ -3562,7 +3532,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E75" t="n">
-        <v>0.3596773505210876</v>
+        <v>0.658511241277059</v>
       </c>
       <c r="F75" t="n">
         <v>100</v>
@@ -3571,19 +3541,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H75" t="n">
-        <v>40.19866139860349</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="I75" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J75" t="n">
-        <v>40.19866139860349</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="K75" t="n">
-        <v>3.298033702524826</v>
+        <v>0</v>
       </c>
       <c r="L75" t="n">
-        <v>5.213246604302893</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -3604,7 +3574,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E76" t="n">
-        <v>0.2759222602844238</v>
+        <v>0.5730956395467123</v>
       </c>
       <c r="F76" t="n">
         <v>100</v>
@@ -3613,19 +3583,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H76" t="n">
-        <v>31.68225774080297</v>
+        <v>31.88291438831978</v>
       </c>
       <c r="I76" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J76" t="n">
-        <v>31.68225774080297</v>
+        <v>31.88291438831978</v>
       </c>
       <c r="K76" t="n">
-        <v>1.669414454809327</v>
+        <v>1.600326457237609</v>
       </c>
       <c r="L76" t="n">
-        <v>2.336293387734841</v>
+        <v>2.984430831678232</v>
       </c>
     </row>
     <row r="77">
@@ -3646,7 +3616,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E77" t="n">
-        <v>0.2704894804954529</v>
+        <v>0.5648903846740723</v>
       </c>
       <c r="F77" t="n">
         <v>100</v>
@@ -3655,19 +3625,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H77" t="n">
-        <v>42.65164089282676</v>
+        <v>38.84450275393277</v>
       </c>
       <c r="I77" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J77" t="n">
-        <v>42.65164089282676</v>
+        <v>38.84450275393277</v>
       </c>
       <c r="K77" t="n">
-        <v>6.570842334189233</v>
+        <v>1.104456699297865</v>
       </c>
       <c r="L77" t="n">
-        <v>11.63350855984097</v>
+        <v>1.668963723578947</v>
       </c>
     </row>
     <row r="78">
@@ -3688,28 +3658,28 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E78" t="n">
-        <v>0.01343673944473267</v>
+        <v>0.9480663140614828</v>
       </c>
       <c r="F78" t="n">
         <v>100</v>
       </c>
       <c r="G78" t="n">
-        <v>30.95896547744237</v>
+        <v>40.9786911139171</v>
       </c>
       <c r="H78" t="n">
-        <v>30.97669393536907</v>
+        <v>60.30925492758055</v>
       </c>
       <c r="I78" t="n">
-        <v>30.95896547744237</v>
+        <v>40.9786911139171</v>
       </c>
       <c r="J78" t="n">
-        <v>30.97669393536907</v>
+        <v>60.30925492758055</v>
       </c>
       <c r="K78" t="n">
-        <v>0.1772845792669813</v>
+        <v>18.0859020148175</v>
       </c>
       <c r="L78" t="n">
-        <v>0.05726437448181175</v>
+        <v>94.80384437110368</v>
       </c>
     </row>
     <row r="79">
@@ -3730,28 +3700,28 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E79" t="n">
-        <v>0.1610432124137878</v>
+        <v>8.634498596191406</v>
       </c>
       <c r="F79" t="n">
         <v>100</v>
       </c>
       <c r="G79" t="n">
-        <v>38.20684438128487</v>
+        <v>46.35150672415288</v>
       </c>
       <c r="H79" t="n">
-        <v>38.20684438128487</v>
+        <v>65.20360019650697</v>
       </c>
       <c r="I79" t="n">
-        <v>38.20684438128487</v>
+        <v>46.35150672415288</v>
       </c>
       <c r="J79" t="n">
-        <v>38.20684438128487</v>
+        <v>65.20360019650697</v>
       </c>
       <c r="K79" t="n">
-        <v>1.428244637593269e-14</v>
+        <v>16.57616084249375</v>
       </c>
       <c r="L79" t="n">
-        <v>0</v>
+        <v>70.65947542227831</v>
       </c>
     </row>
     <row r="80">
@@ -3772,7 +3742,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E80" t="n">
-        <v>0.532923948764801</v>
+        <v>0.8686463038126627</v>
       </c>
       <c r="F80" t="n">
         <v>100</v>
@@ -3781,19 +3751,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H80" t="n">
-        <v>1.482212030891633</v>
+        <v>1.273146143170434</v>
       </c>
       <c r="I80" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J80" t="n">
-        <v>1.482212030891633</v>
+        <v>1.273146143170434</v>
       </c>
       <c r="K80" t="n">
-        <v>1.288251998500642</v>
+        <v>0.4275746877548631</v>
       </c>
       <c r="L80" t="n">
-        <v>44.42488210874114</v>
+        <v>24.05376410551598</v>
       </c>
     </row>
     <row r="81">
@@ -3814,28 +3784,28 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E81" t="n">
-        <v>0.5244971489906312</v>
+        <v>0.9065333207448324</v>
       </c>
       <c r="F81" t="n">
         <v>100</v>
       </c>
       <c r="G81" t="n">
-        <v>18.17186472076723</v>
+        <v>19.29718019360264</v>
       </c>
       <c r="H81" t="n">
-        <v>21.56787090188577</v>
+        <v>19.83334689708312</v>
       </c>
       <c r="I81" t="n">
-        <v>18.17186472076723</v>
+        <v>19.29718019360264</v>
       </c>
       <c r="J81" t="n">
-        <v>21.56787090188577</v>
+        <v>19.83334689708312</v>
       </c>
       <c r="K81" t="n">
-        <v>3.977812161828188</v>
+        <v>0.5417048304786438</v>
       </c>
       <c r="L81" t="n">
-        <v>18.68826470646959</v>
+        <v>9.143157303042813</v>
       </c>
     </row>
     <row r="82">
@@ -3856,28 +3826,28 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E82" t="n">
-        <v>0.3955034112930298</v>
+        <v>0.7165652910868326</v>
       </c>
       <c r="F82" t="n">
         <v>100</v>
       </c>
       <c r="G82" t="n">
-        <v>1.026285782096494</v>
+        <v>1.766866865318315</v>
       </c>
       <c r="H82" t="n">
-        <v>4.778366316858686</v>
+        <v>3.514450942422638</v>
       </c>
       <c r="I82" t="n">
-        <v>1.026285782096494</v>
+        <v>1.766866865318315</v>
       </c>
       <c r="J82" t="n">
-        <v>4.778366316858686</v>
+        <v>3.514450942422638</v>
       </c>
       <c r="K82" t="n">
-        <v>5.270840478941794</v>
+        <v>1.558092636885859</v>
       </c>
       <c r="L82" t="n">
-        <v>365.5980234957023</v>
+        <v>242.4436939234729</v>
       </c>
     </row>
     <row r="83">
@@ -3898,28 +3868,28 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E83" t="n">
-        <v>0.3907591199874878</v>
+        <v>0.7029693921407064</v>
       </c>
       <c r="F83" t="n">
         <v>100</v>
       </c>
       <c r="G83" t="n">
-        <v>18.17186472076723</v>
+        <v>28.82591742481698</v>
       </c>
       <c r="H83" t="n">
-        <v>24.33509387540884</v>
+        <v>29.82313964390611</v>
       </c>
       <c r="I83" t="n">
-        <v>18.17186472076723</v>
+        <v>28.82591742481698</v>
       </c>
       <c r="J83" t="n">
-        <v>24.33509387540884</v>
+        <v>29.82313964390611</v>
       </c>
       <c r="K83" t="n">
-        <v>5.927749011974221</v>
+        <v>1.727239549898954</v>
       </c>
       <c r="L83" t="n">
-        <v>33.91632751700012</v>
+        <v>64.11711237220213</v>
       </c>
     </row>
     <row r="84">
@@ -3940,7 +3910,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E84" t="n">
-        <v>0.01594146013259888</v>
+        <v>0.9585286776224772</v>
       </c>
       <c r="F84" t="n">
         <v>100</v>
@@ -3949,19 +3919,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H84" t="n">
-        <v>1.04109740376093</v>
+        <v>11.80789107907135</v>
       </c>
       <c r="I84" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J84" t="n">
-        <v>1.04109740376093</v>
+        <v>11.80789107907135</v>
       </c>
       <c r="K84" t="n">
-        <v>0.1042036791464984</v>
+        <v>18.03672752721468</v>
       </c>
       <c r="L84" t="n">
-        <v>1.443225846330945</v>
+        <v>1050.546103732454</v>
       </c>
     </row>
     <row r="85">
@@ -3982,7 +3952,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E85" t="n">
-        <v>0.1967201089859009</v>
+        <v>7.935341676076253</v>
       </c>
       <c r="F85" t="n">
         <v>100</v>
@@ -3991,19 +3961,19 @@
         <v>18.17186472076723</v>
       </c>
       <c r="H85" t="n">
-        <v>18.17186472076723</v>
+        <v>24.01530249686201</v>
       </c>
       <c r="I85" t="n">
         <v>18.17186472076723</v>
       </c>
       <c r="J85" t="n">
-        <v>18.17186472076723</v>
+        <v>24.01530249686201</v>
       </c>
       <c r="K85" t="n">
-        <v>3.570611593983174e-15</v>
+        <v>10.12113111906344</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>32.15651154070478</v>
       </c>
     </row>
     <row r="86">
@@ -4024,7 +3994,7 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E86" t="n">
-        <v>2.254394590854645</v>
+        <v>1.030043999354045</v>
       </c>
       <c r="F86" t="n">
         <v>100</v>
@@ -4033,19 +4003,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="H86" t="n">
-        <v>45.73137409085769</v>
+        <v>45.01044323572248</v>
       </c>
       <c r="I86" t="n">
         <v>44.28900565726017</v>
       </c>
       <c r="J86" t="n">
-        <v>45.73137409085769</v>
+        <v>45.01044323572248</v>
       </c>
       <c r="K86" t="n">
-        <v>2.844380686534761</v>
+        <v>1.249566540386187</v>
       </c>
       <c r="L86" t="n">
-        <v>3.256718935529046</v>
+        <v>1.628931532230169</v>
       </c>
     </row>
     <row r="87">
@@ -4066,7 +4036,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E87" t="n">
-        <v>0.6372906613349915</v>
+        <v>1.023363351821899</v>
       </c>
       <c r="F87" t="n">
         <v>100</v>
@@ -4075,19 +4045,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H87" t="n">
-        <v>52.66253699384136</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="I87" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J87" t="n">
-        <v>52.66253699384136</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="K87" t="n">
-        <v>3.69088760159136</v>
+        <v>0</v>
       </c>
       <c r="L87" t="n">
-        <v>4.20668198343103</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -4108,28 +4078,28 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E88" t="n">
-        <v>0.4856209206581116</v>
+        <v>0.8899719715118408</v>
       </c>
       <c r="F88" t="n">
         <v>100</v>
       </c>
       <c r="G88" t="n">
-        <v>44.28900565726017</v>
+        <v>51.67833774745558</v>
       </c>
       <c r="H88" t="n">
-        <v>50.99879962602679</v>
+        <v>52.41137127350223</v>
       </c>
       <c r="I88" t="n">
-        <v>44.28900565726017</v>
+        <v>51.67833774745558</v>
       </c>
       <c r="J88" t="n">
-        <v>50.99879962602679</v>
+        <v>52.41137127350223</v>
       </c>
       <c r="K88" t="n">
-        <v>4.689307717249227</v>
+        <v>0.6348256553820762</v>
       </c>
       <c r="L88" t="n">
-        <v>15.15002170220705</v>
+        <v>18.33946257249192</v>
       </c>
     </row>
     <row r="89">
@@ -4150,28 +4120,28 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E89" t="n">
-        <v>0.4766767072677612</v>
+        <v>0.8668596744537354</v>
       </c>
       <c r="F89" t="n">
         <v>100</v>
       </c>
       <c r="G89" t="n">
-        <v>50.53662202027962</v>
+        <v>51.50656411814308</v>
       </c>
       <c r="H89" t="n">
-        <v>57.61343046341774</v>
+        <v>52.9684330467984</v>
       </c>
       <c r="I89" t="n">
-        <v>50.53662202027962</v>
+        <v>51.50656411814308</v>
       </c>
       <c r="J89" t="n">
-        <v>57.61343046341774</v>
+        <v>52.9684330467984</v>
       </c>
       <c r="K89" t="n">
-        <v>4.991667725708012</v>
+        <v>2.419869637688528</v>
       </c>
       <c r="L89" t="n">
-        <v>14.00332701362253</v>
+        <v>4.811977788192747</v>
       </c>
     </row>
     <row r="90">
@@ -4192,28 +4162,30 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E90" t="n">
-        <v>0.01850558996200562</v>
+        <v>0.8682553768157959</v>
       </c>
       <c r="F90" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G90" t="n">
-        <v>44.28900565726017</v>
+        <v>66.67915660867422</v>
       </c>
       <c r="H90" t="n">
-        <v>45.44935890994204</v>
+        <v>67.59736162089149</v>
       </c>
       <c r="I90" t="n">
-        <v>44.28900565726017</v>
-      </c>
-      <c r="J90" t="n">
-        <v>45.44935890994204</v>
+        <v>66.67915660867422</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K90" t="n">
-        <v>1.704561875361765</v>
+        <v>1.298537981316628</v>
       </c>
       <c r="L90" t="n">
-        <v>2.61995778740555</v>
+        <v>52.62786016016697</v>
       </c>
     </row>
     <row r="91">
@@ -4234,28 +4206,28 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E91" t="n">
-        <v>0.2175374698638916</v>
+        <v>8.402032295862833</v>
       </c>
       <c r="F91" t="n">
         <v>100</v>
       </c>
       <c r="G91" t="n">
-        <v>50.53662202027962</v>
+        <v>51.637093647164</v>
       </c>
       <c r="H91" t="n">
-        <v>50.53662202027962</v>
+        <v>72.51902409364122</v>
       </c>
       <c r="I91" t="n">
-        <v>50.53662202027962</v>
+        <v>51.637093647164</v>
       </c>
       <c r="J91" t="n">
-        <v>50.53662202027962</v>
+        <v>72.51902409364122</v>
       </c>
       <c r="K91" t="n">
-        <v>7.141223187966347e-15</v>
+        <v>18.21296541760399</v>
       </c>
       <c r="L91" t="n">
-        <v>1.405995706390842e-14</v>
+        <v>43.4979648314056</v>
       </c>
     </row>
     <row r="92">
@@ -4276,7 +4248,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E92" t="n">
-        <v>0.6990683484077453</v>
+        <v>1.112603346506755</v>
       </c>
       <c r="F92" t="n">
         <v>100</v>
@@ -4285,19 +4257,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H92" t="n">
-        <v>48.17965504840349</v>
+        <v>47.99866847890613</v>
       </c>
       <c r="I92" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J92" t="n">
-        <v>48.17965504840349</v>
+        <v>47.99866847890613</v>
       </c>
       <c r="K92" t="n">
-        <v>2.660085952667409</v>
+        <v>1.149830251536129</v>
       </c>
       <c r="L92" t="n">
-        <v>1.784820323934757</v>
+        <v>1.402466290083181</v>
       </c>
     </row>
     <row r="93">
@@ -4318,28 +4290,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E93" t="n">
-        <v>0.6919659090042114</v>
+        <v>1.096572001775106</v>
       </c>
       <c r="F93" t="n">
         <v>100</v>
       </c>
       <c r="G93" t="n">
-        <v>54.33806753213224</v>
+        <v>54.90718637611567</v>
       </c>
       <c r="H93" t="n">
-        <v>58.47879925218077</v>
+        <v>54.9175958715221</v>
       </c>
       <c r="I93" t="n">
-        <v>54.33806753213224</v>
+        <v>54.90718637611567</v>
       </c>
       <c r="J93" t="n">
-        <v>58.47879925218077</v>
+        <v>54.9175958715221</v>
       </c>
       <c r="K93" t="n">
-        <v>5.012389607812267</v>
+        <v>0.009014887462542011</v>
       </c>
       <c r="L93" t="n">
-        <v>7.620314648841625</v>
+        <v>1.066523646699732</v>
       </c>
     </row>
     <row r="94">
@@ -4360,7 +4332,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E94" t="n">
-        <v>0.5555941009521485</v>
+        <v>0.947083314259847</v>
       </c>
       <c r="F94" t="n">
         <v>100</v>
@@ -4369,19 +4341,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H94" t="n">
-        <v>55.16478562210857</v>
+        <v>56.24888602612805</v>
       </c>
       <c r="I94" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J94" t="n">
-        <v>55.16478562210857</v>
+        <v>56.24888602612805</v>
       </c>
       <c r="K94" t="n">
-        <v>8.426754492484168</v>
+        <v>15.30669546393318</v>
       </c>
       <c r="L94" t="n">
-        <v>16.54167691972217</v>
+        <v>18.83195825787974</v>
       </c>
     </row>
     <row r="95">
@@ -4402,28 +4374,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E95" t="n">
-        <v>0.5420695209503174</v>
+        <v>0.9631433486938477</v>
       </c>
       <c r="F95" t="n">
         <v>100</v>
       </c>
       <c r="G95" t="n">
-        <v>54.33806753213224</v>
+        <v>64.86384032096603</v>
       </c>
       <c r="H95" t="n">
-        <v>66.54862656309342</v>
+        <v>68.87375783903298</v>
       </c>
       <c r="I95" t="n">
-        <v>54.33806753213224</v>
+        <v>64.86384032096603</v>
       </c>
       <c r="J95" t="n">
-        <v>66.54862656309342</v>
+        <v>68.87375783903298</v>
       </c>
       <c r="K95" t="n">
-        <v>8.932622953389657</v>
+        <v>6.82955042618832</v>
       </c>
       <c r="L95" t="n">
-        <v>22.47146353473206</v>
+        <v>26.7504734103862</v>
       </c>
     </row>
     <row r="96">
@@ -4444,28 +4416,28 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E96" t="n">
-        <v>0.02307023048400879</v>
+        <v>1.069497346878052</v>
       </c>
       <c r="F96" t="n">
         <v>100</v>
       </c>
       <c r="G96" t="n">
-        <v>47.33481367365937</v>
+        <v>54.3724651017605</v>
       </c>
       <c r="H96" t="n">
-        <v>49.06946089259275</v>
+        <v>57.81332455030586</v>
       </c>
       <c r="I96" t="n">
-        <v>47.33481367365937</v>
+        <v>54.3724651017605</v>
       </c>
       <c r="J96" t="n">
-        <v>49.06946089259275</v>
+        <v>57.81332455030586</v>
       </c>
       <c r="K96" t="n">
-        <v>2.270751167183505</v>
+        <v>3.014036392617975</v>
       </c>
       <c r="L96" t="n">
-        <v>3.664633034984714</v>
+        <v>22.1370067048083</v>
       </c>
     </row>
     <row r="97">
@@ -4486,28 +4458,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E97" t="n">
-        <v>0.2737784099578857</v>
+        <v>19.92718005180359</v>
       </c>
       <c r="F97" t="n">
         <v>100</v>
       </c>
       <c r="G97" t="n">
-        <v>54.33806753213224</v>
+        <v>76.34124740580116</v>
       </c>
       <c r="H97" t="n">
-        <v>54.34114189273103</v>
+        <v>115.5801339057931</v>
       </c>
       <c r="I97" t="n">
-        <v>54.33806753213224</v>
+        <v>76.34124740580116</v>
       </c>
       <c r="J97" t="n">
-        <v>54.34114189273103</v>
+        <v>115.5801339057931</v>
       </c>
       <c r="K97" t="n">
-        <v>0.02162894061667199</v>
+        <v>34.00234192437474</v>
       </c>
       <c r="L97" t="n">
-        <v>0.005657839408753304</v>
+        <v>112.705639260075</v>
       </c>
     </row>
     <row r="98">
@@ -4528,28 +4500,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8661245393753052</v>
+        <v>1.290271997451782</v>
       </c>
       <c r="F98" t="n">
         <v>100</v>
       </c>
       <c r="G98" t="n">
-        <v>0.1017009531136672</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="H98" t="n">
-        <v>2.085010959758808</v>
+        <v>1.591327590959869</v>
       </c>
       <c r="I98" t="n">
-        <v>0.1017009531136672</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="J98" t="n">
-        <v>2.085010959758808</v>
+        <v>1.591327590959869</v>
       </c>
       <c r="K98" t="n">
-        <v>2.912846636412049</v>
+        <v>0.4933607090175952</v>
       </c>
       <c r="L98" t="n">
-        <v>1950.139055657101</v>
+        <v>1464.712563884533</v>
       </c>
     </row>
     <row r="99">
@@ -4570,7 +4542,7 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E99" t="n">
-        <v>0.8166107010841369</v>
+        <v>1.27419638633728</v>
       </c>
       <c r="F99" t="n">
         <v>100</v>
@@ -4579,19 +4551,19 @@
         <v>10.54487657926557</v>
       </c>
       <c r="H99" t="n">
-        <v>19.80986964450671</v>
+        <v>22.89634351331695</v>
       </c>
       <c r="I99" t="n">
         <v>10.54487657926557</v>
       </c>
       <c r="J99" t="n">
-        <v>19.80986964450671</v>
+        <v>22.89634351331695</v>
       </c>
       <c r="K99" t="n">
-        <v>6.532783985572673</v>
+        <v>21.39336827778398</v>
       </c>
       <c r="L99" t="n">
-        <v>87.86250835271922</v>
+        <v>117.1323992386797</v>
       </c>
     </row>
     <row r="100">
@@ -4612,28 +4584,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E100" t="n">
-        <v>0.6621059823036194</v>
+        <v>1.166152000427246</v>
       </c>
       <c r="F100" t="n">
         <v>100</v>
       </c>
       <c r="G100" t="n">
-        <v>0.1017009531136672</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="H100" t="n">
-        <v>10.41332765203487</v>
+        <v>6.615765352849009</v>
       </c>
       <c r="I100" t="n">
-        <v>0.1017009531136672</v>
+        <v>1.306485652800976</v>
       </c>
       <c r="J100" t="n">
-        <v>10.41332765203487</v>
+        <v>6.615765352849009</v>
       </c>
       <c r="K100" t="n">
-        <v>8.134361461979164</v>
+        <v>5.222769989219668</v>
       </c>
       <c r="L100" t="n">
-        <v>10139.1642685947</v>
+        <v>6405.116373348855</v>
       </c>
     </row>
     <row r="101">
@@ -4654,28 +4626,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E101" t="n">
-        <v>0.6329903674125671</v>
+        <v>1.067466656366984</v>
       </c>
       <c r="F101" t="n">
         <v>100</v>
       </c>
       <c r="G101" t="n">
-        <v>10.54487657926557</v>
+        <v>21.6799181202689</v>
       </c>
       <c r="H101" t="n">
-        <v>31.96446820773227</v>
+        <v>53.77892825703592</v>
       </c>
       <c r="I101" t="n">
-        <v>10.54487657926557</v>
+        <v>21.6799181202689</v>
       </c>
       <c r="J101" t="n">
-        <v>31.96446820773227</v>
+        <v>53.77892825703592</v>
       </c>
       <c r="K101" t="n">
-        <v>14.36505863199191</v>
+        <v>28.34536542287317</v>
       </c>
       <c r="L101" t="n">
-        <v>203.1279500282074</v>
+        <v>410.00054721154</v>
       </c>
     </row>
     <row r="102">
@@ -4696,28 +4668,30 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E102" t="n">
-        <v>0.0265893292427063</v>
+        <v>0.928563674290975</v>
       </c>
       <c r="F102" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G102" t="n">
-        <v>0.1017009531136672</v>
+        <v>6.793312519849838</v>
       </c>
       <c r="H102" t="n">
-        <v>3.917027155943254</v>
+        <v>17.01574544376469</v>
       </c>
       <c r="I102" t="n">
-        <v>0.1017009531136672</v>
-      </c>
-      <c r="J102" t="n">
-        <v>3.917027155943254</v>
+        <v>6.793312519849838</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K102" t="n">
-        <v>4.076786859968062</v>
+        <v>14.45670328144963</v>
       </c>
       <c r="L102" t="n">
-        <v>3751.51469678494</v>
+        <v>16631.15631939737</v>
       </c>
     </row>
     <row r="103">
@@ -4738,28 +4712,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E103" t="n">
-        <v>0.2968737006187439</v>
+        <v>8.370152632395426</v>
       </c>
       <c r="F103" t="n">
-        <v>81</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="G103" t="n">
-        <v>10.54487657926557</v>
+        <v>28.23002195945354</v>
       </c>
       <c r="H103" t="n">
-        <v>18.80629214001168</v>
+        <v>52.0991475958883</v>
       </c>
       <c r="I103" t="n">
-        <v>2.525125306232527</v>
+        <v>28.23002195945354</v>
       </c>
       <c r="J103" t="n">
-        <v>23.64187151603962</v>
+        <v>75.49412273332037</v>
       </c>
       <c r="K103" t="n">
-        <v>24.79844328455565</v>
+        <v>33.75604119703338</v>
       </c>
       <c r="L103" t="n">
-        <v>78.3453035096737</v>
+        <v>394.0707195979046</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Experiment is finished in about 10 hours
</commit_message>
<xml_diff>
--- a/results/graphs/benchmark_results.xlsx
+++ b/results/graphs/benchmark_results.xlsx
@@ -496,7 +496,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1879293123881022</v>
+        <v>0.1225967001914978</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -538,7 +538,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2010863622029622</v>
+        <v>0.1113041377067566</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -580,7 +580,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1523040135701497</v>
+        <v>0.05275631904602051</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -622,7 +622,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1542932192484538</v>
+        <v>0.05257159233093261</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -664,7 +664,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6868889331817627</v>
+        <v>1.038922340869904</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -706,7 +706,7 @@
         <v>0.1285787260737514</v>
       </c>
       <c r="E7" t="n">
-        <v>7.052044312159221</v>
+        <v>32.17039316415786</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -748,7 +748,7 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E8" t="n">
-        <v>1.463008006413778</v>
+        <v>1.557159039974213</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -757,19 +757,19 @@
         <v>12.04748748354309</v>
       </c>
       <c r="H8" t="n">
-        <v>12.04748748354309</v>
+        <v>13.31954960345476</v>
       </c>
       <c r="I8" t="n">
         <v>12.04748748354309</v>
       </c>
       <c r="J8" t="n">
-        <v>12.04748748354309</v>
+        <v>13.31954960345476</v>
       </c>
       <c r="K8" t="n">
-        <v>2.175583928816829e-15</v>
+        <v>3.879918244765663</v>
       </c>
       <c r="L8" t="n">
-        <v>-1.474462490064223e-14</v>
+        <v>10.55873369156272</v>
       </c>
     </row>
     <row r="9">
@@ -790,7 +790,7 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E9" t="n">
-        <v>1.401365677515666</v>
+        <v>1.410780410766602</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -799,19 +799,19 @@
         <v>53.31120138136255</v>
       </c>
       <c r="H9" t="n">
-        <v>74.68741544755886</v>
+        <v>68.00304483753665</v>
       </c>
       <c r="I9" t="n">
         <v>53.31120138136255</v>
       </c>
       <c r="J9" t="n">
-        <v>74.68741544755886</v>
+        <v>68.00304483753665</v>
       </c>
       <c r="K9" t="n">
-        <v>23.71273295981149</v>
+        <v>13.22182557408432</v>
       </c>
       <c r="L9" t="n">
-        <v>40.09704060743486</v>
+        <v>27.55864260322283</v>
       </c>
     </row>
     <row r="10">
@@ -832,7 +832,7 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E10" t="n">
-        <v>1.283445119857788</v>
+        <v>1.207657351493835</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -841,19 +841,19 @@
         <v>12.04748748354309</v>
       </c>
       <c r="H10" t="n">
-        <v>21.98188464172121</v>
+        <v>27.40211757812223</v>
       </c>
       <c r="I10" t="n">
         <v>12.04748748354309</v>
       </c>
       <c r="J10" t="n">
-        <v>21.98188464172121</v>
+        <v>27.40211757812223</v>
       </c>
       <c r="K10" t="n">
-        <v>12.02269175057124</v>
+        <v>13.54979007249694</v>
       </c>
       <c r="L10" t="n">
-        <v>82.46032354670251</v>
+        <v>127.4508906156044</v>
       </c>
     </row>
     <row r="11">
@@ -874,28 +874,28 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E11" t="n">
-        <v>1.17594838142395</v>
+        <v>1.098425698280334</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>70.55706073287621</v>
+        <v>53.31120138136255</v>
       </c>
       <c r="H11" t="n">
-        <v>84.6847268524665</v>
+        <v>84.35006944786234</v>
       </c>
       <c r="I11" t="n">
-        <v>70.55706073287621</v>
+        <v>53.31120138136255</v>
       </c>
       <c r="J11" t="n">
-        <v>84.6847268524665</v>
+        <v>84.35006944786234</v>
       </c>
       <c r="K11" t="n">
-        <v>12.39306178552477</v>
+        <v>15.97685395199573</v>
       </c>
       <c r="L11" t="n">
-        <v>58.84978139335656</v>
+        <v>58.22203826258339</v>
       </c>
     </row>
     <row r="12">
@@ -916,28 +916,30 @@
         <v>12.04748748354309</v>
       </c>
       <c r="E12" t="n">
-        <v>1.115394592285156</v>
+        <v>1.177528121471405</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G12" t="n">
-        <v>19.45696800172116</v>
+        <v>12.04748748354309</v>
       </c>
       <c r="H12" t="n">
-        <v>20.62873454896448</v>
+        <v>41.24872702800602</v>
       </c>
       <c r="I12" t="n">
-        <v>19.45696800172116</v>
-      </c>
-      <c r="J12" t="n">
-        <v>20.62873454896448</v>
+        <v>12.04748748354309</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K12" t="n">
-        <v>1.553604857683085</v>
+        <v>22.17342695957565</v>
       </c>
       <c r="L12" t="n">
-        <v>71.22852027979616</v>
+        <v>242.3844771314511</v>
       </c>
     </row>
     <row r="13">
@@ -958,21 +960,31 @@
         <v>53.31120138136255</v>
       </c>
       <c r="E13" t="n">
-        <v>8.618704001108805</v>
+        <v>36.71475698232651</v>
       </c>
       <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>141.7282374772931</v>
+      </c>
+      <c r="H13" t="n">
+        <v>141.7282374772931</v>
+      </c>
+      <c r="I13" t="n">
+        <v>12.65112876324897</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="n">
-        <v>47.57847490964248</v>
-      </c>
-      <c r="J13" t="n">
-        <v>79.50395106466219</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>165.8507664523218</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -992,7 +1004,7 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E14" t="n">
-        <v>1.610737323760986</v>
+        <v>1.676236872673035</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1001,19 +1013,19 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2852081487284537</v>
+        <v>-6.117313146860117</v>
       </c>
       <c r="I14" t="n">
         <v>-11.80593354076133</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.2852081487284537</v>
+        <v>-6.117313146860117</v>
       </c>
       <c r="K14" t="n">
-        <v>10.04646731912484</v>
+        <v>6.772202762944361</v>
       </c>
       <c r="L14" t="n">
-        <v>97.58419655892742</v>
+        <v>48.18441823563214</v>
       </c>
     </row>
     <row r="15">
@@ -1034,7 +1046,7 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E15" t="n">
-        <v>1.612162351608276</v>
+        <v>1.681800019741058</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1043,19 +1055,19 @@
         <v>13.7263575295875</v>
       </c>
       <c r="H15" t="n">
-        <v>18.97706366014659</v>
+        <v>30.60598725996532</v>
       </c>
       <c r="I15" t="n">
         <v>13.7263575295875</v>
       </c>
       <c r="J15" t="n">
-        <v>18.97706366014659</v>
+        <v>30.60598725996532</v>
       </c>
       <c r="K15" t="n">
-        <v>4.850132045736043</v>
+        <v>16.15414640205883</v>
       </c>
       <c r="L15" t="n">
-        <v>38.25272742051967</v>
+        <v>122.9723886616923</v>
       </c>
     </row>
     <row r="16">
@@ -1076,28 +1088,28 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E16" t="n">
-        <v>1.638352394104004</v>
+        <v>1.306139440536499</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>4.297797156658406</v>
+        <v>-11.80593354076133</v>
       </c>
       <c r="H16" t="n">
-        <v>21.84179742087983</v>
+        <v>26.16081363195159</v>
       </c>
       <c r="I16" t="n">
-        <v>4.297797156658406</v>
+        <v>-11.80593354076133</v>
       </c>
       <c r="J16" t="n">
-        <v>21.84179742087983</v>
+        <v>26.16081363195159</v>
       </c>
       <c r="K16" t="n">
-        <v>15.86367097427612</v>
+        <v>19.0948981465087</v>
       </c>
       <c r="L16" t="n">
-        <v>285.0069487979797</v>
+        <v>321.5903853907732</v>
       </c>
     </row>
     <row r="17">
@@ -1118,28 +1130,28 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E17" t="n">
-        <v>1.431125720342</v>
+        <v>1.288183188438416</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>64.48172630257449</v>
+        <v>16.32499152035578</v>
       </c>
       <c r="H17" t="n">
-        <v>70.66150778251817</v>
+        <v>61.85414410388719</v>
       </c>
       <c r="I17" t="n">
-        <v>64.48172630257449</v>
+        <v>16.32499152035578</v>
       </c>
       <c r="J17" t="n">
-        <v>70.66150778251817</v>
+        <v>61.85414410388719</v>
       </c>
       <c r="K17" t="n">
-        <v>8.18443166056025</v>
+        <v>24.62268517885848</v>
       </c>
       <c r="L17" t="n">
-        <v>414.7870265669938</v>
+        <v>350.6231458022207</v>
       </c>
     </row>
     <row r="18">
@@ -1160,19 +1172,19 @@
         <v>-11.80593354076133</v>
       </c>
       <c r="E18" t="n">
-        <v>0.9904703299204508</v>
+        <v>1.194366590976715</v>
       </c>
       <c r="F18" t="n">
-        <v>66.66666666666666</v>
+        <v>93</v>
       </c>
       <c r="G18" t="n">
-        <v>4.896138561360734</v>
+        <v>-8.322401803670134</v>
       </c>
       <c r="H18" t="n">
-        <v>10.69764543237702</v>
+        <v>33.12441143005452</v>
       </c>
       <c r="I18" t="n">
-        <v>4.896138561360734</v>
+        <v>-8.322401803670134</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1180,10 +1192,10 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>8.204569699191927</v>
+        <v>28.77151895539288</v>
       </c>
       <c r="L18" t="n">
-        <v>190.6124483543989</v>
+        <v>380.5742664541412</v>
       </c>
     </row>
     <row r="19">
@@ -1204,21 +1216,31 @@
         <v>13.7263575295875</v>
       </c>
       <c r="E19" t="n">
-        <v>8.696507374445597</v>
+        <v>31.8091460609436</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="G19" t="n">
+        <v>48.45977014890117</v>
+      </c>
+      <c r="H19" t="n">
+        <v>135.3709263064193</v>
+      </c>
       <c r="I19" t="n">
-        <v>27.99504865350196</v>
-      </c>
-      <c r="J19" t="n">
-        <v>92.18875943360921</v>
-      </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+        <v>-11.65335479704901</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>49.52602920503304</v>
+      </c>
+      <c r="L19" t="n">
+        <v>886.2115715303489</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1238,28 +1260,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E20" t="n">
-        <v>1.927209297815959</v>
+        <v>2.712522768974304</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>-3.758716405667779</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="H20" t="n">
-        <v>0.770409565324441</v>
+        <v>-1.545451331787637</v>
       </c>
       <c r="I20" t="n">
-        <v>-3.758716405667779</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="J20" t="n">
-        <v>0.770409565324441</v>
+        <v>-1.545451331787637</v>
       </c>
       <c r="K20" t="n">
-        <v>4.266504127476306</v>
+        <v>7.565549347530935</v>
       </c>
       <c r="L20" t="n">
-        <v>108.1411354131304</v>
+        <v>83.6687793963367</v>
       </c>
     </row>
     <row r="21">
@@ -1280,28 +1302,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E21" t="n">
-        <v>1.770529349644979</v>
+        <v>2.169182329177856</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>24.95684465099749</v>
+        <v>15.06947538019221</v>
       </c>
       <c r="H21" t="n">
-        <v>33.36420076015548</v>
+        <v>30.82110677777466</v>
       </c>
       <c r="I21" t="n">
-        <v>24.95684465099749</v>
+        <v>15.06947538019221</v>
       </c>
       <c r="J21" t="n">
-        <v>33.36420076015548</v>
+        <v>30.82110677777466</v>
       </c>
       <c r="K21" t="n">
-        <v>7.447466314686423</v>
+        <v>12.66174598987365</v>
       </c>
       <c r="L21" t="n">
-        <v>121.4025367068215</v>
+        <v>104.5267403156377</v>
       </c>
     </row>
     <row r="22">
@@ -1322,28 +1344,28 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E22" t="n">
-        <v>1.59409236907959</v>
+        <v>2.004274439811707</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>7.060641592855646</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="H22" t="n">
-        <v>27.07035246089511</v>
+        <v>27.21538053844584</v>
       </c>
       <c r="I22" t="n">
-        <v>7.060641592855646</v>
+        <v>-9.463170998014522</v>
       </c>
       <c r="J22" t="n">
-        <v>27.07035246089511</v>
+        <v>27.21538053844584</v>
       </c>
       <c r="K22" t="n">
-        <v>22.78881140942149</v>
+        <v>18.2157949523639</v>
       </c>
       <c r="L22" t="n">
-        <v>386.0600581620555</v>
+        <v>387.5926108083213</v>
       </c>
     </row>
     <row r="23">
@@ -1364,28 +1386,28 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E23" t="n">
-        <v>1.520270983378093</v>
+        <v>1.733283178806305</v>
       </c>
       <c r="F23" t="n">
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>42.03499384317907</v>
+        <v>15.06947538019221</v>
       </c>
       <c r="H23" t="n">
-        <v>66.78404275042151</v>
+        <v>66.1914736958168</v>
       </c>
       <c r="I23" t="n">
-        <v>42.03499384317907</v>
+        <v>15.06947538019221</v>
       </c>
       <c r="J23" t="n">
-        <v>66.78404275042151</v>
+        <v>66.1914736958168</v>
       </c>
       <c r="K23" t="n">
-        <v>29.05257162586466</v>
+        <v>23.87476746837804</v>
       </c>
       <c r="L23" t="n">
-        <v>343.1743047817349</v>
+        <v>339.2420573766022</v>
       </c>
     </row>
     <row r="24">
@@ -1406,19 +1428,19 @@
         <v>-9.463170998014522</v>
       </c>
       <c r="E24" t="n">
-        <v>1.160794019699097</v>
+        <v>1.262820382118225</v>
       </c>
       <c r="F24" t="n">
-        <v>66.66666666666666</v>
+        <v>69</v>
       </c>
       <c r="G24" t="n">
-        <v>27.0642714807036</v>
+        <v>-8.408186147317938</v>
       </c>
       <c r="H24" t="n">
-        <v>31.35686774303407</v>
+        <v>57.57586395209224</v>
       </c>
       <c r="I24" t="n">
-        <v>27.0642714807036</v>
+        <v>-8.408186147317938</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1426,10 +1448,10 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>6.070647851979807</v>
+        <v>42.7671336233896</v>
       </c>
       <c r="L24" t="n">
-        <v>431.3568755083585</v>
+        <v>708.4204117644318</v>
       </c>
     </row>
     <row r="25">
@@ -1450,28 +1472,30 @@
         <v>15.06947538019221</v>
       </c>
       <c r="E25" t="n">
-        <v>9.525638659795126</v>
+        <v>16.24097564935684</v>
       </c>
       <c r="F25" t="n">
-        <v>33.33333333333333</v>
+        <v>25</v>
       </c>
       <c r="G25" t="n">
-        <v>189.0690162466089</v>
+        <v>42.47802159443006</v>
       </c>
       <c r="H25" t="n">
-        <v>189.0690162466089</v>
+        <v>148.5197807972362</v>
       </c>
       <c r="I25" t="n">
-        <v>11.71921242943418</v>
-      </c>
-      <c r="J25" t="n">
-        <v>104.6340857300811</v>
+        <v>-1.306577823785296</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>64.46986492295616</v>
       </c>
       <c r="L25" t="n">
-        <v>1154.648960740379</v>
+        <v>885.5670290450541</v>
       </c>
     </row>
     <row r="26">
@@ -1492,28 +1516,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E26" t="n">
-        <v>1.994977712631226</v>
+        <v>9.578639540672302</v>
       </c>
       <c r="F26" t="n">
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>-12.26324715798393</v>
+        <v>-21.96317396534843</v>
       </c>
       <c r="H26" t="n">
-        <v>-5.828972495513599</v>
+        <v>-9.846380563443967</v>
       </c>
       <c r="I26" t="n">
-        <v>-12.26324715798393</v>
+        <v>-21.96317396534843</v>
       </c>
       <c r="J26" t="n">
-        <v>-5.828972495513599</v>
+        <v>-9.846380563443967</v>
       </c>
       <c r="K26" t="n">
-        <v>5.572246791414693</v>
+        <v>9.422437378526126</v>
       </c>
       <c r="L26" t="n">
-        <v>73.46024529646743</v>
+        <v>55.16868108872278</v>
       </c>
     </row>
     <row r="27">
@@ -1534,28 +1558,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E27" t="n">
-        <v>1.867767731348674</v>
+        <v>1.924055869579315</v>
       </c>
       <c r="F27" t="n">
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>41.59734965676242</v>
+        <v>22.8444824168921</v>
       </c>
       <c r="H27" t="n">
-        <v>48.24650341074641</v>
+        <v>47.79787256910916</v>
       </c>
       <c r="I27" t="n">
-        <v>41.59734965676242</v>
+        <v>22.8444824168921</v>
       </c>
       <c r="J27" t="n">
-        <v>48.24650341074641</v>
+        <v>47.79787256910916</v>
       </c>
       <c r="K27" t="n">
-        <v>11.51667212923761</v>
+        <v>13.90406981574331</v>
       </c>
       <c r="L27" t="n">
-        <v>111.195432359943</v>
+        <v>109.2315846638117</v>
       </c>
     </row>
     <row r="28">
@@ -1576,28 +1600,28 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E28" t="n">
-        <v>1.640861590703328</v>
+        <v>1.628971109390259</v>
       </c>
       <c r="F28" t="n">
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>-8.638095787128815</v>
+        <v>-21.96317396534843</v>
       </c>
       <c r="H28" t="n">
-        <v>5.831544285723369</v>
+        <v>14.8814850321496</v>
       </c>
       <c r="I28" t="n">
-        <v>-8.638095787128815</v>
+        <v>-21.96317396534843</v>
       </c>
       <c r="J28" t="n">
-        <v>5.831544285723369</v>
+        <v>14.8814850321496</v>
       </c>
       <c r="K28" t="n">
-        <v>13.8823299483488</v>
+        <v>15.57482844545494</v>
       </c>
       <c r="L28" t="n">
-        <v>126.5514642597826</v>
+        <v>167.756532164378</v>
       </c>
     </row>
     <row r="29">
@@ -1618,28 +1642,28 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E29" t="n">
-        <v>1.627530336380005</v>
+        <v>1.514579222202301</v>
       </c>
       <c r="F29" t="n">
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>82.49122720406568</v>
+        <v>27.17282895821982</v>
       </c>
       <c r="H29" t="n">
-        <v>99.34603813998324</v>
+        <v>74.32871228467482</v>
       </c>
       <c r="I29" t="n">
-        <v>82.49122720406568</v>
+        <v>27.17282895821982</v>
       </c>
       <c r="J29" t="n">
-        <v>99.34603813998324</v>
+        <v>74.32871228467482</v>
       </c>
       <c r="K29" t="n">
-        <v>20.90248942691398</v>
+        <v>21.90818323147889</v>
       </c>
       <c r="L29" t="n">
-        <v>334.8797942846932</v>
+        <v>225.3683358994087</v>
       </c>
     </row>
     <row r="30">
@@ -1660,19 +1684,19 @@
         <v>-21.96317396534843</v>
       </c>
       <c r="E30" t="n">
-        <v>1.153596003850301</v>
+        <v>1.258333721160889</v>
       </c>
       <c r="F30" t="n">
-        <v>66.66666666666666</v>
+        <v>64</v>
       </c>
       <c r="G30" t="n">
-        <v>25.60736840705994</v>
+        <v>-6.511581934144693</v>
       </c>
       <c r="H30" t="n">
-        <v>33.95232120936691</v>
+        <v>41.83040828195204</v>
       </c>
       <c r="I30" t="n">
-        <v>25.60736840705994</v>
+        <v>-6.511581934144693</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1680,10 +1704,10 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>11.80154543038589</v>
+        <v>32.08692402595996</v>
       </c>
       <c r="L30" t="n">
-        <v>254.5874984323027</v>
+        <v>290.4570275131836</v>
       </c>
     </row>
     <row r="31">
@@ -1704,21 +1728,31 @@
         <v>22.8444824168921</v>
       </c>
       <c r="E31" t="n">
-        <v>10.18371327718099</v>
+        <v>17.64342714309693</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G31" t="n">
+        <v>110.3542761904784</v>
+      </c>
+      <c r="H31" t="n">
+        <v>155.2909169018649</v>
+      </c>
       <c r="I31" t="n">
-        <v>50.13618324377208</v>
-      </c>
-      <c r="J31" t="n">
-        <v>161.4826535735259</v>
-      </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+        <v>0.5684093252476607</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>30.15180490192368</v>
+      </c>
+      <c r="L31" t="n">
+        <v>579.7742845206103</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1738,28 +1772,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E32" t="n">
-        <v>2.323824008305868</v>
+        <v>1.688587250709534</v>
       </c>
       <c r="F32" t="n">
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>-7.873400703841429</v>
+        <v>-8.841290064295642</v>
       </c>
       <c r="H32" t="n">
-        <v>-2.774184083904669</v>
+        <v>-2.279296963522997</v>
       </c>
       <c r="I32" t="n">
-        <v>-7.873400703841429</v>
+        <v>-8.841290064295642</v>
       </c>
       <c r="J32" t="n">
-        <v>-2.774184083904669</v>
+        <v>-2.279296963522997</v>
       </c>
       <c r="K32" t="n">
-        <v>4.690364302942437</v>
+        <v>5.099974005865271</v>
       </c>
       <c r="L32" t="n">
-        <v>68.62240619038347</v>
+        <v>74.2198599192257</v>
       </c>
     </row>
     <row r="33">
@@ -1780,28 +1814,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E33" t="n">
-        <v>2.154251654942831</v>
+        <v>1.556748149394989</v>
       </c>
       <c r="F33" t="n">
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.08281480268923147</v>
+        <v>-1.050704163143443</v>
       </c>
       <c r="H33" t="n">
-        <v>21.83548256033676</v>
+        <v>16.15308876601903</v>
       </c>
       <c r="I33" t="n">
-        <v>-0.08281480268923147</v>
+        <v>-1.050704163143443</v>
       </c>
       <c r="J33" t="n">
-        <v>21.83548256033676</v>
+        <v>16.15308876601903</v>
       </c>
       <c r="K33" t="n">
-        <v>35.05637043329526</v>
+        <v>19.4858873418631</v>
       </c>
       <c r="L33" t="n">
-        <v>2178.176077175755</v>
+        <v>1637.358405213989</v>
       </c>
     </row>
     <row r="34">
@@ -1822,28 +1856,28 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E34" t="n">
-        <v>1.864962259928385</v>
+        <v>1.258051218986511</v>
       </c>
       <c r="F34" t="n">
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>18.40332392589283</v>
+        <v>-4.805345538997294</v>
       </c>
       <c r="H34" t="n">
-        <v>36.17862124687474</v>
+        <v>34.29284576698974</v>
       </c>
       <c r="I34" t="n">
-        <v>18.40332392589283</v>
+        <v>-4.805345538997294</v>
       </c>
       <c r="J34" t="n">
-        <v>36.17862124687474</v>
+        <v>34.29284576698974</v>
       </c>
       <c r="K34" t="n">
-        <v>18.01661396749524</v>
+        <v>20.38481858881511</v>
       </c>
       <c r="L34" t="n">
-        <v>509.2007046910182</v>
+        <v>487.8715155549162</v>
       </c>
     </row>
     <row r="35">
@@ -1864,28 +1898,28 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E35" t="n">
-        <v>1.850282351175944</v>
+        <v>1.215788850784302</v>
       </c>
       <c r="F35" t="n">
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>10.11440880163737</v>
+        <v>8.146515230894508</v>
       </c>
       <c r="H35" t="n">
-        <v>60.40349913801371</v>
+        <v>89.52562824910204</v>
       </c>
       <c r="I35" t="n">
-        <v>10.11440880163737</v>
+        <v>8.146515230894508</v>
       </c>
       <c r="J35" t="n">
-        <v>60.40349913801371</v>
+        <v>89.52562824910204</v>
       </c>
       <c r="K35" t="n">
-        <v>46.25775095134383</v>
+        <v>38.07310944587593</v>
       </c>
       <c r="L35" t="n">
-        <v>5848.858837420192</v>
+        <v>8620.536168931112</v>
       </c>
     </row>
     <row r="36">
@@ -1906,28 +1940,30 @@
         <v>-8.841290064295642</v>
       </c>
       <c r="E36" t="n">
-        <v>1.310578346252441</v>
+        <v>0.6976067924499512</v>
       </c>
       <c r="F36" t="n">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="G36" t="n">
-        <v>19.44669875577845</v>
+        <v>-6.721699441703031</v>
       </c>
       <c r="H36" t="n">
-        <v>54.48244429275157</v>
+        <v>51.20122057779486</v>
       </c>
       <c r="I36" t="n">
-        <v>19.44669875577845</v>
-      </c>
-      <c r="J36" t="n">
-        <v>54.48244429275157</v>
+        <v>-6.721699441703031</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K36" t="n">
-        <v>45.06483211228916</v>
+        <v>35.31873369976594</v>
       </c>
       <c r="L36" t="n">
-        <v>716.2273140745781</v>
+        <v>679.1148147549654</v>
       </c>
     </row>
     <row r="37">
@@ -1948,23 +1984,31 @@
         <v>-1.050704163143443</v>
       </c>
       <c r="E37" t="n">
-        <v>9.690512975056967</v>
+        <v>9.436911969184875</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G37" t="n">
+        <v>252.9310956178438</v>
+      </c>
+      <c r="H37" t="n">
+        <v>265.732605417168</v>
+      </c>
       <c r="I37" t="n">
-        <v>60.09728936452053</v>
+        <v>-6.721699441703031</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>18.10406877705625</v>
+      </c>
+      <c r="L37" t="n">
+        <v>25390.90630250885</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1984,7 +2028,7 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E38" t="n">
-        <v>2.47080667813619</v>
+        <v>1.525962879657745</v>
       </c>
       <c r="F38" t="n">
         <v>100</v>
@@ -1993,19 +2037,19 @@
         <v>9.383712874145662</v>
       </c>
       <c r="H38" t="n">
-        <v>19.64053134499601</v>
+        <v>20.35489113743854</v>
       </c>
       <c r="I38" t="n">
         <v>9.383712874145662</v>
       </c>
       <c r="J38" t="n">
-        <v>19.64053134499601</v>
+        <v>20.35489113743854</v>
       </c>
       <c r="K38" t="n">
-        <v>9.145696988089208</v>
+        <v>9.608582019133928</v>
       </c>
       <c r="L38" t="n">
-        <v>109.3044790310059</v>
+        <v>116.917241719118</v>
       </c>
     </row>
     <row r="39">
@@ -2026,28 +2070,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E39" t="n">
-        <v>2.155666987101237</v>
+        <v>1.510630440711975</v>
       </c>
       <c r="F39" t="n">
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>41.34874866528129</v>
+        <v>26.21619167672251</v>
       </c>
       <c r="H39" t="n">
-        <v>53.77413253383622</v>
+        <v>45.59692654069034</v>
       </c>
       <c r="I39" t="n">
-        <v>41.34874866528129</v>
+        <v>26.21619167672251</v>
       </c>
       <c r="J39" t="n">
-        <v>53.77413253383622</v>
+        <v>45.59692654069034</v>
       </c>
       <c r="K39" t="n">
-        <v>16.47205155000465</v>
+        <v>9.41791958869609</v>
       </c>
       <c r="L39" t="n">
-        <v>105.1180171282564</v>
+        <v>73.92658362799536</v>
       </c>
     </row>
     <row r="40">
@@ -2068,28 +2112,28 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E40" t="n">
-        <v>1.869088729222615</v>
+        <v>1.238764090538025</v>
       </c>
       <c r="F40" t="n">
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>41.43632650113572</v>
+        <v>13.67196736587999</v>
       </c>
       <c r="H40" t="n">
-        <v>47.11875873930884</v>
+        <v>55.30327587336041</v>
       </c>
       <c r="I40" t="n">
-        <v>41.43632650113572</v>
+        <v>13.67196736587999</v>
       </c>
       <c r="J40" t="n">
-        <v>47.11875873930884</v>
+        <v>55.30327587336041</v>
       </c>
       <c r="K40" t="n">
-        <v>5.824129165080397</v>
+        <v>16.6797058693754</v>
       </c>
       <c r="L40" t="n">
-        <v>402.1334238511507</v>
+        <v>489.3538795899643</v>
       </c>
     </row>
     <row r="41">
@@ -2110,28 +2154,28 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E41" t="n">
-        <v>1.82608699798584</v>
+        <v>1.207720050811768</v>
       </c>
       <c r="F41" t="n">
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>46.08755662137803</v>
+        <v>37.99671425149539</v>
       </c>
       <c r="H41" t="n">
-        <v>61.9756856565895</v>
+        <v>72.36065309667025</v>
       </c>
       <c r="I41" t="n">
-        <v>46.08755662137803</v>
+        <v>37.99671425149539</v>
       </c>
       <c r="J41" t="n">
-        <v>61.9756856565895</v>
+        <v>72.36065309667025</v>
       </c>
       <c r="K41" t="n">
-        <v>20.23663457870682</v>
+        <v>20.35015324867954</v>
       </c>
       <c r="L41" t="n">
-        <v>136.4023212098271</v>
+        <v>176.0151206894006</v>
       </c>
     </row>
     <row r="42">
@@ -2152,19 +2196,19 @@
         <v>9.383712874145662</v>
       </c>
       <c r="E42" t="n">
-        <v>1.131096998850505</v>
+        <v>0.6930194497108459</v>
       </c>
       <c r="F42" t="n">
-        <v>66.66666666666666</v>
+        <v>78</v>
       </c>
       <c r="G42" t="n">
-        <v>29.0643863437334</v>
+        <v>27.65288672397242</v>
       </c>
       <c r="H42" t="n">
-        <v>44.47247064366387</v>
+        <v>66.09368157164353</v>
       </c>
       <c r="I42" t="n">
-        <v>29.0643863437334</v>
+        <v>27.65288672397242</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2172,10 +2216,10 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>21.79032178714962</v>
+        <v>28.04914663461815</v>
       </c>
       <c r="L42" t="n">
-        <v>373.932559959246</v>
+        <v>604.3446710070082</v>
       </c>
     </row>
     <row r="43">
@@ -2196,28 +2240,30 @@
         <v>26.21619167672251</v>
       </c>
       <c r="E43" t="n">
-        <v>10.01489273707072</v>
+        <v>8.27317785024643</v>
       </c>
       <c r="F43" t="n">
-        <v>66.66666666666666</v>
+        <v>20</v>
       </c>
       <c r="G43" t="n">
-        <v>65.2667442259319</v>
+        <v>45.02375600227383</v>
       </c>
       <c r="H43" t="n">
-        <v>71.57931473911299</v>
+        <v>71.24315672707151</v>
       </c>
       <c r="I43" t="n">
-        <v>24.30247503222626</v>
-      </c>
-      <c r="J43" t="n">
-        <v>55.82036817015075</v>
+        <v>25.38322859243531</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K43" t="n">
-        <v>8.927322833177191</v>
+        <v>38.90326656304834</v>
       </c>
       <c r="L43" t="n">
-        <v>173.0347550924745</v>
+        <v>171.7525016813508</v>
       </c>
     </row>
     <row r="44">
@@ -2238,7 +2284,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E44" t="n">
-        <v>0.3895590305328369</v>
+        <v>0.1513384199142456</v>
       </c>
       <c r="F44" t="n">
         <v>100</v>
@@ -2256,7 +2302,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
@@ -2280,7 +2326,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E45" t="n">
-        <v>0.4008009433746338</v>
+        <v>0.1572854804992676</v>
       </c>
       <c r="F45" t="n">
         <v>100</v>
@@ -2322,7 +2368,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3364046414693196</v>
+        <v>0.09838800907135009</v>
       </c>
       <c r="F46" t="n">
         <v>100</v>
@@ -2340,7 +2386,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2364,7 +2410,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3455493450164795</v>
+        <v>0.1051426696777344</v>
       </c>
       <c r="F47" t="n">
         <v>100</v>
@@ -2406,7 +2452,7 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="E48" t="n">
-        <v>0.8248132864634196</v>
+        <v>0.5579094576835633</v>
       </c>
       <c r="F48" t="n">
         <v>100</v>
@@ -2415,19 +2461,19 @@
         <v>-10.65196883415753</v>
       </c>
       <c r="H48" t="n">
-        <v>-10.65196883415753</v>
+        <v>-10.03863650171084</v>
       </c>
       <c r="I48" t="n">
         <v>-10.65196883415753</v>
       </c>
       <c r="J48" t="n">
-        <v>-10.65196883415753</v>
+        <v>-10.03863650171084</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>2.775471437065472</v>
       </c>
       <c r="L48" t="n">
-        <v>0</v>
+        <v>5.757924586485133</v>
       </c>
     </row>
     <row r="49">
@@ -2448,7 +2494,7 @@
         <v>0.06733358914136289</v>
       </c>
       <c r="E49" t="n">
-        <v>7.259474595387776</v>
+        <v>6.834791178703308</v>
       </c>
       <c r="F49" t="n">
         <v>100</v>
@@ -2490,28 +2536,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E50" t="n">
-        <v>3.528955618540446</v>
+        <v>2.739487187862396</v>
       </c>
       <c r="F50" t="n">
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>30.27537186972479</v>
+        <v>13.02451543344857</v>
       </c>
       <c r="H50" t="n">
-        <v>47.59417951446528</v>
+        <v>39.4957381539649</v>
       </c>
       <c r="I50" t="n">
-        <v>30.27537186972479</v>
+        <v>13.02451543344857</v>
       </c>
       <c r="J50" t="n">
-        <v>47.59417951446528</v>
+        <v>39.4957381539649</v>
       </c>
       <c r="K50" t="n">
-        <v>15.00319976160127</v>
+        <v>15.36165942722505</v>
       </c>
       <c r="L50" t="n">
-        <v>265.4199632812253</v>
+        <v>203.2415167825357</v>
       </c>
     </row>
     <row r="51">
@@ -2532,28 +2578,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E51" t="n">
-        <v>3.546395381291708</v>
+        <v>2.642260408401489</v>
       </c>
       <c r="F51" t="n">
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>37.60618409062889</v>
+        <v>31.42655177776513</v>
       </c>
       <c r="H51" t="n">
-        <v>68.09142119442838</v>
+        <v>66.14182458928123</v>
       </c>
       <c r="I51" t="n">
-        <v>37.60618409062889</v>
+        <v>31.42655177776513</v>
       </c>
       <c r="J51" t="n">
-        <v>68.09142119442838</v>
+        <v>66.14182458928123</v>
       </c>
       <c r="K51" t="n">
-        <v>29.11079206897703</v>
+        <v>19.81584881522823</v>
       </c>
       <c r="L51" t="n">
-        <v>191.7405299686475</v>
+        <v>183.3874021173926</v>
       </c>
     </row>
     <row r="52">
@@ -2574,28 +2620,28 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E52" t="n">
-        <v>3.003234624862671</v>
+        <v>2.179648342132568</v>
       </c>
       <c r="F52" t="n">
         <v>100</v>
       </c>
       <c r="G52" t="n">
-        <v>89.20867358878883</v>
+        <v>60.21127380311113</v>
       </c>
       <c r="H52" t="n">
-        <v>94.29226409484549</v>
+        <v>115.0862134014713</v>
       </c>
       <c r="I52" t="n">
-        <v>89.20867358878883</v>
+        <v>60.21127380311113</v>
       </c>
       <c r="J52" t="n">
-        <v>94.29226409484549</v>
+        <v>115.0862134014713</v>
       </c>
       <c r="K52" t="n">
-        <v>4.922387598102157</v>
+        <v>24.78522513348075</v>
       </c>
       <c r="L52" t="n">
-        <v>623.9598630494249</v>
+        <v>783.6122463789754</v>
       </c>
     </row>
     <row r="53">
@@ -2616,28 +2662,28 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E53" t="n">
-        <v>2.980710983276367</v>
+        <v>2.114515678882599</v>
       </c>
       <c r="F53" t="n">
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>152.3677802137354</v>
+        <v>64.70025535731861</v>
       </c>
       <c r="H53" t="n">
-        <v>167.2062146222932</v>
+        <v>155.6551704954819</v>
       </c>
       <c r="I53" t="n">
-        <v>152.3677802137354</v>
+        <v>64.70025535731861</v>
       </c>
       <c r="J53" t="n">
-        <v>167.2062146222932</v>
+        <v>155.6551704954819</v>
       </c>
       <c r="K53" t="n">
-        <v>12.88274822662302</v>
+        <v>36.36569795657164</v>
       </c>
       <c r="L53" t="n">
-        <v>616.401990328126</v>
+        <v>566.9110606906801</v>
       </c>
     </row>
     <row r="54">
@@ -2658,25 +2704,31 @@
         <v>13.02451543344857</v>
       </c>
       <c r="E54" t="n">
-        <v>1.320327361424764</v>
+        <v>0.7555224108695984</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="G54" t="n">
+        <v>92.24865449221173</v>
+      </c>
+      <c r="H54" t="n">
+        <v>110.5426115207384</v>
+      </c>
+      <c r="I54" t="n">
+        <v>92.24865449221173</v>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>16.00230907694063</v>
+      </c>
+      <c r="L54" t="n">
+        <v>748.7272488990359</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2696,17 +2748,15 @@
         <v>23.33971944239148</v>
       </c>
       <c r="E55" t="n">
-        <v>9.390654961268107</v>
+        <v>9.131371018886567</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="I55" t="n">
+        <v>91.11774527108693</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -2734,7 +2784,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E56" t="n">
-        <v>0.414016326268514</v>
+        <v>0.2062857794761658</v>
       </c>
       <c r="F56" t="n">
         <v>100</v>
@@ -2752,7 +2802,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>3.570611593983174e-15</v>
       </c>
       <c r="L56" t="n">
         <v>0</v>
@@ -2776,7 +2826,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E57" t="n">
-        <v>0.4078160127003987</v>
+        <v>0.2083084678649902</v>
       </c>
       <c r="F57" t="n">
         <v>100</v>
@@ -2794,7 +2844,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L57" t="n">
         <v>0</v>
@@ -2818,7 +2868,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E58" t="n">
-        <v>0.3458969593048096</v>
+        <v>0.1459188318252563</v>
       </c>
       <c r="F58" t="n">
         <v>100</v>
@@ -2836,7 +2886,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="K58" t="n">
-        <v>0</v>
+        <v>3.570611593983174e-15</v>
       </c>
       <c r="L58" t="n">
         <v>0</v>
@@ -2860,7 +2910,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E59" t="n">
-        <v>0.3465774059295654</v>
+        <v>0.145380449295044</v>
       </c>
       <c r="F59" t="n">
         <v>100</v>
@@ -2878,7 +2928,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L59" t="n">
         <v>0</v>
@@ -2902,7 +2952,7 @@
         <v>13.90826436045291</v>
       </c>
       <c r="E60" t="n">
-        <v>0.8312124411265055</v>
+        <v>0.5752708101272583</v>
       </c>
       <c r="F60" t="n">
         <v>100</v>
@@ -2911,19 +2961,19 @@
         <v>13.90826436045291</v>
       </c>
       <c r="H60" t="n">
-        <v>18.68256530384832</v>
+        <v>18.11467872342908</v>
       </c>
       <c r="I60" t="n">
         <v>13.90826436045291</v>
       </c>
       <c r="J60" t="n">
-        <v>18.68256530384832</v>
+        <v>18.11467872342908</v>
       </c>
       <c r="K60" t="n">
-        <v>5.962790698516184</v>
+        <v>5.260817414539803</v>
       </c>
       <c r="L60" t="n">
-        <v>34.32707935125806</v>
+        <v>30.24399201770126</v>
       </c>
     </row>
     <row r="61">
@@ -2944,7 +2994,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="E61" t="n">
-        <v>7.960235754648845</v>
+        <v>7.49886721611023</v>
       </c>
       <c r="F61" t="n">
         <v>100</v>
@@ -2962,7 +3012,7 @@
         <v>16.77327413265929</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
@@ -2986,7 +3036,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E62" t="n">
-        <v>0.5718727111816406</v>
+        <v>0.3371634578704834</v>
       </c>
       <c r="F62" t="n">
         <v>100</v>
@@ -3004,7 +3054,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="K62" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>7.141223187966347e-15</v>
       </c>
       <c r="L62" t="n">
         <v>-1.431247886831891e-14</v>
@@ -3028,7 +3078,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E63" t="n">
-        <v>0.5649979909261068</v>
+        <v>0.3403460097312927</v>
       </c>
       <c r="F63" t="n">
         <v>100</v>
@@ -3037,19 +3087,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H63" t="n">
-        <v>48.65032644645115</v>
+        <v>48.95661104998514</v>
       </c>
       <c r="I63" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J63" t="n">
-        <v>48.65032644645115</v>
+        <v>48.95661104998514</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>1.508041140520523</v>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
+        <v>0.6295633059546266</v>
       </c>
     </row>
     <row r="64">
@@ -3070,7 +3120,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E64" t="n">
-        <v>0.4589842955271403</v>
+        <v>0.2480891013145447</v>
       </c>
       <c r="F64" t="n">
         <v>100</v>
@@ -3079,19 +3129,19 @@
         <v>24.82249030015713</v>
       </c>
       <c r="H64" t="n">
-        <v>24.82249030015713</v>
+        <v>24.86957653283245</v>
       </c>
       <c r="I64" t="n">
         <v>24.82249030015713</v>
       </c>
       <c r="J64" t="n">
-        <v>24.82249030015713</v>
+        <v>24.86957653283245</v>
       </c>
       <c r="K64" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>0.470862326753177</v>
       </c>
       <c r="L64" t="n">
-        <v>-1.431247886831891e-14</v>
+        <v>0.1896918161954972</v>
       </c>
     </row>
     <row r="65">
@@ -3112,7 +3162,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E65" t="n">
-        <v>0.520045280456543</v>
+        <v>0.2432095575332641</v>
       </c>
       <c r="F65" t="n">
         <v>100</v>
@@ -3121,19 +3171,19 @@
         <v>48.65032644645115</v>
       </c>
       <c r="H65" t="n">
-        <v>51.20269814256776</v>
+        <v>49.28954977553857</v>
       </c>
       <c r="I65" t="n">
         <v>48.65032644645115</v>
       </c>
       <c r="J65" t="n">
-        <v>51.20269814256776</v>
+        <v>49.28954977553857</v>
       </c>
       <c r="K65" t="n">
-        <v>4.420837457474725</v>
+        <v>3.031050996771072</v>
       </c>
       <c r="L65" t="n">
-        <v>5.246360882955188</v>
+        <v>1.313913751002297</v>
       </c>
     </row>
     <row r="66">
@@ -3154,7 +3204,7 @@
         <v>24.82249030015713</v>
       </c>
       <c r="E66" t="n">
-        <v>0.8588020006815592</v>
+        <v>0.6090101790428162</v>
       </c>
       <c r="F66" t="n">
         <v>100</v>
@@ -3163,19 +3213,19 @@
         <v>24.82249030015713</v>
       </c>
       <c r="H66" t="n">
-        <v>26.99605343621456</v>
+        <v>30.66087556562202</v>
       </c>
       <c r="I66" t="n">
         <v>24.82249030015713</v>
       </c>
       <c r="J66" t="n">
-        <v>26.99605343621456</v>
+        <v>30.66087556562202</v>
       </c>
       <c r="K66" t="n">
-        <v>3.764721785110208</v>
+        <v>7.036802355447115</v>
       </c>
       <c r="L66" t="n">
-        <v>8.756426570317439</v>
+        <v>23.52054606474326</v>
       </c>
     </row>
     <row r="67">
@@ -3196,7 +3246,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="E67" t="n">
-        <v>7.666666984558105</v>
+        <v>7.077053349018097</v>
       </c>
       <c r="F67" t="n">
         <v>100</v>
@@ -3214,7 +3264,7 @@
         <v>48.65032644645115</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>2.142366956389904e-14</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
@@ -3238,7 +3288,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E68" t="n">
-        <v>0.1903249422709147</v>
+        <v>0.0910670804977417</v>
       </c>
       <c r="F68" t="n">
         <v>100</v>
@@ -3256,7 +3306,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
@@ -3280,7 +3330,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E69" t="n">
-        <v>0.2013113498687744</v>
+        <v>0.09215166807174682</v>
       </c>
       <c r="F69" t="n">
         <v>100</v>
@@ -3298,7 +3348,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L69" t="n">
         <v>0</v>
@@ -3322,7 +3372,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E70" t="n">
-        <v>0.1571446259816488</v>
+        <v>0.05009796857833862</v>
       </c>
       <c r="F70" t="n">
         <v>100</v>
@@ -3340,7 +3390,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
@@ -3364,7 +3414,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E71" t="n">
-        <v>0.1580249468485514</v>
+        <v>0.05049026012420654</v>
       </c>
       <c r="F71" t="n">
         <v>100</v>
@@ -3382,7 +3432,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
@@ -3406,7 +3456,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E72" t="n">
-        <v>0.9425457318623861</v>
+        <v>0.5515336012840271</v>
       </c>
       <c r="F72" t="n">
         <v>100</v>
@@ -3424,7 +3474,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K72" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L72" t="n">
         <v>0</v>
@@ -3448,7 +3498,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="E73" t="n">
-        <v>7.38074803352356</v>
+        <v>6.749778590202332</v>
       </c>
       <c r="F73" t="n">
         <v>100</v>
@@ -3466,7 +3516,7 @@
         <v>8.340019847439855</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>1.785305796991587e-15</v>
       </c>
       <c r="L73" t="n">
         <v>0</v>
@@ -3490,7 +3540,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E74" t="n">
-        <v>0.6762966314951578</v>
+        <v>0.3685086512565613</v>
       </c>
       <c r="F74" t="n">
         <v>100</v>
@@ -3499,19 +3549,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H74" t="n">
-        <v>30.95896547744237</v>
+        <v>31.15128597017634</v>
       </c>
       <c r="I74" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J74" t="n">
-        <v>30.95896547744237</v>
+        <v>31.15128597017634</v>
       </c>
       <c r="K74" t="n">
-        <v>4.351167857633658e-15</v>
+        <v>0.9711460725235028</v>
       </c>
       <c r="L74" t="n">
-        <v>-1.147555683470468e-14</v>
+        <v>0.6212109796566158</v>
       </c>
     </row>
     <row r="75">
@@ -3532,7 +3582,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E75" t="n">
-        <v>0.658511241277059</v>
+        <v>0.3644229125976562</v>
       </c>
       <c r="F75" t="n">
         <v>100</v>
@@ -3541,19 +3591,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H75" t="n">
-        <v>38.20684438128487</v>
+        <v>40.19373377989256</v>
       </c>
       <c r="I75" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J75" t="n">
-        <v>38.20684438128487</v>
+        <v>40.19373377989256</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>3.019204922589855</v>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>5.200349389705019</v>
       </c>
     </row>
     <row r="76">
@@ -3574,7 +3624,7 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E76" t="n">
-        <v>0.5730956395467123</v>
+        <v>0.2800627565383911</v>
       </c>
       <c r="F76" t="n">
         <v>100</v>
@@ -3583,19 +3633,19 @@
         <v>30.95896547744237</v>
       </c>
       <c r="H76" t="n">
-        <v>31.88291438831978</v>
+        <v>32.22952931122617</v>
       </c>
       <c r="I76" t="n">
         <v>30.95896547744237</v>
       </c>
       <c r="J76" t="n">
-        <v>31.88291438831978</v>
+        <v>32.22952931122617</v>
       </c>
       <c r="K76" t="n">
-        <v>1.600326457237609</v>
+        <v>2.766782578127574</v>
       </c>
       <c r="L76" t="n">
-        <v>2.984430831678232</v>
+        <v>4.104025487252046</v>
       </c>
     </row>
     <row r="77">
@@ -3616,7 +3666,7 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E77" t="n">
-        <v>0.5648903846740723</v>
+        <v>0.2726493382453918</v>
       </c>
       <c r="F77" t="n">
         <v>100</v>
@@ -3625,19 +3675,19 @@
         <v>38.20684438128487</v>
       </c>
       <c r="H77" t="n">
-        <v>38.84450275393277</v>
+        <v>41.63559334052122</v>
       </c>
       <c r="I77" t="n">
         <v>38.20684438128487</v>
       </c>
       <c r="J77" t="n">
-        <v>38.84450275393277</v>
+        <v>41.63559334052122</v>
       </c>
       <c r="K77" t="n">
-        <v>1.104456699297865</v>
+        <v>4.476723655869379</v>
       </c>
       <c r="L77" t="n">
-        <v>1.668963723578947</v>
+        <v>8.97417469241684</v>
       </c>
     </row>
     <row r="78">
@@ -3658,28 +3708,28 @@
         <v>30.95896547744237</v>
       </c>
       <c r="E78" t="n">
-        <v>0.9480663140614828</v>
+        <v>0.5976583075523376</v>
       </c>
       <c r="F78" t="n">
         <v>100</v>
       </c>
       <c r="G78" t="n">
-        <v>40.9786911139171</v>
+        <v>30.95896547744237</v>
       </c>
       <c r="H78" t="n">
-        <v>60.30925492758055</v>
+        <v>56.47370484630336</v>
       </c>
       <c r="I78" t="n">
-        <v>40.9786911139171</v>
+        <v>30.95896547744237</v>
       </c>
       <c r="J78" t="n">
-        <v>60.30925492758055</v>
+        <v>56.47370484630336</v>
       </c>
       <c r="K78" t="n">
-        <v>18.0859020148175</v>
+        <v>15.84990798961469</v>
       </c>
       <c r="L78" t="n">
-        <v>94.80384437110368</v>
+        <v>82.4147027375698</v>
       </c>
     </row>
     <row r="79">
@@ -3700,28 +3750,28 @@
         <v>38.20684438128487</v>
       </c>
       <c r="E79" t="n">
-        <v>8.634498596191406</v>
+        <v>7.194549322128296</v>
       </c>
       <c r="F79" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G79" t="n">
-        <v>46.35150672415288</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="H79" t="n">
-        <v>65.20360019650697</v>
+        <v>59.30545610958403</v>
       </c>
       <c r="I79" t="n">
-        <v>46.35150672415288</v>
+        <v>38.20684438128487</v>
       </c>
       <c r="J79" t="n">
-        <v>65.20360019650697</v>
+        <v>59.90724001821787</v>
       </c>
       <c r="K79" t="n">
-        <v>16.57616084249375</v>
+        <v>13.94305603738762</v>
       </c>
       <c r="L79" t="n">
-        <v>70.65947542227831</v>
+        <v>55.22207361002063</v>
       </c>
     </row>
     <row r="80">
@@ -3742,7 +3792,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E80" t="n">
-        <v>0.8686463038126627</v>
+        <v>0.5365091490745545</v>
       </c>
       <c r="F80" t="n">
         <v>100</v>
@@ -3751,19 +3801,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H80" t="n">
-        <v>1.273146143170434</v>
+        <v>1.329456235319742</v>
       </c>
       <c r="I80" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J80" t="n">
-        <v>1.273146143170434</v>
+        <v>1.329456235319742</v>
       </c>
       <c r="K80" t="n">
-        <v>0.4275746877548631</v>
+        <v>0.7293760834463431</v>
       </c>
       <c r="L80" t="n">
-        <v>24.05376410551598</v>
+        <v>29.54054889116094</v>
       </c>
     </row>
     <row r="81">
@@ -3784,28 +3834,28 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E81" t="n">
-        <v>0.9065333207448324</v>
+        <v>0.5278788137435914</v>
       </c>
       <c r="F81" t="n">
         <v>100</v>
       </c>
       <c r="G81" t="n">
-        <v>19.29718019360264</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="H81" t="n">
-        <v>19.83334689708312</v>
+        <v>21.66288163703738</v>
       </c>
       <c r="I81" t="n">
-        <v>19.29718019360264</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="J81" t="n">
-        <v>19.83334689708312</v>
+        <v>21.66288163703738</v>
       </c>
       <c r="K81" t="n">
-        <v>0.5417048304786438</v>
+        <v>4.170583041447423</v>
       </c>
       <c r="L81" t="n">
-        <v>9.143157303042813</v>
+        <v>19.21110997640506</v>
       </c>
     </row>
     <row r="82">
@@ -3826,28 +3876,28 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E82" t="n">
-        <v>0.7165652910868326</v>
+        <v>0.4054171991348267</v>
       </c>
       <c r="F82" t="n">
         <v>100</v>
       </c>
       <c r="G82" t="n">
-        <v>1.766866865318315</v>
+        <v>1.026285782096494</v>
       </c>
       <c r="H82" t="n">
-        <v>3.514450942422638</v>
+        <v>4.838593404087128</v>
       </c>
       <c r="I82" t="n">
-        <v>1.766866865318315</v>
+        <v>1.026285782096494</v>
       </c>
       <c r="J82" t="n">
-        <v>3.514450942422638</v>
+        <v>4.838593404087128</v>
       </c>
       <c r="K82" t="n">
-        <v>1.558092636885859</v>
+        <v>5.159355878678491</v>
       </c>
       <c r="L82" t="n">
-        <v>242.4436939234729</v>
+        <v>371.4664753713008</v>
       </c>
     </row>
     <row r="83">
@@ -3868,28 +3918,28 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E83" t="n">
-        <v>0.7029693921407064</v>
+        <v>0.3947764611244202</v>
       </c>
       <c r="F83" t="n">
         <v>100</v>
       </c>
       <c r="G83" t="n">
-        <v>28.82591742481698</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="H83" t="n">
-        <v>29.82313964390611</v>
+        <v>24.91173472300643</v>
       </c>
       <c r="I83" t="n">
-        <v>28.82591742481698</v>
+        <v>18.17186472076723</v>
       </c>
       <c r="J83" t="n">
-        <v>29.82313964390611</v>
+        <v>24.91173472300643</v>
       </c>
       <c r="K83" t="n">
-        <v>1.727239549898954</v>
+        <v>5.448398048916882</v>
       </c>
       <c r="L83" t="n">
-        <v>64.11711237220213</v>
+        <v>37.08958935038029</v>
       </c>
     </row>
     <row r="84">
@@ -3910,7 +3960,7 @@
         <v>1.026285782096494</v>
       </c>
       <c r="E84" t="n">
-        <v>0.9585286776224772</v>
+        <v>0.6014848184585572</v>
       </c>
       <c r="F84" t="n">
         <v>100</v>
@@ -3919,19 +3969,19 @@
         <v>1.026285782096494</v>
       </c>
       <c r="H84" t="n">
-        <v>11.80789107907135</v>
+        <v>20.98971460120523</v>
       </c>
       <c r="I84" t="n">
         <v>1.026285782096494</v>
       </c>
       <c r="J84" t="n">
-        <v>11.80789107907135</v>
+        <v>20.98971460120523</v>
       </c>
       <c r="K84" t="n">
-        <v>18.03672752721468</v>
+        <v>14.73863988683439</v>
       </c>
       <c r="L84" t="n">
-        <v>1050.546103732454</v>
+        <v>1945.211476897546</v>
       </c>
     </row>
     <row r="85">
@@ -3952,7 +4002,7 @@
         <v>18.17186472076723</v>
       </c>
       <c r="E85" t="n">
-        <v>7.935341676076253</v>
+        <v>7.484333307743072</v>
       </c>
       <c r="F85" t="n">
         <v>100</v>
@@ -3961,19 +4011,19 @@
         <v>18.17186472076723</v>
       </c>
       <c r="H85" t="n">
-        <v>24.01530249686201</v>
+        <v>22.27716329315527</v>
       </c>
       <c r="I85" t="n">
         <v>18.17186472076723</v>
       </c>
       <c r="J85" t="n">
-        <v>24.01530249686201</v>
+        <v>22.27716329315527</v>
       </c>
       <c r="K85" t="n">
-        <v>10.12113111906344</v>
+        <v>6.456556433816468</v>
       </c>
       <c r="L85" t="n">
-        <v>32.15651154070478</v>
+        <v>22.59150965226155</v>
       </c>
     </row>
     <row r="86">
@@ -3994,7 +4044,7 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E86" t="n">
-        <v>1.030043999354045</v>
+        <v>6.320690729618073</v>
       </c>
       <c r="F86" t="n">
         <v>100</v>
@@ -4003,19 +4053,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="H86" t="n">
-        <v>45.01044323572248</v>
+        <v>46.3487983292337</v>
       </c>
       <c r="I86" t="n">
         <v>44.28900565726017</v>
       </c>
       <c r="J86" t="n">
-        <v>45.01044323572248</v>
+        <v>46.3487983292337</v>
       </c>
       <c r="K86" t="n">
-        <v>1.249566540386187</v>
+        <v>3.494828163530634</v>
       </c>
       <c r="L86" t="n">
-        <v>1.628931532230169</v>
+        <v>4.650799089764339</v>
       </c>
     </row>
     <row r="87">
@@ -4036,7 +4086,7 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E87" t="n">
-        <v>1.023363351821899</v>
+        <v>0.6552797794342041</v>
       </c>
       <c r="F87" t="n">
         <v>100</v>
@@ -4045,19 +4095,19 @@
         <v>50.53662202027962</v>
       </c>
       <c r="H87" t="n">
-        <v>50.53662202027962</v>
+        <v>53.04027633980247</v>
       </c>
       <c r="I87" t="n">
         <v>50.53662202027962</v>
       </c>
       <c r="J87" t="n">
-        <v>50.53662202027962</v>
+        <v>53.04027633980247</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>3.635653770791587</v>
       </c>
       <c r="L87" t="n">
-        <v>0</v>
+        <v>4.95413864131673</v>
       </c>
     </row>
     <row r="88">
@@ -4078,28 +4128,28 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E88" t="n">
-        <v>0.8899719715118408</v>
+        <v>0.5053746604919434</v>
       </c>
       <c r="F88" t="n">
         <v>100</v>
       </c>
       <c r="G88" t="n">
-        <v>51.67833774745558</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="H88" t="n">
-        <v>52.41137127350223</v>
+        <v>51.34703473342334</v>
       </c>
       <c r="I88" t="n">
-        <v>51.67833774745558</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="J88" t="n">
-        <v>52.41137127350223</v>
+        <v>51.34703473342334</v>
       </c>
       <c r="K88" t="n">
-        <v>0.6348256553820762</v>
+        <v>5.253618305337874</v>
       </c>
       <c r="L88" t="n">
-        <v>18.33946257249192</v>
+        <v>15.93630060422494</v>
       </c>
     </row>
     <row r="89">
@@ -4120,28 +4170,28 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E89" t="n">
-        <v>0.8668596744537354</v>
+        <v>0.4961222696304322</v>
       </c>
       <c r="F89" t="n">
         <v>100</v>
       </c>
       <c r="G89" t="n">
-        <v>51.50656411814308</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="H89" t="n">
-        <v>52.9684330467984</v>
+        <v>58.15883738323353</v>
       </c>
       <c r="I89" t="n">
-        <v>51.50656411814308</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="J89" t="n">
-        <v>52.9684330467984</v>
+        <v>58.15883738323353</v>
       </c>
       <c r="K89" t="n">
-        <v>2.419869637688528</v>
+        <v>5.68267798730279</v>
       </c>
       <c r="L89" t="n">
-        <v>4.811977788192747</v>
+        <v>15.08255807025494</v>
       </c>
     </row>
     <row r="90">
@@ -4162,19 +4212,19 @@
         <v>44.28900565726017</v>
       </c>
       <c r="E90" t="n">
-        <v>0.8682553768157959</v>
+        <v>0.6386403918266297</v>
       </c>
       <c r="F90" t="n">
-        <v>66.66666666666666</v>
+        <v>88</v>
       </c>
       <c r="G90" t="n">
-        <v>66.67915660867422</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="H90" t="n">
-        <v>67.59736162089149</v>
+        <v>88.07200264150443</v>
       </c>
       <c r="I90" t="n">
-        <v>66.67915660867422</v>
+        <v>44.28900565726017</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -4182,10 +4232,10 @@
         </is>
       </c>
       <c r="K90" t="n">
-        <v>1.298537981316628</v>
+        <v>28.8096436497013</v>
       </c>
       <c r="L90" t="n">
-        <v>52.62786016016697</v>
+        <v>98.85748468382477</v>
       </c>
     </row>
     <row r="91">
@@ -4206,28 +4256,28 @@
         <v>50.53662202027962</v>
       </c>
       <c r="E91" t="n">
-        <v>8.402032295862833</v>
+        <v>7.514532868862152</v>
       </c>
       <c r="F91" t="n">
         <v>100</v>
       </c>
       <c r="G91" t="n">
-        <v>51.637093647164</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="H91" t="n">
-        <v>72.51902409364122</v>
+        <v>74.288590120333</v>
       </c>
       <c r="I91" t="n">
-        <v>51.637093647164</v>
+        <v>50.53662202027962</v>
       </c>
       <c r="J91" t="n">
-        <v>72.51902409364122</v>
+        <v>74.288590120333</v>
       </c>
       <c r="K91" t="n">
-        <v>18.21296541760399</v>
+        <v>15.01451509818837</v>
       </c>
       <c r="L91" t="n">
-        <v>43.4979648314056</v>
+        <v>46.99951668815945</v>
       </c>
     </row>
     <row r="92">
@@ -4248,7 +4298,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E92" t="n">
-        <v>1.112603346506755</v>
+        <v>0.6994628286361695</v>
       </c>
       <c r="F92" t="n">
         <v>100</v>
@@ -4257,19 +4307,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H92" t="n">
-        <v>47.99866847890613</v>
+        <v>48.178349929368</v>
       </c>
       <c r="I92" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J92" t="n">
-        <v>47.99866847890613</v>
+        <v>48.178349929368</v>
       </c>
       <c r="K92" t="n">
-        <v>1.149830251536129</v>
+        <v>3.15305046634857</v>
       </c>
       <c r="L92" t="n">
-        <v>1.402466290083181</v>
+        <v>1.782063116428916</v>
       </c>
     </row>
     <row r="93">
@@ -4290,28 +4340,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E93" t="n">
-        <v>1.096572001775106</v>
+        <v>0.6957696104049682</v>
       </c>
       <c r="F93" t="n">
         <v>100</v>
       </c>
       <c r="G93" t="n">
-        <v>54.90718637611567</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="H93" t="n">
-        <v>54.9175958715221</v>
+        <v>57.90520692932407</v>
       </c>
       <c r="I93" t="n">
-        <v>54.90718637611567</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="J93" t="n">
-        <v>54.9175958715221</v>
+        <v>57.90520692932407</v>
       </c>
       <c r="K93" t="n">
-        <v>0.009014887462542011</v>
+        <v>4.841977743171176</v>
       </c>
       <c r="L93" t="n">
-        <v>1.066523646699732</v>
+        <v>6.564715234089694</v>
       </c>
     </row>
     <row r="94">
@@ -4332,7 +4382,7 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E94" t="n">
-        <v>0.947083314259847</v>
+        <v>0.5562766885757446</v>
       </c>
       <c r="F94" t="n">
         <v>100</v>
@@ -4341,19 +4391,19 @@
         <v>47.33481367365937</v>
       </c>
       <c r="H94" t="n">
-        <v>56.24888602612805</v>
+        <v>53.78424857145355</v>
       </c>
       <c r="I94" t="n">
         <v>47.33481367365937</v>
       </c>
       <c r="J94" t="n">
-        <v>56.24888602612805</v>
+        <v>53.78424857145355</v>
       </c>
       <c r="K94" t="n">
-        <v>15.30669546393318</v>
+        <v>7.359848336540527</v>
       </c>
       <c r="L94" t="n">
-        <v>18.83195825787974</v>
+        <v>13.62514056199428</v>
       </c>
     </row>
     <row r="95">
@@ -4374,28 +4424,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E95" t="n">
-        <v>0.9631433486938477</v>
+        <v>0.544902560710907</v>
       </c>
       <c r="F95" t="n">
         <v>100</v>
       </c>
       <c r="G95" t="n">
-        <v>64.86384032096603</v>
+        <v>54.90718637611567</v>
       </c>
       <c r="H95" t="n">
-        <v>68.87375783903298</v>
+        <v>66.41569343031314</v>
       </c>
       <c r="I95" t="n">
-        <v>64.86384032096603</v>
+        <v>54.90718637611567</v>
       </c>
       <c r="J95" t="n">
-        <v>68.87375783903298</v>
+        <v>66.41569343031314</v>
       </c>
       <c r="K95" t="n">
-        <v>6.82955042618832</v>
+        <v>7.605197194649718</v>
       </c>
       <c r="L95" t="n">
-        <v>26.7504734103862</v>
+        <v>22.22682264333181</v>
       </c>
     </row>
     <row r="96">
@@ -4416,28 +4466,30 @@
         <v>47.33481367365937</v>
       </c>
       <c r="E96" t="n">
-        <v>1.069497346878052</v>
+        <v>0.6292386889457703</v>
       </c>
       <c r="F96" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="G96" t="n">
-        <v>54.3724651017605</v>
+        <v>47.33481367365937</v>
       </c>
       <c r="H96" t="n">
-        <v>57.81332455030586</v>
+        <v>73.03401874057975</v>
       </c>
       <c r="I96" t="n">
-        <v>54.3724651017605</v>
-      </c>
-      <c r="J96" t="n">
-        <v>57.81332455030586</v>
+        <v>47.33481367365937</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="K96" t="n">
-        <v>3.014036392617975</v>
+        <v>18.05991056173489</v>
       </c>
       <c r="L96" t="n">
-        <v>22.1370067048083</v>
+        <v>54.29239722817657</v>
       </c>
     </row>
     <row r="97">
@@ -4458,28 +4510,28 @@
         <v>54.33806753213224</v>
       </c>
       <c r="E97" t="n">
-        <v>19.92718005180359</v>
+        <v>7.502623150348663</v>
       </c>
       <c r="F97" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G97" t="n">
-        <v>76.34124740580116</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="H97" t="n">
-        <v>115.5801339057931</v>
+        <v>89.16735923453278</v>
       </c>
       <c r="I97" t="n">
-        <v>76.34124740580116</v>
+        <v>54.33806753213224</v>
       </c>
       <c r="J97" t="n">
-        <v>115.5801339057931</v>
+        <v>89.6798060759062</v>
       </c>
       <c r="K97" t="n">
-        <v>34.00234192437474</v>
+        <v>36.56502544821623</v>
       </c>
       <c r="L97" t="n">
-        <v>112.705639260075</v>
+        <v>64.09740589652844</v>
       </c>
     </row>
     <row r="98">
@@ -4500,28 +4552,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E98" t="n">
-        <v>1.290271997451782</v>
+        <v>0.8762500095367431</v>
       </c>
       <c r="F98" t="n">
         <v>100</v>
       </c>
       <c r="G98" t="n">
-        <v>1.306485652800976</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="H98" t="n">
-        <v>1.591327590959869</v>
+        <v>2.631412088421083</v>
       </c>
       <c r="I98" t="n">
-        <v>1.306485652800976</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="J98" t="n">
-        <v>1.591327590959869</v>
+        <v>2.631412088421083</v>
       </c>
       <c r="K98" t="n">
-        <v>0.4933607090175952</v>
+        <v>4.096007851569302</v>
       </c>
       <c r="L98" t="n">
-        <v>1464.712563884533</v>
+        <v>2487.401600337074</v>
       </c>
     </row>
     <row r="99">
@@ -4542,7 +4594,7 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E99" t="n">
-        <v>1.27419638633728</v>
+        <v>0.8175764489173889</v>
       </c>
       <c r="F99" t="n">
         <v>100</v>
@@ -4551,19 +4603,19 @@
         <v>10.54487657926557</v>
       </c>
       <c r="H99" t="n">
-        <v>22.89634351331695</v>
+        <v>19.68549164563769</v>
       </c>
       <c r="I99" t="n">
         <v>10.54487657926557</v>
       </c>
       <c r="J99" t="n">
-        <v>22.89634351331695</v>
+        <v>19.68549164563769</v>
       </c>
       <c r="K99" t="n">
-        <v>21.39336827778398</v>
+        <v>6.049136816577715</v>
       </c>
       <c r="L99" t="n">
-        <v>117.1323992386797</v>
+        <v>86.68299716608674</v>
       </c>
     </row>
     <row r="100">
@@ -4584,28 +4636,28 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E100" t="n">
-        <v>1.166152000427246</v>
+        <v>0.6721225810050965</v>
       </c>
       <c r="F100" t="n">
         <v>100</v>
       </c>
       <c r="G100" t="n">
-        <v>1.306485652800976</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="H100" t="n">
-        <v>6.615765352849009</v>
+        <v>10.19118464630782</v>
       </c>
       <c r="I100" t="n">
-        <v>1.306485652800976</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="J100" t="n">
-        <v>6.615765352849009</v>
+        <v>10.19118464630782</v>
       </c>
       <c r="K100" t="n">
-        <v>5.222769989219668</v>
+        <v>9.6176740663952</v>
       </c>
       <c r="L100" t="n">
-        <v>6405.116373348855</v>
+        <v>9920.736614845217</v>
       </c>
     </row>
     <row r="101">
@@ -4626,28 +4678,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E101" t="n">
-        <v>1.067466656366984</v>
+        <v>0.6427696585655213</v>
       </c>
       <c r="F101" t="n">
         <v>100</v>
       </c>
       <c r="G101" t="n">
-        <v>21.6799181202689</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="H101" t="n">
-        <v>53.77892825703592</v>
+        <v>34.07776229529959</v>
       </c>
       <c r="I101" t="n">
-        <v>21.6799181202689</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="J101" t="n">
-        <v>53.77892825703592</v>
+        <v>34.07776229529959</v>
       </c>
       <c r="K101" t="n">
-        <v>28.34536542287317</v>
+        <v>15.24318051442878</v>
       </c>
       <c r="L101" t="n">
-        <v>410.00054721154</v>
+        <v>223.1689061425984</v>
       </c>
     </row>
     <row r="102">
@@ -4668,19 +4720,19 @@
         <v>0.1017009531136672</v>
       </c>
       <c r="E102" t="n">
-        <v>0.928563674290975</v>
+        <v>0.6312933921813965</v>
       </c>
       <c r="F102" t="n">
-        <v>66.66666666666666</v>
+        <v>80</v>
       </c>
       <c r="G102" t="n">
-        <v>6.793312519849838</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="H102" t="n">
-        <v>17.01574544376469</v>
+        <v>25.10546106357515</v>
       </c>
       <c r="I102" t="n">
-        <v>6.793312519849838</v>
+        <v>0.1017009531136672</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -4688,10 +4740,10 @@
         </is>
       </c>
       <c r="K102" t="n">
-        <v>14.45670328144963</v>
+        <v>18.37865938981922</v>
       </c>
       <c r="L102" t="n">
-        <v>16631.15631939737</v>
+        <v>24585.57107376933</v>
       </c>
     </row>
     <row r="103">
@@ -4712,28 +4764,28 @@
         <v>10.54487657926557</v>
       </c>
       <c r="E103" t="n">
-        <v>8.370152632395426</v>
+        <v>7.833008828163147</v>
       </c>
       <c r="F103" t="n">
-        <v>66.66666666666666</v>
+        <v>78</v>
       </c>
       <c r="G103" t="n">
-        <v>28.23002195945354</v>
+        <v>10.54487657926557</v>
       </c>
       <c r="H103" t="n">
-        <v>52.0991475958883</v>
+        <v>68.87403209071439</v>
       </c>
       <c r="I103" t="n">
-        <v>28.23002195945354</v>
+        <v>7.497196031731945</v>
       </c>
       <c r="J103" t="n">
-        <v>75.49412273332037</v>
+        <v>65.5511038673356</v>
       </c>
       <c r="K103" t="n">
-        <v>33.75604119703338</v>
+        <v>35.85527815653631</v>
       </c>
       <c r="L103" t="n">
-        <v>394.0707195979046</v>
+        <v>553.1516189211893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>